<commit_message>
Criar uma nova coleção no banco (Skip Cloud/PocketBase) chamada "negoci…
</commit_message>
<xml_diff>
--- a/public/schema-delfos-solar.xlsx
+++ b/public/schema-delfos-solar.xlsx
@@ -1188,22 +1188,50 @@
     <row r="40">
       <c r="A40" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TOTAL: 38 coleções</t>
+          <t xml:space="preserve">negocios</t>
         </is>
       </c>
       <c r="B40" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Coleção de dados do sistema.</t>
+        </is>
+      </c>
+      <c r="C40" s="2">
+        <v>15</v>
+      </c>
+      <c r="D40" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">base</t>
+        </is>
+      </c>
+      <c r="E40" s="2">
+        <v>1</v>
+      </c>
+      <c r="F40" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Regras RLS configuradas (autenticado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TOTAL: 39 coleções</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Total geral de campos e relacionamentos no banco PocketBase Delfos Solar</t>
         </is>
       </c>
-      <c r="C40" s="2">
-        <v>659</v>
-      </c>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2">
-        <v>45</v>
-      </c>
-      <c r="F40" s="2"/>
+      <c r="C41" s="2">
+        <v>674</v>
+      </c>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2">
+        <v>46</v>
+      </c>
+      <c r="F41" s="2"/>
     </row>
   </sheetData>
 </worksheet>
@@ -18649,6 +18677,409 @@
         </is>
       </c>
     </row>
+    <row r="661">
+      <c r="A661" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">cliente_id</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">relation</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E661" s="2"/>
+      <c r="F661" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
+      <c r="G661" s="2"/>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">tipo_negocio</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">select</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">venda usina | bateria | expansão | renovação | serviço</t>
+        </is>
+      </c>
+      <c r="F662" s="2"/>
+      <c r="G662" s="2"/>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">valor_estimado</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E663" s="2"/>
+      <c r="F663" s="2"/>
+      <c r="G663" s="2"/>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">valor_final</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E664" s="2"/>
+      <c r="F664" s="2"/>
+      <c r="G664" s="2"/>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">etapa_funil</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">select</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">novo lead | qualificado | proposta enviada | negociação | contrato assinado</t>
+        </is>
+      </c>
+      <c r="F665" s="2"/>
+      <c r="G665" s="2"/>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">probabilidade</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E666" s="2"/>
+      <c r="F666" s="2"/>
+      <c r="G666" s="2"/>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">data_previsao_fechamento</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">date</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E667" s="2"/>
+      <c r="F667" s="2"/>
+      <c r="G667" s="2"/>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">data_fechamento</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">date</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E668" s="2"/>
+      <c r="F668" s="2"/>
+      <c r="G668" s="2"/>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">status</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">select</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">em andamento | ganho | perdido</t>
+        </is>
+      </c>
+      <c r="F669" s="2"/>
+      <c r="G669" s="2"/>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">motivo_perda</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E670" s="2"/>
+      <c r="F670" s="2"/>
+      <c r="G670" s="2"/>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">reabertura</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">bool</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
+      <c r="F671" s="2"/>
+      <c r="G671" s="2"/>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">motivo_reabertura</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E672" s="2"/>
+      <c r="F672" s="2"/>
+      <c r="G672" s="2"/>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">condicao_pagamento</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E673" s="2"/>
+      <c r="F673" s="2"/>
+      <c r="G673" s="2"/>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">created</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E674" s="2"/>
+      <c r="F674" s="2"/>
+      <c r="G674" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">updated</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E675" s="2"/>
+      <c r="F675" s="2"/>
+      <c r="G675" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -20136,6 +20567,38 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">cliente_id</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Vínculo do registro ao cliente proprietário</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adicionar campos titulo, valor e consultor_responsavel na colecao negocios e opcao venda bateria no select tipo_negocio
</commit_message>
<xml_diff>
--- a/public/schema-delfos-solar.xlsx
+++ b/public/schema-delfos-solar.xlsx
@@ -1197,7 +1197,7 @@
         </is>
       </c>
       <c r="C40" s="2">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D40" t="inlineStr" s="2">
         <is>
@@ -1205,7 +1205,7 @@
         </is>
       </c>
       <c r="E40" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F40" t="inlineStr" s="2">
         <is>
@@ -1225,11 +1225,11 @@
         </is>
       </c>
       <c r="C41" s="2">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="2">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F41" s="2"/>
     </row>
@@ -18758,7 +18758,7 @@
       </c>
       <c r="E663" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">venda usina | bateria | expansão | renovação | serviço</t>
+          <t xml:space="preserve">venda usina | bateria | expansão | renovação | serviço | venda bateria</t>
         </is>
       </c>
       <c r="F663" s="2"/>
@@ -19137,6 +19137,85 @@
       </c>
       <c r="F677" s="2"/>
       <c r="G677" s="2"/>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">titulo</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E678" s="2"/>
+      <c r="F678" s="2"/>
+      <c r="G678" s="2"/>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">valor</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E679" s="2"/>
+      <c r="F679" s="2"/>
+      <c r="G679" s="2"/>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">consultor_responsavel</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">relation</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E680" s="2"/>
+      <c r="F680" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">users</t>
+        </is>
+      </c>
+      <c r="G680" s="2"/>
     </row>
   </sheetData>
 </worksheet>
@@ -20657,6 +20736,38 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">consultor_responsavel</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">users</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Relaciona o registro de negocios com users</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: unificar coleções sistemas e usinas absorvendo tudo em usinas
</commit_message>
<xml_diff>
--- a/public/schema-delfos-solar.xlsx
+++ b/public/schema-delfos-solar.xlsx
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="C31" s="2">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="D31" t="inlineStr" s="2">
         <is>
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="C41" s="2">
-        <v>679</v>
+        <v>708</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="2">
@@ -16653,71 +16653,71 @@
     <row r="586">
       <c r="A586" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contatos_adicionais</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B586" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente</t>
+          <t xml:space="preserve">padrao_entrada</t>
         </is>
       </c>
       <c r="C586" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D586" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E586" s="2"/>
-      <c r="F586" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+      <c r="F586" s="2"/>
       <c r="G586" s="2"/>
     </row>
     <row r="587">
       <c r="A587" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contatos_adicionais</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B587" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">nome</t>
+          <t xml:space="preserve">tipo_atendimento</t>
         </is>
       </c>
       <c r="C587" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D587" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E587" s="2"/>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">aéreo | subterrâneo</t>
+        </is>
+      </c>
       <c r="F587" s="2"/>
       <c r="G587" s="2"/>
     </row>
     <row r="588">
       <c r="A588" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contatos_adicionais</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B588" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cargo</t>
+          <t xml:space="preserve">numero_fases</t>
         </is>
       </c>
       <c r="C588" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D588" t="inlineStr" s="2">
@@ -16725,19 +16725,23 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E588" s="2"/>
+      <c r="E588" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">monofásico | bifásico | trifásico</t>
+        </is>
+      </c>
       <c r="F588" s="2"/>
       <c r="G588" s="2"/>
     </row>
     <row r="589">
       <c r="A589" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contatos_adicionais</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B589" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">telefone</t>
+          <t xml:space="preserve">secao_cabos</t>
         </is>
       </c>
       <c r="C589" t="inlineStr" s="2">
@@ -16757,12 +16761,12 @@
     <row r="590">
       <c r="A590" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contatos_adicionais</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B590" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">email</t>
+          <t xml:space="preserve">amperagem_disjuntor</t>
         </is>
       </c>
       <c r="C590" t="inlineStr" s="2">
@@ -16782,17 +16786,17 @@
     <row r="591">
       <c r="A591" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contatos_adicionais</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B591" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">tipo_caixa_medicao</t>
         </is>
       </c>
       <c r="C591" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D591" t="inlineStr" s="2">
@@ -16802,26 +16806,22 @@
       </c>
       <c r="E591" s="2"/>
       <c r="F591" s="2"/>
-      <c r="G591" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G591" s="2"/>
     </row>
     <row r="592">
       <c r="A592" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contatos_adicionais</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B592" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">latitude</t>
         </is>
       </c>
       <c r="C592" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D592" t="inlineStr" s="2">
@@ -16831,31 +16831,27 @@
       </c>
       <c r="E592" s="2"/>
       <c r="F592" s="2"/>
-      <c r="G592" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G592" s="2"/>
     </row>
     <row r="593">
       <c r="A593" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">instalacoes_galeria</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B593" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">longitude</t>
         </is>
       </c>
       <c r="C593" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D593" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E593" s="2"/>
@@ -16865,17 +16861,17 @@
     <row r="594">
       <c r="A594" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">instalacoes_galeria</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B594" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cidade</t>
+          <t xml:space="preserve">tarifa</t>
         </is>
       </c>
       <c r="C594" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D594" t="inlineStr" s="2">
@@ -16890,17 +16886,17 @@
     <row r="595">
       <c r="A595" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">instalacoes_galeria</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B595" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">potencia_kwp</t>
+          <t xml:space="preserve">classe_consumo</t>
         </is>
       </c>
       <c r="C595" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D595" t="inlineStr" s="2">
@@ -16915,17 +16911,17 @@
     <row r="596">
       <c r="A596" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">instalacoes_galeria</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B596" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">foto</t>
+          <t xml:space="preserve">geracao_media_mensal_kwh</t>
         </is>
       </c>
       <c r="C596" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">file</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D596" t="inlineStr" s="2">
@@ -16935,21 +16931,17 @@
       </c>
       <c r="E596" s="2"/>
       <c r="F596" s="2"/>
-      <c r="G596" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
-        </is>
-      </c>
+      <c r="G596" s="2"/>
     </row>
     <row r="597">
       <c r="A597" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">instalacoes_galeria</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B597" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">foto_url</t>
+          <t xml:space="preserve">monitoramento_app_nome</t>
         </is>
       </c>
       <c r="C597" t="inlineStr" s="2">
@@ -16969,17 +16961,17 @@
     <row r="598">
       <c r="A598" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">instalacoes_galeria</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B598" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ordem</t>
+          <t xml:space="preserve">monitoramento_login</t>
         </is>
       </c>
       <c r="C598" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D598" t="inlineStr" s="2">
@@ -16994,17 +16986,17 @@
     <row r="599">
       <c r="A599" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">instalacoes_galeria</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B599" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">destaque</t>
+          <t xml:space="preserve">monitoramento_senha</t>
         </is>
       </c>
       <c r="C599" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D599" t="inlineStr" s="2">
@@ -17012,28 +17004,24 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E599" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E599" s="2"/>
       <c r="F599" s="2"/>
       <c r="G599" s="2"/>
     </row>
     <row r="600">
       <c r="A600" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">instalacoes_galeria</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B600" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">monitoramento_datalogger_url</t>
         </is>
       </c>
       <c r="C600" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D600" t="inlineStr" s="2">
@@ -17043,26 +17031,22 @@
       </c>
       <c r="E600" s="2"/>
       <c r="F600" s="2"/>
-      <c r="G600" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G600" s="2"/>
     </row>
     <row r="601">
       <c r="A601" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">instalacoes_galeria</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B601" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">solarview_login</t>
         </is>
       </c>
       <c r="C601" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D601" t="inlineStr" s="2">
@@ -17072,31 +17056,27 @@
       </c>
       <c r="E601" s="2"/>
       <c r="F601" s="2"/>
-      <c r="G601" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G601" s="2"/>
     </row>
     <row r="602">
       <c r="A602" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">projecao_tarifaria</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B602" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ano</t>
+          <t xml:space="preserve">solarview_senha</t>
         </is>
       </c>
       <c r="C602" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D602" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E602" s="2"/>
@@ -17106,46 +17086,42 @@
     <row r="603">
       <c r="A603" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">projecao_tarifaria</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B603" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_cliente</t>
+          <t xml:space="preserve">solarview_link_ios</t>
         </is>
       </c>
       <c r="C603" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D603" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E603" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">residencial | comercial</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E603" s="2"/>
       <c r="F603" s="2"/>
       <c r="G603" s="2"/>
     </row>
     <row r="604">
       <c r="A604" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">projecao_tarifaria</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B604" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tarifa_kwh</t>
+          <t xml:space="preserve">solarview_link_android</t>
         </is>
       </c>
       <c r="C604" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D604" t="inlineStr" s="2">
@@ -17160,17 +17136,17 @@
     <row r="605">
       <c r="A605" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">projecao_tarifaria</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B605" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fio_b_kwh</t>
+          <t xml:space="preserve">solarview_link_texto</t>
         </is>
       </c>
       <c r="C605" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D605" t="inlineStr" s="2">
@@ -17185,17 +17161,17 @@
     <row r="606">
       <c r="A606" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">projecao_tarifaria</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B606" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fs</t>
+          <t xml:space="preserve">fabricante_inversores</t>
         </is>
       </c>
       <c r="C606" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D606" t="inlineStr" s="2">
@@ -17210,17 +17186,17 @@
     <row r="607">
       <c r="A607" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">projecao_tarifaria</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B607" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gd_eco_liquida</t>
+          <t xml:space="preserve">modelo_inversores</t>
         </is>
       </c>
       <c r="C607" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D607" t="inlineStr" s="2">
@@ -17235,12 +17211,12 @@
     <row r="608">
       <c r="A608" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">projecao_tarifaria</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B608" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">economia_acumulada</t>
+          <t xml:space="preserve">potencia_pico_inversores_kwp</t>
         </is>
       </c>
       <c r="C608" t="inlineStr" s="2">
@@ -17260,17 +17236,17 @@
     <row r="609">
       <c r="A609" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">projecao_tarifaria</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B609" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gasto_acumulado</t>
+          <t xml:space="preserve">fabricante_modulos</t>
         </is>
       </c>
       <c r="C609" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D609" t="inlineStr" s="2">
@@ -17285,17 +17261,17 @@
     <row r="610">
       <c r="A610" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">projecao_tarifaria</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B610" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">modelo_modulos</t>
         </is>
       </c>
       <c r="C610" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D610" t="inlineStr" s="2">
@@ -17305,26 +17281,22 @@
       </c>
       <c r="E610" s="2"/>
       <c r="F610" s="2"/>
-      <c r="G610" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G610" s="2"/>
     </row>
     <row r="611">
       <c r="A611" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">projecao_tarifaria</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B611" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">potencia_pico_modulos_kwp</t>
         </is>
       </c>
       <c r="C611" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D611" t="inlineStr" s="2">
@@ -17334,50 +17306,42 @@
       </c>
       <c r="E611" s="2"/>
       <c r="F611" s="2"/>
-      <c r="G611" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G611" s="2"/>
     </row>
     <row r="612">
       <c r="A612" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">equipamentos</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B612" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo</t>
+          <t xml:space="preserve">quantidade_placas</t>
         </is>
       </c>
       <c r="C612" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D612" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E612" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">inversor | modulo_fv</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E612" s="2"/>
       <c r="F612" s="2"/>
       <c r="G612" s="2"/>
     </row>
     <row r="613">
       <c r="A613" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">equipamentos</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B613" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">marca</t>
+          <t xml:space="preserve">marca_placas</t>
         </is>
       </c>
       <c r="C613" t="inlineStr" s="2">
@@ -17387,7 +17351,7 @@
       </c>
       <c r="D613" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E613" s="2"/>
@@ -17397,42 +17361,46 @@
     <row r="614">
       <c r="A614" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">equipamentos</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B614" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">modelo</t>
+          <t xml:space="preserve">tipo_telhado</t>
         </is>
       </c>
       <c r="C614" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D614" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E614" s="2"/>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ceramico | metalico | laje | fibrocimento</t>
+        </is>
+      </c>
       <c r="F614" s="2"/>
       <c r="G614" s="2"/>
     </row>
     <row r="615">
       <c r="A615" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">equipamentos</t>
+          <t xml:space="preserve">contatos_adicionais</t>
         </is>
       </c>
       <c r="B615" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">potencia_w</t>
+          <t xml:space="preserve">cliente</t>
         </is>
       </c>
       <c r="C615" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D615" t="inlineStr" s="2">
@@ -17441,18 +17409,22 @@
         </is>
       </c>
       <c r="E615" s="2"/>
-      <c r="F615" s="2"/>
+      <c r="F615" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G615" s="2"/>
     </row>
     <row r="616">
       <c r="A616" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">equipamentos</t>
+          <t xml:space="preserve">contatos_adicionais</t>
         </is>
       </c>
       <c r="B616" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">descricao_padrao</t>
+          <t xml:space="preserve">nome</t>
         </is>
       </c>
       <c r="C616" t="inlineStr" s="2">
@@ -17462,7 +17434,7 @@
       </c>
       <c r="D616" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E616" s="2"/>
@@ -17472,17 +17444,17 @@
     <row r="617">
       <c r="A617" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">equipamentos</t>
+          <t xml:space="preserve">contatos_adicionais</t>
         </is>
       </c>
       <c r="B617" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">garantia_anos</t>
+          <t xml:space="preserve">cargo</t>
         </is>
       </c>
       <c r="C617" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D617" t="inlineStr" s="2">
@@ -17497,17 +17469,17 @@
     <row r="618">
       <c r="A618" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">equipamentos</t>
+          <t xml:space="preserve">contatos_adicionais</t>
         </is>
       </c>
       <c r="B618" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">foto</t>
+          <t xml:space="preserve">telefone</t>
         </is>
       </c>
       <c r="C618" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">file</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D618" t="inlineStr" s="2">
@@ -17517,26 +17489,22 @@
       </c>
       <c r="E618" s="2"/>
       <c r="F618" s="2"/>
-      <c r="G618" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
-        </is>
-      </c>
+      <c r="G618" s="2"/>
     </row>
     <row r="619">
       <c r="A619" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">equipamentos</t>
+          <t xml:space="preserve">contatos_adicionais</t>
         </is>
       </c>
       <c r="B619" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">email</t>
         </is>
       </c>
       <c r="C619" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D619" t="inlineStr" s="2">
@@ -17546,21 +17514,17 @@
       </c>
       <c r="E619" s="2"/>
       <c r="F619" s="2"/>
-      <c r="G619" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G619" s="2"/>
     </row>
     <row r="620">
       <c r="A620" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">equipamentos</t>
+          <t xml:space="preserve">contatos_adicionais</t>
         </is>
       </c>
       <c r="B620" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C620" t="inlineStr" s="2">
@@ -17577,49 +17541,53 @@
       <c r="F620" s="2"/>
       <c r="G620" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="621">
       <c r="A621" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">parametros_tarifarios</t>
+          <t xml:space="preserve">contatos_adicionais</t>
         </is>
       </c>
       <c r="B621" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ano</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C621" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D621" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E621" s="2"/>
       <c r="F621" s="2"/>
-      <c r="G621" s="2"/>
+      <c r="G621" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="622">
       <c r="A622" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">parametros_tarifarios</t>
+          <t xml:space="preserve">instalacoes_galeria</t>
         </is>
       </c>
       <c r="B622" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">classe</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C622" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D622" t="inlineStr" s="2">
@@ -17627,28 +17595,24 @@
           <t xml:space="preserve">Sim</t>
         </is>
       </c>
-      <c r="E622" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">residencial | comercial</t>
-        </is>
-      </c>
+      <c r="E622" s="2"/>
       <c r="F622" s="2"/>
       <c r="G622" s="2"/>
     </row>
     <row r="623">
       <c r="A623" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">parametros_tarifarios</t>
+          <t xml:space="preserve">instalacoes_galeria</t>
         </is>
       </c>
       <c r="B623" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tarifa</t>
+          <t xml:space="preserve">cidade</t>
         </is>
       </c>
       <c r="C623" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D623" t="inlineStr" s="2">
@@ -17663,12 +17627,12 @@
     <row r="624">
       <c r="A624" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">parametros_tarifarios</t>
+          <t xml:space="preserve">instalacoes_galeria</t>
         </is>
       </c>
       <c r="B624" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fio_b</t>
+          <t xml:space="preserve">potencia_kwp</t>
         </is>
       </c>
       <c r="C624" t="inlineStr" s="2">
@@ -17688,17 +17652,17 @@
     <row r="625">
       <c r="A625" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">parametros_tarifarios</t>
+          <t xml:space="preserve">instalacoes_galeria</t>
         </is>
       </c>
       <c r="B625" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fs</t>
+          <t xml:space="preserve">foto</t>
         </is>
       </c>
       <c r="C625" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="D625" t="inlineStr" s="2">
@@ -17708,22 +17672,26 @@
       </c>
       <c r="E625" s="2"/>
       <c r="F625" s="2"/>
-      <c r="G625" s="2"/>
+      <c r="G625" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
+        </is>
+      </c>
     </row>
     <row r="626">
       <c r="A626" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">parametros_tarifarios</t>
+          <t xml:space="preserve">instalacoes_galeria</t>
         </is>
       </c>
       <c r="B626" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gd_eco_liquida</t>
+          <t xml:space="preserve">foto_url</t>
         </is>
       </c>
       <c r="C626" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D626" t="inlineStr" s="2">
@@ -17738,17 +17706,17 @@
     <row r="627">
       <c r="A627" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">parametros_tarifarios</t>
+          <t xml:space="preserve">instalacoes_galeria</t>
         </is>
       </c>
       <c r="B627" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">ordem</t>
         </is>
       </c>
       <c r="C627" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D627" t="inlineStr" s="2">
@@ -17758,26 +17726,22 @@
       </c>
       <c r="E627" s="2"/>
       <c r="F627" s="2"/>
-      <c r="G627" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G627" s="2"/>
     </row>
     <row r="628">
       <c r="A628" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">parametros_tarifarios</t>
+          <t xml:space="preserve">instalacoes_galeria</t>
         </is>
       </c>
       <c r="B628" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">destaque</t>
         </is>
       </c>
       <c r="C628" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D628" t="inlineStr" s="2">
@@ -17785,106 +17749,106 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E628" s="2"/>
+      <c r="E628" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F628" s="2"/>
-      <c r="G628" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G628" s="2"/>
     </row>
     <row r="629">
       <c r="A629" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">instalacoes_galeria</t>
         </is>
       </c>
       <c r="B629" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">nome</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C629" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D629" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E629" s="2"/>
       <c r="F629" s="2"/>
-      <c r="G629" s="2"/>
+      <c r="G629" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="630">
       <c r="A630" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">instalacoes_galeria</t>
         </is>
       </c>
       <c r="B630" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gatilho</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C630" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D630" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E630" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">status_mudou | instalacao_concluida | atividade_concluida | data_especifica | dias_apos_evento</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E630" s="2"/>
       <c r="F630" s="2"/>
-      <c r="G630" s="2"/>
+      <c r="G630" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="631">
       <c r="A631" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">projecao_tarifaria</t>
         </is>
       </c>
       <c r="B631" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">configuracao_gatilho</t>
+          <t xml:space="preserve">ano</t>
         </is>
       </c>
       <c r="C631" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D631" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E631" s="2"/>
       <c r="F631" s="2"/>
-      <c r="G631" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="G631" s="2"/>
     </row>
     <row r="632">
       <c r="A632" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">projecao_tarifaria</t>
         </is>
       </c>
       <c r="B632" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">acao</t>
+          <t xml:space="preserve">tipo_cliente</t>
         </is>
       </c>
       <c r="C632" t="inlineStr" s="2">
@@ -17899,7 +17863,7 @@
       </c>
       <c r="E632" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">criar_atividade | enviar_whatsapp | enviar_email | mudar_status</t>
+          <t xml:space="preserve">residencial | comercial</t>
         </is>
       </c>
       <c r="F632" s="2"/>
@@ -17908,17 +17872,17 @@
     <row r="633">
       <c r="A633" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">projecao_tarifaria</t>
         </is>
       </c>
       <c r="B633" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">configuracao_acao</t>
+          <t xml:space="preserve">tarifa_kwh</t>
         </is>
       </c>
       <c r="C633" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D633" t="inlineStr" s="2">
@@ -17928,55 +17892,47 @@
       </c>
       <c r="E633" s="2"/>
       <c r="F633" s="2"/>
-      <c r="G633" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="G633" s="2"/>
     </row>
     <row r="634">
       <c r="A634" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">projecao_tarifaria</t>
         </is>
       </c>
       <c r="B634" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">destino</t>
+          <t xml:space="preserve">fio_b_kwh</t>
         </is>
       </c>
       <c r="C634" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D634" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E634" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">cliente_evento | responsavel_empresa | cliente_especifico</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E634" s="2"/>
       <c r="F634" s="2"/>
       <c r="G634" s="2"/>
     </row>
     <row r="635">
       <c r="A635" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">projecao_tarifaria</t>
         </is>
       </c>
       <c r="B635" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_especifico_id</t>
+          <t xml:space="preserve">fs</t>
         </is>
       </c>
       <c r="C635" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D635" t="inlineStr" s="2">
@@ -17985,27 +17941,23 @@
         </is>
       </c>
       <c r="E635" s="2"/>
-      <c r="F635" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+      <c r="F635" s="2"/>
       <c r="G635" s="2"/>
     </row>
     <row r="636">
       <c r="A636" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">projecao_tarifaria</t>
         </is>
       </c>
       <c r="B636" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ativa</t>
+          <t xml:space="preserve">gd_eco_liquida</t>
         </is>
       </c>
       <c r="C636" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D636" t="inlineStr" s="2">
@@ -18013,28 +17965,24 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E636" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E636" s="2"/>
       <c r="F636" s="2"/>
       <c r="G636" s="2"/>
     </row>
     <row r="637">
       <c r="A637" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">projecao_tarifaria</t>
         </is>
       </c>
       <c r="B637" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">economia_acumulada</t>
         </is>
       </c>
       <c r="C637" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D637" t="inlineStr" s="2">
@@ -18044,26 +17992,22 @@
       </c>
       <c r="E637" s="2"/>
       <c r="F637" s="2"/>
-      <c r="G637" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G637" s="2"/>
     </row>
     <row r="638">
       <c r="A638" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">projecao_tarifaria</t>
         </is>
       </c>
       <c r="B638" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">gasto_acumulado</t>
         </is>
       </c>
       <c r="C638" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D638" t="inlineStr" s="2">
@@ -18073,90 +18017,90 @@
       </c>
       <c r="E638" s="2"/>
       <c r="F638" s="2"/>
-      <c r="G638" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G638" s="2"/>
     </row>
     <row r="639">
       <c r="A639" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes_execucoes</t>
+          <t xml:space="preserve">projecao_tarifaria</t>
         </is>
       </c>
       <c r="B639" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacao</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C639" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D639" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E639" s="2"/>
-      <c r="F639" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">automacoes</t>
-        </is>
-      </c>
-      <c r="G639" s="2"/>
+      <c r="F639" s="2"/>
+      <c r="G639" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="640">
       <c r="A640" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes_execucoes</t>
+          <t xml:space="preserve">projecao_tarifaria</t>
         </is>
       </c>
       <c r="B640" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_execucao</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C640" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D640" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E640" s="2"/>
       <c r="F640" s="2"/>
-      <c r="G640" s="2"/>
+      <c r="G640" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="641">
       <c r="A641" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes_execucoes</t>
+          <t xml:space="preserve">equipamentos</t>
         </is>
       </c>
       <c r="B641" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">sucesso</t>
+          <t xml:space="preserve">tipo</t>
         </is>
       </c>
       <c r="C641" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D641" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E641" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">true / false</t>
+          <t xml:space="preserve">inversor | modulo_fv</t>
         </is>
       </c>
       <c r="F641" s="2"/>
@@ -18165,12 +18109,12 @@
     <row r="642">
       <c r="A642" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes_execucoes</t>
+          <t xml:space="preserve">equipamentos</t>
         </is>
       </c>
       <c r="B642" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mensagem</t>
+          <t xml:space="preserve">marca</t>
         </is>
       </c>
       <c r="C642" t="inlineStr" s="2">
@@ -18180,7 +18124,7 @@
       </c>
       <c r="D642" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E642" s="2"/>
@@ -18190,12 +18134,12 @@
     <row r="643">
       <c r="A643" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes_execucoes</t>
+          <t xml:space="preserve">equipamentos</t>
         </is>
       </c>
       <c r="B643" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">referencia_registro</t>
+          <t xml:space="preserve">modelo</t>
         </is>
       </c>
       <c r="C643" t="inlineStr" s="2">
@@ -18205,7 +18149,7 @@
       </c>
       <c r="D643" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E643" s="2"/>
@@ -18215,46 +18159,42 @@
     <row r="644">
       <c r="A644" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes_execucoes</t>
+          <t xml:space="preserve">equipamentos</t>
         </is>
       </c>
       <c r="B644" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente</t>
+          <t xml:space="preserve">potencia_w</t>
         </is>
       </c>
       <c r="C644" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D644" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E644" s="2"/>
-      <c r="F644" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+      <c r="F644" s="2"/>
       <c r="G644" s="2"/>
     </row>
     <row r="645">
       <c r="A645" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes_execucoes</t>
+          <t xml:space="preserve">equipamentos</t>
         </is>
       </c>
       <c r="B645" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">dados_execucao</t>
+          <t xml:space="preserve">descricao_padrao</t>
         </is>
       </c>
       <c r="C645" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D645" t="inlineStr" s="2">
@@ -18264,26 +18204,22 @@
       </c>
       <c r="E645" s="2"/>
       <c r="F645" s="2"/>
-      <c r="G645" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="G645" s="2"/>
     </row>
     <row r="646">
       <c r="A646" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes_execucoes</t>
+          <t xml:space="preserve">equipamentos</t>
         </is>
       </c>
       <c r="B646" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">garantia_anos</t>
         </is>
       </c>
       <c r="C646" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D646" t="inlineStr" s="2">
@@ -18293,26 +18229,22 @@
       </c>
       <c r="E646" s="2"/>
       <c r="F646" s="2"/>
-      <c r="G646" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G646" s="2"/>
     </row>
     <row r="647">
       <c r="A647" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes_execucoes</t>
+          <t xml:space="preserve">equipamentos</t>
         </is>
       </c>
       <c r="B647" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">foto</t>
         </is>
       </c>
       <c r="C647" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="D647" t="inlineStr" s="2">
@@ -18324,83 +18256,87 @@
       <c r="F647" s="2"/>
       <c r="G647" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
         </is>
       </c>
     </row>
     <row r="648">
       <c r="A648" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">equipamentos</t>
         </is>
       </c>
       <c r="B648" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C648" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D648" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E648" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">atividade_atrasada | lembrete | sistema</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E648" s="2"/>
       <c r="F648" s="2"/>
-      <c r="G648" s="2"/>
+      <c r="G648" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="649">
       <c r="A649" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">equipamentos</t>
         </is>
       </c>
       <c r="B649" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C649" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D649" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E649" s="2"/>
       <c r="F649" s="2"/>
-      <c r="G649" s="2"/>
+      <c r="G649" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="650">
       <c r="A650" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">parametros_tarifarios</t>
         </is>
       </c>
       <c r="B650" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mensagem</t>
+          <t xml:space="preserve">ano</t>
         </is>
       </c>
       <c r="C650" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D650" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E650" s="2"/>
@@ -18410,46 +18346,46 @@
     <row r="651">
       <c r="A651" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">parametros_tarifarios</t>
         </is>
       </c>
       <c r="B651" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">atividade_id</t>
+          <t xml:space="preserve">classe</t>
         </is>
       </c>
       <c r="C651" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D651" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E651" s="2"/>
-      <c r="F651" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">atividades</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">residencial | comercial</t>
+        </is>
+      </c>
+      <c r="F651" s="2"/>
       <c r="G651" s="2"/>
     </row>
     <row r="652">
       <c r="A652" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">parametros_tarifarios</t>
         </is>
       </c>
       <c r="B652" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_id</t>
+          <t xml:space="preserve">tarifa</t>
         </is>
       </c>
       <c r="C652" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D652" t="inlineStr" s="2">
@@ -18458,27 +18394,23 @@
         </is>
       </c>
       <c r="E652" s="2"/>
-      <c r="F652" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+      <c r="F652" s="2"/>
       <c r="G652" s="2"/>
     </row>
     <row r="653">
       <c r="A653" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">parametros_tarifarios</t>
         </is>
       </c>
       <c r="B653" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_nome</t>
+          <t xml:space="preserve">fio_b</t>
         </is>
       </c>
       <c r="C653" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D653" t="inlineStr" s="2">
@@ -18493,17 +18425,17 @@
     <row r="654">
       <c r="A654" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">parametros_tarifarios</t>
         </is>
       </c>
       <c r="B654" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_prevista</t>
+          <t xml:space="preserve">fs</t>
         </is>
       </c>
       <c r="C654" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D654" t="inlineStr" s="2">
@@ -18518,12 +18450,12 @@
     <row r="655">
       <c r="A655" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">parametros_tarifarios</t>
         </is>
       </c>
       <c r="B655" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">dias_atraso</t>
+          <t xml:space="preserve">gd_eco_liquida</t>
         </is>
       </c>
       <c r="C655" t="inlineStr" s="2">
@@ -18543,17 +18475,17 @@
     <row r="656">
       <c r="A656" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">parametros_tarifarios</t>
         </is>
       </c>
       <c r="B656" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">lida</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C656" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D656" t="inlineStr" s="2">
@@ -18561,28 +18493,28 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E656" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E656" s="2"/>
       <c r="F656" s="2"/>
-      <c r="G656" s="2"/>
+      <c r="G656" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="657">
       <c r="A657" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">parametros_tarifarios</t>
         </is>
       </c>
       <c r="B657" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">lida_em</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C657" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D657" t="inlineStr" s="2">
@@ -18592,22 +18524,26 @@
       </c>
       <c r="E657" s="2"/>
       <c r="F657" s="2"/>
-      <c r="G657" s="2"/>
+      <c r="G657" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="658">
       <c r="A658" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">automacoes</t>
         </is>
       </c>
       <c r="B658" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">nome</t>
         </is>
       </c>
       <c r="C658" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D658" t="inlineStr" s="2">
@@ -18615,53 +18551,53 @@
           <t xml:space="preserve">Sim</t>
         </is>
       </c>
-      <c r="E658" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">ativa | resolvida | arquivada</t>
-        </is>
-      </c>
+      <c r="E658" s="2"/>
       <c r="F658" s="2"/>
       <c r="G658" s="2"/>
     </row>
     <row r="659">
       <c r="A659" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">automacoes</t>
         </is>
       </c>
       <c r="B659" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">resolvida_em</t>
+          <t xml:space="preserve">gatilho</t>
         </is>
       </c>
       <c r="C659" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D659" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E659" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">status_mudou | instalacao_concluida | atividade_concluida | data_especifica | dias_apos_evento</t>
+        </is>
+      </c>
       <c r="F659" s="2"/>
       <c r="G659" s="2"/>
     </row>
     <row r="660">
       <c r="A660" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">automacoes</t>
         </is>
       </c>
       <c r="B660" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">configuracao_gatilho</t>
         </is>
       </c>
       <c r="C660" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D660" t="inlineStr" s="2">
@@ -18673,77 +18609,77 @@
       <c r="F660" s="2"/>
       <c r="G660" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
+          <t xml:space="preserve">Estrutura JSON livre</t>
         </is>
       </c>
     </row>
     <row r="661">
       <c r="A661" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">automacoes</t>
         </is>
       </c>
       <c r="B661" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">acao</t>
         </is>
       </c>
       <c r="C661" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D661" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E661" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">criar_atividade | enviar_whatsapp | enviar_email | mudar_status</t>
+        </is>
+      </c>
       <c r="F661" s="2"/>
-      <c r="G661" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G661" s="2"/>
     </row>
     <row r="662">
       <c r="A662" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">automacoes</t>
         </is>
       </c>
       <c r="B662" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_id</t>
+          <t xml:space="preserve">configuracao_acao</t>
         </is>
       </c>
       <c r="C662" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D662" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E662" s="2"/>
-      <c r="F662" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
-      <c r="G662" s="2"/>
+      <c r="F662" s="2"/>
+      <c r="G662" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Estrutura JSON livre</t>
+        </is>
+      </c>
     </row>
     <row r="663">
       <c r="A663" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">automacoes</t>
         </is>
       </c>
       <c r="B663" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_negocio</t>
+          <t xml:space="preserve">destino</t>
         </is>
       </c>
       <c r="C663" t="inlineStr" s="2">
@@ -18753,12 +18689,12 @@
       </c>
       <c r="D663" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E663" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">venda usina | bateria | expansão | renovação | serviço | venda bateria</t>
+          <t xml:space="preserve">cliente_evento | responsavel_empresa | cliente_especifico</t>
         </is>
       </c>
       <c r="F663" s="2"/>
@@ -18767,17 +18703,17 @@
     <row r="664">
       <c r="A664" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">automacoes</t>
         </is>
       </c>
       <c r="B664" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">valor_estimado</t>
+          <t xml:space="preserve">cliente_especifico_id</t>
         </is>
       </c>
       <c r="C664" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D664" t="inlineStr" s="2">
@@ -18786,23 +18722,27 @@
         </is>
       </c>
       <c r="E664" s="2"/>
-      <c r="F664" s="2"/>
+      <c r="F664" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G664" s="2"/>
     </row>
     <row r="665">
       <c r="A665" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">automacoes</t>
         </is>
       </c>
       <c r="B665" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">valor_final</t>
+          <t xml:space="preserve">ativa</t>
         </is>
       </c>
       <c r="C665" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D665" t="inlineStr" s="2">
@@ -18810,24 +18750,28 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E665" s="2"/>
+      <c r="E665" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F665" s="2"/>
       <c r="G665" s="2"/>
     </row>
     <row r="666">
       <c r="A666" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">automacoes</t>
         </is>
       </c>
       <c r="B666" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">etapa_funil</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C666" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D666" t="inlineStr" s="2">
@@ -18835,28 +18779,28 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E666" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">novo lead | qualificado | proposta enviada | negociação | contrato assinado</t>
-        </is>
-      </c>
+      <c r="E666" s="2"/>
       <c r="F666" s="2"/>
-      <c r="G666" s="2"/>
+      <c r="G666" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="667">
       <c r="A667" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">automacoes</t>
         </is>
       </c>
       <c r="B667" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">probabilidade</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C667" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D667" t="inlineStr" s="2">
@@ -18866,42 +18810,50 @@
       </c>
       <c r="E667" s="2"/>
       <c r="F667" s="2"/>
-      <c r="G667" s="2"/>
+      <c r="G667" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="668">
       <c r="A668" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">automacoes_execucoes</t>
         </is>
       </c>
       <c r="B668" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_previsao_fechamento</t>
+          <t xml:space="preserve">automacao</t>
         </is>
       </c>
       <c r="C668" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D668" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E668" s="2"/>
-      <c r="F668" s="2"/>
+      <c r="F668" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">automacoes</t>
+        </is>
+      </c>
       <c r="G668" s="2"/>
     </row>
     <row r="669">
       <c r="A669" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">automacoes_execucoes</t>
         </is>
       </c>
       <c r="B669" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_fechamento</t>
+          <t xml:space="preserve">data_execucao</t>
         </is>
       </c>
       <c r="C669" t="inlineStr" s="2">
@@ -18911,7 +18863,7 @@
       </c>
       <c r="D669" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E669" s="2"/>
@@ -18921,17 +18873,17 @@
     <row r="670">
       <c r="A670" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">automacoes_execucoes</t>
         </is>
       </c>
       <c r="B670" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">sucesso</t>
         </is>
       </c>
       <c r="C670" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D670" t="inlineStr" s="2">
@@ -18941,7 +18893,7 @@
       </c>
       <c r="E670" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">em andamento | ganho | perdido</t>
+          <t xml:space="preserve">true / false</t>
         </is>
       </c>
       <c r="F670" s="2"/>
@@ -18950,12 +18902,12 @@
     <row r="671">
       <c r="A671" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">automacoes_execucoes</t>
         </is>
       </c>
       <c r="B671" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">motivo_perda</t>
+          <t xml:space="preserve">mensagem</t>
         </is>
       </c>
       <c r="C671" t="inlineStr" s="2">
@@ -18975,17 +18927,17 @@
     <row r="672">
       <c r="A672" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">automacoes_execucoes</t>
         </is>
       </c>
       <c r="B672" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">reabertura</t>
+          <t xml:space="preserve">referencia_registro</t>
         </is>
       </c>
       <c r="C672" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D672" t="inlineStr" s="2">
@@ -18993,28 +18945,24 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E672" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E672" s="2"/>
       <c r="F672" s="2"/>
       <c r="G672" s="2"/>
     </row>
     <row r="673">
       <c r="A673" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">automacoes_execucoes</t>
         </is>
       </c>
       <c r="B673" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">motivo_reabertura</t>
+          <t xml:space="preserve">cliente</t>
         </is>
       </c>
       <c r="C673" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D673" t="inlineStr" s="2">
@@ -19023,23 +18971,27 @@
         </is>
       </c>
       <c r="E673" s="2"/>
-      <c r="F673" s="2"/>
+      <c r="F673" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G673" s="2"/>
     </row>
     <row r="674">
       <c r="A674" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">automacoes_execucoes</t>
         </is>
       </c>
       <c r="B674" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">condicao_pagamento</t>
+          <t xml:space="preserve">dados_execucao</t>
         </is>
       </c>
       <c r="C674" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D674" t="inlineStr" s="2">
@@ -19049,12 +19001,16 @@
       </c>
       <c r="E674" s="2"/>
       <c r="F674" s="2"/>
-      <c r="G674" s="2"/>
+      <c r="G674" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Estrutura JSON livre</t>
+        </is>
+      </c>
     </row>
     <row r="675">
       <c r="A675" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">automacoes_execucoes</t>
         </is>
       </c>
       <c r="B675" t="inlineStr" s="2">
@@ -19083,7 +19039,7 @@
     <row r="676">
       <c r="A676" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">automacoes_execucoes</t>
         </is>
       </c>
       <c r="B676" t="inlineStr" s="2">
@@ -19112,12 +19068,12 @@
     <row r="677">
       <c r="A677" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">notificacoes_internas</t>
         </is>
       </c>
       <c r="B677" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_venda</t>
+          <t xml:space="preserve">tipo</t>
         </is>
       </c>
       <c r="C677" t="inlineStr" s="2">
@@ -19127,12 +19083,12 @@
       </c>
       <c r="D677" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E677" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Energia Solar | O&amp;M (Operação e Manutenção) | Baterias | Carregadores Veículos Elétricos</t>
+          <t xml:space="preserve">atividade_atrasada | lembrete | sistema</t>
         </is>
       </c>
       <c r="F677" s="2"/>
@@ -19141,7 +19097,7 @@
     <row r="678">
       <c r="A678" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">notificacoes_internas</t>
         </is>
       </c>
       <c r="B678" t="inlineStr" s="2">
@@ -19156,7 +19112,7 @@
       </c>
       <c r="D678" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E678" s="2"/>
@@ -19166,17 +19122,17 @@
     <row r="679">
       <c r="A679" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">notificacoes_internas</t>
         </is>
       </c>
       <c r="B679" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">valor</t>
+          <t xml:space="preserve">mensagem</t>
         </is>
       </c>
       <c r="C679" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D679" t="inlineStr" s="2">
@@ -19191,12 +19147,12 @@
     <row r="680">
       <c r="A680" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">notificacoes_internas</t>
         </is>
       </c>
       <c r="B680" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">consultor_responsavel</t>
+          <t xml:space="preserve">atividade_id</t>
         </is>
       </c>
       <c r="C680" t="inlineStr" s="2">
@@ -19212,10 +19168,791 @@
       <c r="E680" s="2"/>
       <c r="F680" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">atividades</t>
+        </is>
+      </c>
+      <c r="G680" s="2"/>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">notificacoes_internas</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">cliente_id</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">relation</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E681" s="2"/>
+      <c r="F681" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
+      <c r="G681" s="2"/>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">notificacoes_internas</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">cliente_nome</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E682" s="2"/>
+      <c r="F682" s="2"/>
+      <c r="G682" s="2"/>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">notificacoes_internas</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">data_prevista</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">date</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E683" s="2"/>
+      <c r="F683" s="2"/>
+      <c r="G683" s="2"/>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">notificacoes_internas</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">dias_atraso</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E684" s="2"/>
+      <c r="F684" s="2"/>
+      <c r="G684" s="2"/>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">notificacoes_internas</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">lida</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">bool</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
+      <c r="F685" s="2"/>
+      <c r="G685" s="2"/>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">notificacoes_internas</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">lida_em</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">date</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E686" s="2"/>
+      <c r="F686" s="2"/>
+      <c r="G686" s="2"/>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">notificacoes_internas</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">status</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">select</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativa | resolvida | arquivada</t>
+        </is>
+      </c>
+      <c r="F687" s="2"/>
+      <c r="G687" s="2"/>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">notificacoes_internas</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">resolvida_em</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">date</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E688" s="2"/>
+      <c r="F688" s="2"/>
+      <c r="G688" s="2"/>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">notificacoes_internas</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">created</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E689" s="2"/>
+      <c r="F689" s="2"/>
+      <c r="G689" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">notificacoes_internas</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">updated</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E690" s="2"/>
+      <c r="F690" s="2"/>
+      <c r="G690" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">cliente_id</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">relation</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E691" s="2"/>
+      <c r="F691" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
+      <c r="G691" s="2"/>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">tipo_negocio</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">select</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">venda usina | bateria | expansão | renovação | serviço | venda bateria</t>
+        </is>
+      </c>
+      <c r="F692" s="2"/>
+      <c r="G692" s="2"/>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">valor_estimado</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E693" s="2"/>
+      <c r="F693" s="2"/>
+      <c r="G693" s="2"/>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">valor_final</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E694" s="2"/>
+      <c r="F694" s="2"/>
+      <c r="G694" s="2"/>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">etapa_funil</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">select</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">novo lead | qualificado | proposta enviada | negociação | contrato assinado</t>
+        </is>
+      </c>
+      <c r="F695" s="2"/>
+      <c r="G695" s="2"/>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">probabilidade</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E696" s="2"/>
+      <c r="F696" s="2"/>
+      <c r="G696" s="2"/>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">data_previsao_fechamento</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">date</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E697" s="2"/>
+      <c r="F697" s="2"/>
+      <c r="G697" s="2"/>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">data_fechamento</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">date</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E698" s="2"/>
+      <c r="F698" s="2"/>
+      <c r="G698" s="2"/>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">status</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">select</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">em andamento | ganho | perdido</t>
+        </is>
+      </c>
+      <c r="F699" s="2"/>
+      <c r="G699" s="2"/>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">motivo_perda</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E700" s="2"/>
+      <c r="F700" s="2"/>
+      <c r="G700" s="2"/>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">reabertura</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">bool</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
+      <c r="F701" s="2"/>
+      <c r="G701" s="2"/>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">motivo_reabertura</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E702" s="2"/>
+      <c r="F702" s="2"/>
+      <c r="G702" s="2"/>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">condicao_pagamento</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E703" s="2"/>
+      <c r="F703" s="2"/>
+      <c r="G703" s="2"/>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">created</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E704" s="2"/>
+      <c r="F704" s="2"/>
+      <c r="G704" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">updated</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E705" s="2"/>
+      <c r="F705" s="2"/>
+      <c r="G705" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">tipo_venda</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">select</t>
+        </is>
+      </c>
+      <c r="D706" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Energia Solar | O&amp;M (Operação e Manutenção) | Baterias | Carregadores Veículos Elétricos</t>
+        </is>
+      </c>
+      <c r="F706" s="2"/>
+      <c r="G706" s="2"/>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">titulo</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E707" s="2"/>
+      <c r="F707" s="2"/>
+      <c r="G707" s="2"/>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">valor</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E708" s="2"/>
+      <c r="F708" s="2"/>
+      <c r="G708" s="2"/>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">consultor_responsavel</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">relation</t>
+        </is>
+      </c>
+      <c r="D709" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E709" s="2"/>
+      <c r="F709" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">users</t>
         </is>
       </c>
-      <c r="G680" s="2"/>
+      <c r="G709" s="2"/>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>

<commit_message>
feat: adicionar upload de datasheet PDF com extração automática no cadastro de equipamentos e link na ficha da usina
</commit_message>
<xml_diff>
--- a/public/schema-delfos-solar.xlsx
+++ b/public/schema-delfos-solar.xlsx
@@ -1057,7 +1057,7 @@
         </is>
       </c>
       <c r="C35" s="2">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D35" t="inlineStr" s="2">
         <is>
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="C41" s="2">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="2">
@@ -18321,27 +18321,31 @@
     <row r="650">
       <c r="A650" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">parametros_tarifarios</t>
+          <t xml:space="preserve">equipamentos</t>
         </is>
       </c>
       <c r="B650" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ano</t>
+          <t xml:space="preserve">datasheet_pdf</t>
         </is>
       </c>
       <c r="C650" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="D650" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E650" s="2"/>
       <c r="F650" s="2"/>
-      <c r="G650" s="2"/>
+      <c r="G650" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
+        </is>
+      </c>
     </row>
     <row r="651">
       <c r="A651" t="inlineStr" s="2">
@@ -18351,12 +18355,12 @@
       </c>
       <c r="B651" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">classe</t>
+          <t xml:space="preserve">ano</t>
         </is>
       </c>
       <c r="C651" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D651" t="inlineStr" s="2">
@@ -18364,11 +18368,7 @@
           <t xml:space="preserve">Sim</t>
         </is>
       </c>
-      <c r="E651" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">residencial | comercial</t>
-        </is>
-      </c>
+      <c r="E651" s="2"/>
       <c r="F651" s="2"/>
       <c r="G651" s="2"/>
     </row>
@@ -18380,20 +18380,24 @@
       </c>
       <c r="B652" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tarifa</t>
+          <t xml:space="preserve">classe</t>
         </is>
       </c>
       <c r="C652" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D652" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E652" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">residencial | comercial</t>
+        </is>
+      </c>
       <c r="F652" s="2"/>
       <c r="G652" s="2"/>
     </row>
@@ -18405,7 +18409,7 @@
       </c>
       <c r="B653" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fio_b</t>
+          <t xml:space="preserve">tarifa</t>
         </is>
       </c>
       <c r="C653" t="inlineStr" s="2">
@@ -18430,7 +18434,7 @@
       </c>
       <c r="B654" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fs</t>
+          <t xml:space="preserve">fio_b</t>
         </is>
       </c>
       <c r="C654" t="inlineStr" s="2">
@@ -18455,7 +18459,7 @@
       </c>
       <c r="B655" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gd_eco_liquida</t>
+          <t xml:space="preserve">fs</t>
         </is>
       </c>
       <c r="C655" t="inlineStr" s="2">
@@ -18480,12 +18484,12 @@
       </c>
       <c r="B656" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">gd_eco_liquida</t>
         </is>
       </c>
       <c r="C656" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D656" t="inlineStr" s="2">
@@ -18495,11 +18499,7 @@
       </c>
       <c r="E656" s="2"/>
       <c r="F656" s="2"/>
-      <c r="G656" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G656" s="2"/>
     </row>
     <row r="657">
       <c r="A657" t="inlineStr" s="2">
@@ -18509,7 +18509,7 @@
       </c>
       <c r="B657" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C657" t="inlineStr" s="2">
@@ -18526,34 +18526,38 @@
       <c r="F657" s="2"/>
       <c r="G657" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="658">
       <c r="A658" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">parametros_tarifarios</t>
         </is>
       </c>
       <c r="B658" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">nome</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C658" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D658" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E658" s="2"/>
       <c r="F658" s="2"/>
-      <c r="G658" s="2"/>
+      <c r="G658" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="659">
       <c r="A659" t="inlineStr" s="2">
@@ -18563,12 +18567,12 @@
       </c>
       <c r="B659" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gatilho</t>
+          <t xml:space="preserve">nome</t>
         </is>
       </c>
       <c r="C659" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D659" t="inlineStr" s="2">
@@ -18576,11 +18580,7 @@
           <t xml:space="preserve">Sim</t>
         </is>
       </c>
-      <c r="E659" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">status_mudou | instalacao_concluida | atividade_concluida | data_especifica | dias_apos_evento</t>
-        </is>
-      </c>
+      <c r="E659" s="2"/>
       <c r="F659" s="2"/>
       <c r="G659" s="2"/>
     </row>
@@ -18592,26 +18592,26 @@
       </c>
       <c r="B660" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">configuracao_gatilho</t>
+          <t xml:space="preserve">gatilho</t>
         </is>
       </c>
       <c r="C660" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D660" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E660" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">status_mudou | instalacao_concluida | atividade_concluida | data_especifica | dias_apos_evento</t>
+        </is>
+      </c>
       <c r="F660" s="2"/>
-      <c r="G660" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="G660" s="2"/>
     </row>
     <row r="661">
       <c r="A661" t="inlineStr" s="2">
@@ -18621,26 +18621,26 @@
       </c>
       <c r="B661" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">acao</t>
+          <t xml:space="preserve">configuracao_gatilho</t>
         </is>
       </c>
       <c r="C661" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D661" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E661" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">criar_atividade | enviar_whatsapp | enviar_email | mudar_status</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E661" s="2"/>
       <c r="F661" s="2"/>
-      <c r="G661" s="2"/>
+      <c r="G661" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Estrutura JSON livre</t>
+        </is>
+      </c>
     </row>
     <row r="662">
       <c r="A662" t="inlineStr" s="2">
@@ -18650,26 +18650,26 @@
       </c>
       <c r="B662" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">configuracao_acao</t>
+          <t xml:space="preserve">acao</t>
         </is>
       </c>
       <c r="C662" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D662" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E662" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">criar_atividade | enviar_whatsapp | enviar_email | mudar_status</t>
+        </is>
+      </c>
       <c r="F662" s="2"/>
-      <c r="G662" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="G662" s="2"/>
     </row>
     <row r="663">
       <c r="A663" t="inlineStr" s="2">
@@ -18679,26 +18679,26 @@
       </c>
       <c r="B663" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">destino</t>
+          <t xml:space="preserve">configuracao_acao</t>
         </is>
       </c>
       <c r="C663" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D663" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E663" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">cliente_evento | responsavel_empresa | cliente_especifico</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E663" s="2"/>
       <c r="F663" s="2"/>
-      <c r="G663" s="2"/>
+      <c r="G663" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Estrutura JSON livre</t>
+        </is>
+      </c>
     </row>
     <row r="664">
       <c r="A664" t="inlineStr" s="2">
@@ -18708,25 +18708,25 @@
       </c>
       <c r="B664" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_especifico_id</t>
+          <t xml:space="preserve">destino</t>
         </is>
       </c>
       <c r="C664" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D664" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E664" s="2"/>
-      <c r="F664" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">cliente_evento | responsavel_empresa | cliente_especifico</t>
+        </is>
+      </c>
+      <c r="F664" s="2"/>
       <c r="G664" s="2"/>
     </row>
     <row r="665">
@@ -18737,12 +18737,12 @@
       </c>
       <c r="B665" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ativa</t>
+          <t xml:space="preserve">cliente_especifico_id</t>
         </is>
       </c>
       <c r="C665" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D665" t="inlineStr" s="2">
@@ -18750,12 +18750,12 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E665" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
-      <c r="F665" s="2"/>
+      <c r="E665" s="2"/>
+      <c r="F665" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G665" s="2"/>
     </row>
     <row r="666">
@@ -18766,12 +18766,12 @@
       </c>
       <c r="B666" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">ativa</t>
         </is>
       </c>
       <c r="C666" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D666" t="inlineStr" s="2">
@@ -18779,13 +18779,13 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E666" s="2"/>
+      <c r="E666" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F666" s="2"/>
-      <c r="G666" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G666" s="2"/>
     </row>
     <row r="667">
       <c r="A667" t="inlineStr" s="2">
@@ -18795,7 +18795,7 @@
       </c>
       <c r="B667" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C667" t="inlineStr" s="2">
@@ -18812,38 +18812,38 @@
       <c r="F667" s="2"/>
       <c r="G667" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="668">
       <c r="A668" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes_execucoes</t>
+          <t xml:space="preserve">automacoes</t>
         </is>
       </c>
       <c r="B668" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacao</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C668" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D668" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E668" s="2"/>
-      <c r="F668" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">automacoes</t>
-        </is>
-      </c>
-      <c r="G668" s="2"/>
+      <c r="F668" s="2"/>
+      <c r="G668" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="669">
       <c r="A669" t="inlineStr" s="2">
@@ -18853,12 +18853,12 @@
       </c>
       <c r="B669" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_execucao</t>
+          <t xml:space="preserve">automacao</t>
         </is>
       </c>
       <c r="C669" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D669" t="inlineStr" s="2">
@@ -18867,7 +18867,11 @@
         </is>
       </c>
       <c r="E669" s="2"/>
-      <c r="F669" s="2"/>
+      <c r="F669" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">automacoes</t>
+        </is>
+      </c>
       <c r="G669" s="2"/>
     </row>
     <row r="670">
@@ -18878,24 +18882,20 @@
       </c>
       <c r="B670" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">sucesso</t>
+          <t xml:space="preserve">data_execucao</t>
         </is>
       </c>
       <c r="C670" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D670" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E670" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E670" s="2"/>
       <c r="F670" s="2"/>
       <c r="G670" s="2"/>
     </row>
@@ -18907,12 +18907,12 @@
       </c>
       <c r="B671" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mensagem</t>
+          <t xml:space="preserve">sucesso</t>
         </is>
       </c>
       <c r="C671" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D671" t="inlineStr" s="2">
@@ -18920,7 +18920,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E671" s="2"/>
+      <c r="E671" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F671" s="2"/>
       <c r="G671" s="2"/>
     </row>
@@ -18932,7 +18936,7 @@
       </c>
       <c r="B672" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">referencia_registro</t>
+          <t xml:space="preserve">mensagem</t>
         </is>
       </c>
       <c r="C672" t="inlineStr" s="2">
@@ -18957,12 +18961,12 @@
       </c>
       <c r="B673" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente</t>
+          <t xml:space="preserve">referencia_registro</t>
         </is>
       </c>
       <c r="C673" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D673" t="inlineStr" s="2">
@@ -18971,11 +18975,7 @@
         </is>
       </c>
       <c r="E673" s="2"/>
-      <c r="F673" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+      <c r="F673" s="2"/>
       <c r="G673" s="2"/>
     </row>
     <row r="674">
@@ -18986,12 +18986,12 @@
       </c>
       <c r="B674" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">dados_execucao</t>
+          <t xml:space="preserve">cliente</t>
         </is>
       </c>
       <c r="C674" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D674" t="inlineStr" s="2">
@@ -19000,12 +19000,12 @@
         </is>
       </c>
       <c r="E674" s="2"/>
-      <c r="F674" s="2"/>
-      <c r="G674" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="F674" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
+      <c r="G674" s="2"/>
     </row>
     <row r="675">
       <c r="A675" t="inlineStr" s="2">
@@ -19015,12 +19015,12 @@
       </c>
       <c r="B675" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">dados_execucao</t>
         </is>
       </c>
       <c r="C675" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D675" t="inlineStr" s="2">
@@ -19032,7 +19032,7 @@
       <c r="F675" s="2"/>
       <c r="G675" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
+          <t xml:space="preserve">Estrutura JSON livre</t>
         </is>
       </c>
     </row>
@@ -19044,7 +19044,7 @@
       </c>
       <c r="B676" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C676" t="inlineStr" s="2">
@@ -19061,38 +19061,38 @@
       <c r="F676" s="2"/>
       <c r="G676" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="677">
       <c r="A677" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">automacoes_execucoes</t>
         </is>
       </c>
       <c r="B677" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C677" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D677" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E677" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">atividade_atrasada | lembrete | sistema</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E677" s="2"/>
       <c r="F677" s="2"/>
-      <c r="G677" s="2"/>
+      <c r="G677" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="678">
       <c r="A678" t="inlineStr" s="2">
@@ -19102,12 +19102,12 @@
       </c>
       <c r="B678" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">tipo</t>
         </is>
       </c>
       <c r="C678" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D678" t="inlineStr" s="2">
@@ -19115,7 +19115,11 @@
           <t xml:space="preserve">Sim</t>
         </is>
       </c>
-      <c r="E678" s="2"/>
+      <c r="E678" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">atividade_atrasada | lembrete | sistema</t>
+        </is>
+      </c>
       <c r="F678" s="2"/>
       <c r="G678" s="2"/>
     </row>
@@ -19127,7 +19131,7 @@
       </c>
       <c r="B679" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mensagem</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C679" t="inlineStr" s="2">
@@ -19137,7 +19141,7 @@
       </c>
       <c r="D679" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E679" s="2"/>
@@ -19152,12 +19156,12 @@
       </c>
       <c r="B680" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">atividade_id</t>
+          <t xml:space="preserve">mensagem</t>
         </is>
       </c>
       <c r="C680" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D680" t="inlineStr" s="2">
@@ -19166,11 +19170,7 @@
         </is>
       </c>
       <c r="E680" s="2"/>
-      <c r="F680" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">atividades</t>
-        </is>
-      </c>
+      <c r="F680" s="2"/>
       <c r="G680" s="2"/>
     </row>
     <row r="681">
@@ -19181,7 +19181,7 @@
       </c>
       <c r="B681" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_id</t>
+          <t xml:space="preserve">atividade_id</t>
         </is>
       </c>
       <c r="C681" t="inlineStr" s="2">
@@ -19197,7 +19197,7 @@
       <c r="E681" s="2"/>
       <c r="F681" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">clientes</t>
+          <t xml:space="preserve">atividades</t>
         </is>
       </c>
       <c r="G681" s="2"/>
@@ -19210,12 +19210,12 @@
       </c>
       <c r="B682" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_nome</t>
+          <t xml:space="preserve">cliente_id</t>
         </is>
       </c>
       <c r="C682" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D682" t="inlineStr" s="2">
@@ -19224,7 +19224,11 @@
         </is>
       </c>
       <c r="E682" s="2"/>
-      <c r="F682" s="2"/>
+      <c r="F682" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G682" s="2"/>
     </row>
     <row r="683">
@@ -19235,12 +19239,12 @@
       </c>
       <c r="B683" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_prevista</t>
+          <t xml:space="preserve">cliente_nome</t>
         </is>
       </c>
       <c r="C683" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D683" t="inlineStr" s="2">
@@ -19260,12 +19264,12 @@
       </c>
       <c r="B684" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">dias_atraso</t>
+          <t xml:space="preserve">data_prevista</t>
         </is>
       </c>
       <c r="C684" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D684" t="inlineStr" s="2">
@@ -19285,12 +19289,12 @@
       </c>
       <c r="B685" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">lida</t>
+          <t xml:space="preserve">dias_atraso</t>
         </is>
       </c>
       <c r="C685" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D685" t="inlineStr" s="2">
@@ -19298,11 +19302,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E685" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E685" s="2"/>
       <c r="F685" s="2"/>
       <c r="G685" s="2"/>
     </row>
@@ -19314,12 +19314,12 @@
       </c>
       <c r="B686" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">lida_em</t>
+          <t xml:space="preserve">lida</t>
         </is>
       </c>
       <c r="C686" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D686" t="inlineStr" s="2">
@@ -19327,7 +19327,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E686" s="2"/>
+      <c r="E686" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F686" s="2"/>
       <c r="G686" s="2"/>
     </row>
@@ -19339,24 +19343,20 @@
       </c>
       <c r="B687" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">lida_em</t>
         </is>
       </c>
       <c r="C687" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D687" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E687" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">ativa | resolvida | arquivada</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E687" s="2"/>
       <c r="F687" s="2"/>
       <c r="G687" s="2"/>
     </row>
@@ -19368,20 +19368,24 @@
       </c>
       <c r="B688" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">resolvida_em</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="C688" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D688" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E688" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativa | resolvida | arquivada</t>
+        </is>
+      </c>
       <c r="F688" s="2"/>
       <c r="G688" s="2"/>
     </row>
@@ -19393,12 +19397,12 @@
       </c>
       <c r="B689" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">resolvida_em</t>
         </is>
       </c>
       <c r="C689" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D689" t="inlineStr" s="2">
@@ -19408,11 +19412,7 @@
       </c>
       <c r="E689" s="2"/>
       <c r="F689" s="2"/>
-      <c r="G689" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G689" s="2"/>
     </row>
     <row r="690">
       <c r="A690" t="inlineStr" s="2">
@@ -19422,7 +19422,7 @@
       </c>
       <c r="B690" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C690" t="inlineStr" s="2">
@@ -19439,38 +19439,38 @@
       <c r="F690" s="2"/>
       <c r="G690" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="691">
       <c r="A691" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">notificacoes_internas</t>
         </is>
       </c>
       <c r="B691" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_id</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C691" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D691" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E691" s="2"/>
-      <c r="F691" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
-      <c r="G691" s="2"/>
+      <c r="F691" s="2"/>
+      <c r="G691" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="692">
       <c r="A692" t="inlineStr" s="2">
@@ -19480,25 +19480,25 @@
       </c>
       <c r="B692" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_negocio</t>
+          <t xml:space="preserve">cliente_id</t>
         </is>
       </c>
       <c r="C692" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D692" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E692" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">venda usina | bateria | expansão | renovação | serviço | venda bateria</t>
-        </is>
-      </c>
-      <c r="F692" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E692" s="2"/>
+      <c r="F692" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G692" s="2"/>
     </row>
     <row r="693">
@@ -19509,12 +19509,12 @@
       </c>
       <c r="B693" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">valor_estimado</t>
+          <t xml:space="preserve">tipo_negocio</t>
         </is>
       </c>
       <c r="C693" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D693" t="inlineStr" s="2">
@@ -19522,7 +19522,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E693" s="2"/>
+      <c r="E693" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">venda usina | bateria | expansão | renovação | serviço | venda bateria</t>
+        </is>
+      </c>
       <c r="F693" s="2"/>
       <c r="G693" s="2"/>
     </row>
@@ -19534,7 +19538,7 @@
       </c>
       <c r="B694" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">valor_final</t>
+          <t xml:space="preserve">valor_estimado</t>
         </is>
       </c>
       <c r="C694" t="inlineStr" s="2">
@@ -19559,12 +19563,12 @@
       </c>
       <c r="B695" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">etapa_funil</t>
+          <t xml:space="preserve">valor_final</t>
         </is>
       </c>
       <c r="C695" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D695" t="inlineStr" s="2">
@@ -19572,11 +19576,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E695" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">novo lead | qualificado | proposta enviada | negociação | contrato assinado</t>
-        </is>
-      </c>
+      <c r="E695" s="2"/>
       <c r="F695" s="2"/>
       <c r="G695" s="2"/>
     </row>
@@ -19588,12 +19588,12 @@
       </c>
       <c r="B696" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">probabilidade</t>
+          <t xml:space="preserve">etapa_funil</t>
         </is>
       </c>
       <c r="C696" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D696" t="inlineStr" s="2">
@@ -19601,7 +19601,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E696" s="2"/>
+      <c r="E696" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">novo lead | qualificado | proposta enviada | negociação | contrato assinado</t>
+        </is>
+      </c>
       <c r="F696" s="2"/>
       <c r="G696" s="2"/>
     </row>
@@ -19613,12 +19617,12 @@
       </c>
       <c r="B697" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_previsao_fechamento</t>
+          <t xml:space="preserve">probabilidade</t>
         </is>
       </c>
       <c r="C697" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D697" t="inlineStr" s="2">
@@ -19638,7 +19642,7 @@
       </c>
       <c r="B698" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_fechamento</t>
+          <t xml:space="preserve">data_previsao_fechamento</t>
         </is>
       </c>
       <c r="C698" t="inlineStr" s="2">
@@ -19663,12 +19667,12 @@
       </c>
       <c r="B699" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">data_fechamento</t>
         </is>
       </c>
       <c r="C699" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D699" t="inlineStr" s="2">
@@ -19676,11 +19680,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E699" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">em andamento | ganho | perdido</t>
-        </is>
-      </c>
+      <c r="E699" s="2"/>
       <c r="F699" s="2"/>
       <c r="G699" s="2"/>
     </row>
@@ -19692,12 +19692,12 @@
       </c>
       <c r="B700" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">motivo_perda</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="C700" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D700" t="inlineStr" s="2">
@@ -19705,7 +19705,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E700" s="2"/>
+      <c r="E700" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">em andamento | ganho | perdido</t>
+        </is>
+      </c>
       <c r="F700" s="2"/>
       <c r="G700" s="2"/>
     </row>
@@ -19717,12 +19721,12 @@
       </c>
       <c r="B701" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">reabertura</t>
+          <t xml:space="preserve">motivo_perda</t>
         </is>
       </c>
       <c r="C701" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D701" t="inlineStr" s="2">
@@ -19730,11 +19734,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E701" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E701" s="2"/>
       <c r="F701" s="2"/>
       <c r="G701" s="2"/>
     </row>
@@ -19746,12 +19746,12 @@
       </c>
       <c r="B702" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">motivo_reabertura</t>
+          <t xml:space="preserve">reabertura</t>
         </is>
       </c>
       <c r="C702" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D702" t="inlineStr" s="2">
@@ -19759,7 +19759,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E702" s="2"/>
+      <c r="E702" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F702" s="2"/>
       <c r="G702" s="2"/>
     </row>
@@ -19771,7 +19775,7 @@
       </c>
       <c r="B703" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">condicao_pagamento</t>
+          <t xml:space="preserve">motivo_reabertura</t>
         </is>
       </c>
       <c r="C703" t="inlineStr" s="2">
@@ -19796,12 +19800,12 @@
       </c>
       <c r="B704" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">condicao_pagamento</t>
         </is>
       </c>
       <c r="C704" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D704" t="inlineStr" s="2">
@@ -19811,11 +19815,7 @@
       </c>
       <c r="E704" s="2"/>
       <c r="F704" s="2"/>
-      <c r="G704" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G704" s="2"/>
     </row>
     <row r="705">
       <c r="A705" t="inlineStr" s="2">
@@ -19825,7 +19825,7 @@
       </c>
       <c r="B705" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C705" t="inlineStr" s="2">
@@ -19842,7 +19842,7 @@
       <c r="F705" s="2"/>
       <c r="G705" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
@@ -19854,12 +19854,12 @@
       </c>
       <c r="B706" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_venda</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C706" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D706" t="inlineStr" s="2">
@@ -19867,13 +19867,13 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E706" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Energia Solar | O&amp;M (Operação e Manutenção) | Baterias | Carregadores Veículos Elétricos</t>
-        </is>
-      </c>
+      <c r="E706" s="2"/>
       <c r="F706" s="2"/>
-      <c r="G706" s="2"/>
+      <c r="G706" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="707">
       <c r="A707" t="inlineStr" s="2">
@@ -19883,12 +19883,12 @@
       </c>
       <c r="B707" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">tipo_venda</t>
         </is>
       </c>
       <c r="C707" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D707" t="inlineStr" s="2">
@@ -19896,7 +19896,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E707" s="2"/>
+      <c r="E707" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Energia Solar | O&amp;M (Operação e Manutenção) | Baterias | Carregadores Veículos Elétricos</t>
+        </is>
+      </c>
       <c r="F707" s="2"/>
       <c r="G707" s="2"/>
     </row>
@@ -19908,12 +19912,12 @@
       </c>
       <c r="B708" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">valor</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C708" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D708" t="inlineStr" s="2">
@@ -19933,26 +19937,51 @@
       </c>
       <c r="B709" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">valor</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D709" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E709" s="2"/>
+      <c r="F709" s="2"/>
+      <c r="G709" s="2"/>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">consultor_responsavel</t>
         </is>
       </c>
-      <c r="C709" t="inlineStr" s="2">
+      <c r="C710" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">relation</t>
         </is>
       </c>
-      <c r="D709" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E709" s="2"/>
-      <c r="F709" t="inlineStr" s="2">
+      <c r="D710" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E710" s="2"/>
+      <c r="F710" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">users</t>
         </is>
       </c>
-      <c r="G709" s="2"/>
+      <c r="G710" s="2"/>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>

<commit_message>
No CRM Delfos Solar (React + Vite + TS + Tailwind/shadcn, backend Pocke…
</commit_message>
<xml_diff>
--- a/public/schema-delfos-solar.xlsx
+++ b/public/schema-delfos-solar.xlsx
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="C28" s="2">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D28" t="inlineStr" s="2">
         <is>
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="C41" s="2">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="2">
@@ -15738,27 +15738,31 @@
     <row r="551">
       <c r="A551" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">monitoramento_marcas</t>
+          <t xml:space="preserve">ordens_servico</t>
         </is>
       </c>
       <c r="B551" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">marca</t>
+          <t xml:space="preserve">relatorio_pdf</t>
         </is>
       </c>
       <c r="C551" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="D551" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E551" s="2"/>
       <c r="F551" s="2"/>
-      <c r="G551" s="2"/>
+      <c r="G551" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
+        </is>
+      </c>
     </row>
     <row r="552">
       <c r="A552" t="inlineStr" s="2">
@@ -15768,7 +15772,7 @@
       </c>
       <c r="B552" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">app_nome</t>
+          <t xml:space="preserve">marca</t>
         </is>
       </c>
       <c r="C552" t="inlineStr" s="2">
@@ -15778,7 +15782,7 @@
       </c>
       <c r="D552" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E552" s="2"/>
@@ -15793,7 +15797,7 @@
       </c>
       <c r="B553" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">login_padrao</t>
+          <t xml:space="preserve">app_nome</t>
         </is>
       </c>
       <c r="C553" t="inlineStr" s="2">
@@ -15818,7 +15822,7 @@
       </c>
       <c r="B554" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">senha_padrao</t>
+          <t xml:space="preserve">login_padrao</t>
         </is>
       </c>
       <c r="C554" t="inlineStr" s="2">
@@ -15843,7 +15847,7 @@
       </c>
       <c r="B555" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">datalogger_url</t>
+          <t xml:space="preserve">senha_padrao</t>
         </is>
       </c>
       <c r="C555" t="inlineStr" s="2">
@@ -15868,7 +15872,7 @@
       </c>
       <c r="B556" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">instrucoes</t>
+          <t xml:space="preserve">datalogger_url</t>
         </is>
       </c>
       <c r="C556" t="inlineStr" s="2">
@@ -15893,12 +15897,12 @@
       </c>
       <c r="B557" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">instrucoes</t>
         </is>
       </c>
       <c r="C557" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D557" t="inlineStr" s="2">
@@ -15908,11 +15912,7 @@
       </c>
       <c r="E557" s="2"/>
       <c r="F557" s="2"/>
-      <c r="G557" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G557" s="2"/>
     </row>
     <row r="558">
       <c r="A558" t="inlineStr" s="2">
@@ -15922,7 +15922,7 @@
       </c>
       <c r="B558" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C558" t="inlineStr" s="2">
@@ -15939,38 +15939,38 @@
       <c r="F558" s="2"/>
       <c r="G558" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="559">
       <c r="A559" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_inversores</t>
+          <t xml:space="preserve">monitoramento_marcas</t>
         </is>
       </c>
       <c r="B559" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_id</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C559" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D559" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E559" s="2"/>
-      <c r="F559" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
-      <c r="G559" s="2"/>
+      <c r="F559" s="2"/>
+      <c r="G559" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="560">
       <c r="A560" t="inlineStr" s="2">
@@ -15980,21 +15980,25 @@
       </c>
       <c r="B560" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">marca_inversor</t>
+          <t xml:space="preserve">cliente_id</t>
         </is>
       </c>
       <c r="C560" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D560" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E560" s="2"/>
-      <c r="F560" s="2"/>
+      <c r="F560" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G560" s="2"/>
     </row>
     <row r="561">
@@ -16005,7 +16009,7 @@
       </c>
       <c r="B561" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">modelo_inversor</t>
+          <t xml:space="preserve">marca_inversor</t>
         </is>
       </c>
       <c r="C561" t="inlineStr" s="2">
@@ -16030,12 +16034,12 @@
       </c>
       <c r="B562" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">potencia_kwp</t>
+          <t xml:space="preserve">modelo_inversor</t>
         </is>
       </c>
       <c r="C562" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D562" t="inlineStr" s="2">
@@ -16055,12 +16059,12 @@
       </c>
       <c r="B563" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">numero_serie</t>
+          <t xml:space="preserve">potencia_kwp</t>
         </is>
       </c>
       <c r="C563" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D563" t="inlineStr" s="2">
@@ -16080,7 +16084,7 @@
       </c>
       <c r="B564" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">app_nome</t>
+          <t xml:space="preserve">numero_serie</t>
         </is>
       </c>
       <c r="C564" t="inlineStr" s="2">
@@ -16105,7 +16109,7 @@
       </c>
       <c r="B565" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">login</t>
+          <t xml:space="preserve">app_nome</t>
         </is>
       </c>
       <c r="C565" t="inlineStr" s="2">
@@ -16130,7 +16134,7 @@
       </c>
       <c r="B566" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">senha</t>
+          <t xml:space="preserve">login</t>
         </is>
       </c>
       <c r="C566" t="inlineStr" s="2">
@@ -16155,7 +16159,7 @@
       </c>
       <c r="B567" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">datalogger_url</t>
+          <t xml:space="preserve">senha</t>
         </is>
       </c>
       <c r="C567" t="inlineStr" s="2">
@@ -16180,7 +16184,7 @@
       </c>
       <c r="B568" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">observacoes</t>
+          <t xml:space="preserve">datalogger_url</t>
         </is>
       </c>
       <c r="C568" t="inlineStr" s="2">
@@ -16205,12 +16209,12 @@
       </c>
       <c r="B569" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ordem</t>
+          <t xml:space="preserve">observacoes</t>
         </is>
       </c>
       <c r="C569" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D569" t="inlineStr" s="2">
@@ -16230,12 +16234,12 @@
       </c>
       <c r="B570" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">ordem</t>
         </is>
       </c>
       <c r="C570" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D570" t="inlineStr" s="2">
@@ -16245,11 +16249,7 @@
       </c>
       <c r="E570" s="2"/>
       <c r="F570" s="2"/>
-      <c r="G570" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G570" s="2"/>
     </row>
     <row r="571">
       <c r="A571" t="inlineStr" s="2">
@@ -16259,7 +16259,7 @@
       </c>
       <c r="B571" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C571" t="inlineStr" s="2">
@@ -16276,38 +16276,38 @@
       <c r="F571" s="2"/>
       <c r="G571" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="572">
       <c r="A572" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">usinas</t>
+          <t xml:space="preserve">cliente_inversores</t>
         </is>
       </c>
       <c r="B572" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_id</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C572" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D572" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E572" s="2"/>
-      <c r="F572" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
-      <c r="G572" s="2"/>
+      <c r="F572" s="2"/>
+      <c r="G572" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="573">
       <c r="A573" t="inlineStr" s="2">
@@ -16317,12 +16317,12 @@
       </c>
       <c r="B573" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">nome</t>
+          <t xml:space="preserve">cliente_id</t>
         </is>
       </c>
       <c r="C573" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D573" t="inlineStr" s="2">
@@ -16331,7 +16331,11 @@
         </is>
       </c>
       <c r="E573" s="2"/>
-      <c r="F573" s="2"/>
+      <c r="F573" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G573" s="2"/>
     </row>
     <row r="574">
@@ -16342,7 +16346,7 @@
       </c>
       <c r="B574" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">endereco</t>
+          <t xml:space="preserve">nome</t>
         </is>
       </c>
       <c r="C574" t="inlineStr" s="2">
@@ -16352,7 +16356,7 @@
       </c>
       <c r="D574" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E574" s="2"/>
@@ -16367,12 +16371,12 @@
       </c>
       <c r="B575" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">potencia_kwp</t>
+          <t xml:space="preserve">endereco</t>
         </is>
       </c>
       <c r="C575" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D575" t="inlineStr" s="2">
@@ -16392,7 +16396,7 @@
       </c>
       <c r="B576" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">qtd_modulos</t>
+          <t xml:space="preserve">potencia_kwp</t>
         </is>
       </c>
       <c r="C576" t="inlineStr" s="2">
@@ -16417,12 +16421,12 @@
       </c>
       <c r="B577" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">inversores_info</t>
+          <t xml:space="preserve">qtd_modulos</t>
         </is>
       </c>
       <c r="C577" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D577" t="inlineStr" s="2">
@@ -16442,12 +16446,12 @@
       </c>
       <c r="B578" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_estrutura</t>
+          <t xml:space="preserve">inversores_info</t>
         </is>
       </c>
       <c r="C578" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D578" t="inlineStr" s="2">
@@ -16455,11 +16459,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E578" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">solo | telhado</t>
-        </is>
-      </c>
+      <c r="E578" s="2"/>
       <c r="F578" s="2"/>
       <c r="G578" s="2"/>
     </row>
@@ -16471,12 +16471,12 @@
       </c>
       <c r="B579" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contrato_id</t>
+          <t xml:space="preserve">tipo_estrutura</t>
         </is>
       </c>
       <c r="C579" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D579" t="inlineStr" s="2">
@@ -16484,12 +16484,12 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E579" s="2"/>
-      <c r="F579" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">contratos_om</t>
-        </is>
-      </c>
+      <c r="E579" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">solo | telhado</t>
+        </is>
+      </c>
+      <c r="F579" s="2"/>
       <c r="G579" s="2"/>
     </row>
     <row r="580">
@@ -16500,12 +16500,12 @@
       </c>
       <c r="B580" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">contrato_id</t>
         </is>
       </c>
       <c r="C580" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D580" t="inlineStr" s="2">
@@ -16514,12 +16514,12 @@
         </is>
       </c>
       <c r="E580" s="2"/>
-      <c r="F580" s="2"/>
-      <c r="G580" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="F580" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contratos_om</t>
+        </is>
+      </c>
+      <c r="G580" s="2"/>
     </row>
     <row r="581">
       <c r="A581" t="inlineStr" s="2">
@@ -16529,7 +16529,7 @@
       </c>
       <c r="B581" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C581" t="inlineStr" s="2">
@@ -16546,7 +16546,7 @@
       <c r="F581" s="2"/>
       <c r="G581" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
@@ -16558,12 +16558,12 @@
       </c>
       <c r="B582" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">geracao_estimada_kwh</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C582" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D582" t="inlineStr" s="2">
@@ -16573,7 +16573,11 @@
       </c>
       <c r="E582" s="2"/>
       <c r="F582" s="2"/>
-      <c r="G582" s="2"/>
+      <c r="G582" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="583">
       <c r="A583" t="inlineStr" s="2">
@@ -16583,12 +16587,12 @@
       </c>
       <c r="B583" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_instalacao</t>
+          <t xml:space="preserve">geracao_estimada_kwh</t>
         </is>
       </c>
       <c r="C583" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D583" t="inlineStr" s="2">
@@ -16608,12 +16612,12 @@
       </c>
       <c r="B584" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">numero_medidor</t>
+          <t xml:space="preserve">data_instalacao</t>
         </is>
       </c>
       <c r="C584" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D584" t="inlineStr" s="2">
@@ -16633,12 +16637,12 @@
       </c>
       <c r="B585" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">numero_medidor</t>
         </is>
       </c>
       <c r="C585" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D585" t="inlineStr" s="2">
@@ -16646,11 +16650,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E585" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">ativo | inativo</t>
-        </is>
-      </c>
+      <c r="E585" s="2"/>
       <c r="F585" s="2"/>
       <c r="G585" s="2"/>
     </row>
@@ -16662,12 +16662,12 @@
       </c>
       <c r="B586" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">observacoes</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="C586" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D586" t="inlineStr" s="2">
@@ -16675,7 +16675,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E586" s="2"/>
+      <c r="E586" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativo | inativo</t>
+        </is>
+      </c>
       <c r="F586" s="2"/>
       <c r="G586" s="2"/>
     </row>
@@ -16687,12 +16691,12 @@
       </c>
       <c r="B587" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_usina</t>
+          <t xml:space="preserve">observacoes</t>
         </is>
       </c>
       <c r="C587" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D587" t="inlineStr" s="2">
@@ -16700,11 +16704,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E587" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">residencial | comercial | industrial | rural | investidor</t>
-        </is>
-      </c>
+      <c r="E587" s="2"/>
       <c r="F587" s="2"/>
       <c r="G587" s="2"/>
     </row>
@@ -16716,12 +16716,12 @@
       </c>
       <c r="B588" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">concessionaria</t>
+          <t xml:space="preserve">tipo_usina</t>
         </is>
       </c>
       <c r="C588" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D588" t="inlineStr" s="2">
@@ -16729,7 +16729,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E588" s="2"/>
+      <c r="E588" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">residencial | comercial | industrial | rural | investidor</t>
+        </is>
+      </c>
       <c r="F588" s="2"/>
       <c r="G588" s="2"/>
     </row>
@@ -16741,7 +16745,7 @@
       </c>
       <c r="B589" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">numero_uc</t>
+          <t xml:space="preserve">concessionaria</t>
         </is>
       </c>
       <c r="C589" t="inlineStr" s="2">
@@ -16766,7 +16770,7 @@
       </c>
       <c r="B590" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">padrao_entrada</t>
+          <t xml:space="preserve">numero_uc</t>
         </is>
       </c>
       <c r="C590" t="inlineStr" s="2">
@@ -16791,12 +16795,12 @@
       </c>
       <c r="B591" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_atendimento</t>
+          <t xml:space="preserve">padrao_entrada</t>
         </is>
       </c>
       <c r="C591" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D591" t="inlineStr" s="2">
@@ -16804,11 +16808,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E591" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">aéreo | subterrâneo</t>
-        </is>
-      </c>
+      <c r="E591" s="2"/>
       <c r="F591" s="2"/>
       <c r="G591" s="2"/>
     </row>
@@ -16820,7 +16820,7 @@
       </c>
       <c r="B592" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">numero_fases</t>
+          <t xml:space="preserve">tipo_atendimento</t>
         </is>
       </c>
       <c r="C592" t="inlineStr" s="2">
@@ -16835,7 +16835,7 @@
       </c>
       <c r="E592" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">monofásico | bifásico | trifásico</t>
+          <t xml:space="preserve">aéreo | subterrâneo</t>
         </is>
       </c>
       <c r="F592" s="2"/>
@@ -16849,12 +16849,12 @@
       </c>
       <c r="B593" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">secao_cabos</t>
+          <t xml:space="preserve">numero_fases</t>
         </is>
       </c>
       <c r="C593" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D593" t="inlineStr" s="2">
@@ -16862,7 +16862,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E593" s="2"/>
+      <c r="E593" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">monofásico | bifásico | trifásico</t>
+        </is>
+      </c>
       <c r="F593" s="2"/>
       <c r="G593" s="2"/>
     </row>
@@ -16874,7 +16878,7 @@
       </c>
       <c r="B594" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">amperagem_disjuntor</t>
+          <t xml:space="preserve">secao_cabos</t>
         </is>
       </c>
       <c r="C594" t="inlineStr" s="2">
@@ -16899,7 +16903,7 @@
       </c>
       <c r="B595" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_caixa_medicao</t>
+          <t xml:space="preserve">amperagem_disjuntor</t>
         </is>
       </c>
       <c r="C595" t="inlineStr" s="2">
@@ -16924,12 +16928,12 @@
       </c>
       <c r="B596" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">latitude</t>
+          <t xml:space="preserve">tipo_caixa_medicao</t>
         </is>
       </c>
       <c r="C596" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D596" t="inlineStr" s="2">
@@ -16949,7 +16953,7 @@
       </c>
       <c r="B597" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">longitude</t>
+          <t xml:space="preserve">latitude</t>
         </is>
       </c>
       <c r="C597" t="inlineStr" s="2">
@@ -16974,7 +16978,7 @@
       </c>
       <c r="B598" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tarifa</t>
+          <t xml:space="preserve">longitude</t>
         </is>
       </c>
       <c r="C598" t="inlineStr" s="2">
@@ -16999,12 +17003,12 @@
       </c>
       <c r="B599" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">classe_consumo</t>
+          <t xml:space="preserve">tarifa</t>
         </is>
       </c>
       <c r="C599" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D599" t="inlineStr" s="2">
@@ -17024,12 +17028,12 @@
       </c>
       <c r="B600" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">geracao_media_mensal_kwh</t>
+          <t xml:space="preserve">classe_consumo</t>
         </is>
       </c>
       <c r="C600" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D600" t="inlineStr" s="2">
@@ -17049,12 +17053,12 @@
       </c>
       <c r="B601" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">monitoramento_app_nome</t>
+          <t xml:space="preserve">geracao_media_mensal_kwh</t>
         </is>
       </c>
       <c r="C601" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D601" t="inlineStr" s="2">
@@ -17074,7 +17078,7 @@
       </c>
       <c r="B602" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">monitoramento_login</t>
+          <t xml:space="preserve">monitoramento_app_nome</t>
         </is>
       </c>
       <c r="C602" t="inlineStr" s="2">
@@ -17099,7 +17103,7 @@
       </c>
       <c r="B603" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">monitoramento_senha</t>
+          <t xml:space="preserve">monitoramento_login</t>
         </is>
       </c>
       <c r="C603" t="inlineStr" s="2">
@@ -17124,7 +17128,7 @@
       </c>
       <c r="B604" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">monitoramento_datalogger_url</t>
+          <t xml:space="preserve">monitoramento_senha</t>
         </is>
       </c>
       <c r="C604" t="inlineStr" s="2">
@@ -17149,7 +17153,7 @@
       </c>
       <c r="B605" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">solarview_login</t>
+          <t xml:space="preserve">monitoramento_datalogger_url</t>
         </is>
       </c>
       <c r="C605" t="inlineStr" s="2">
@@ -17174,7 +17178,7 @@
       </c>
       <c r="B606" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">solarview_senha</t>
+          <t xml:space="preserve">solarview_login</t>
         </is>
       </c>
       <c r="C606" t="inlineStr" s="2">
@@ -17199,7 +17203,7 @@
       </c>
       <c r="B607" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">solarview_link_ios</t>
+          <t xml:space="preserve">solarview_senha</t>
         </is>
       </c>
       <c r="C607" t="inlineStr" s="2">
@@ -17224,7 +17228,7 @@
       </c>
       <c r="B608" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">solarview_link_android</t>
+          <t xml:space="preserve">solarview_link_ios</t>
         </is>
       </c>
       <c r="C608" t="inlineStr" s="2">
@@ -17249,7 +17253,7 @@
       </c>
       <c r="B609" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">solarview_link_texto</t>
+          <t xml:space="preserve">solarview_link_android</t>
         </is>
       </c>
       <c r="C609" t="inlineStr" s="2">
@@ -17274,7 +17278,7 @@
       </c>
       <c r="B610" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fabricante_inversores</t>
+          <t xml:space="preserve">solarview_link_texto</t>
         </is>
       </c>
       <c r="C610" t="inlineStr" s="2">
@@ -17299,7 +17303,7 @@
       </c>
       <c r="B611" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">modelo_inversores</t>
+          <t xml:space="preserve">fabricante_inversores</t>
         </is>
       </c>
       <c r="C611" t="inlineStr" s="2">
@@ -17324,12 +17328,12 @@
       </c>
       <c r="B612" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">potencia_pico_inversores_kwp</t>
+          <t xml:space="preserve">modelo_inversores</t>
         </is>
       </c>
       <c r="C612" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D612" t="inlineStr" s="2">
@@ -17349,12 +17353,12 @@
       </c>
       <c r="B613" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fabricante_modulos</t>
+          <t xml:space="preserve">potencia_pico_inversores_kwp</t>
         </is>
       </c>
       <c r="C613" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D613" t="inlineStr" s="2">
@@ -17374,7 +17378,7 @@
       </c>
       <c r="B614" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">modelo_modulos</t>
+          <t xml:space="preserve">fabricante_modulos</t>
         </is>
       </c>
       <c r="C614" t="inlineStr" s="2">
@@ -17399,12 +17403,12 @@
       </c>
       <c r="B615" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">potencia_pico_modulos_kwp</t>
+          <t xml:space="preserve">modelo_modulos</t>
         </is>
       </c>
       <c r="C615" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D615" t="inlineStr" s="2">
@@ -17424,7 +17428,7 @@
       </c>
       <c r="B616" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">quantidade_placas</t>
+          <t xml:space="preserve">potencia_pico_modulos_kwp</t>
         </is>
       </c>
       <c r="C616" t="inlineStr" s="2">
@@ -17449,12 +17453,12 @@
       </c>
       <c r="B617" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">marca_placas</t>
+          <t xml:space="preserve">quantidade_placas</t>
         </is>
       </c>
       <c r="C617" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D617" t="inlineStr" s="2">
@@ -17474,12 +17478,12 @@
       </c>
       <c r="B618" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_telhado</t>
+          <t xml:space="preserve">marca_placas</t>
         </is>
       </c>
       <c r="C618" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D618" t="inlineStr" s="2">
@@ -17487,41 +17491,37 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E618" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">ceramico | metalico | laje | fibrocimento</t>
-        </is>
-      </c>
+      <c r="E618" s="2"/>
       <c r="F618" s="2"/>
       <c r="G618" s="2"/>
     </row>
     <row r="619">
       <c r="A619" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contatos_adicionais</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B619" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente</t>
+          <t xml:space="preserve">tipo_telhado</t>
         </is>
       </c>
       <c r="C619" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D619" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E619" s="2"/>
-      <c r="F619" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ceramico | metalico | laje | fibrocimento</t>
+        </is>
+      </c>
+      <c r="F619" s="2"/>
       <c r="G619" s="2"/>
     </row>
     <row r="620">
@@ -17532,12 +17532,12 @@
       </c>
       <c r="B620" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">nome</t>
+          <t xml:space="preserve">cliente</t>
         </is>
       </c>
       <c r="C620" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D620" t="inlineStr" s="2">
@@ -17546,7 +17546,11 @@
         </is>
       </c>
       <c r="E620" s="2"/>
-      <c r="F620" s="2"/>
+      <c r="F620" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G620" s="2"/>
     </row>
     <row r="621">
@@ -17557,7 +17561,7 @@
       </c>
       <c r="B621" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cargo</t>
+          <t xml:space="preserve">nome</t>
         </is>
       </c>
       <c r="C621" t="inlineStr" s="2">
@@ -17567,7 +17571,7 @@
       </c>
       <c r="D621" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E621" s="2"/>
@@ -17582,7 +17586,7 @@
       </c>
       <c r="B622" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">telefone</t>
+          <t xml:space="preserve">cargo</t>
         </is>
       </c>
       <c r="C622" t="inlineStr" s="2">
@@ -17607,7 +17611,7 @@
       </c>
       <c r="B623" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">email</t>
+          <t xml:space="preserve">telefone</t>
         </is>
       </c>
       <c r="C623" t="inlineStr" s="2">
@@ -17632,12 +17636,12 @@
       </c>
       <c r="B624" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">email</t>
         </is>
       </c>
       <c r="C624" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D624" t="inlineStr" s="2">
@@ -17647,11 +17651,7 @@
       </c>
       <c r="E624" s="2"/>
       <c r="F624" s="2"/>
-      <c r="G624" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G624" s="2"/>
     </row>
     <row r="625">
       <c r="A625" t="inlineStr" s="2">
@@ -17661,7 +17661,7 @@
       </c>
       <c r="B625" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C625" t="inlineStr" s="2">
@@ -17678,34 +17678,38 @@
       <c r="F625" s="2"/>
       <c r="G625" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="626">
       <c r="A626" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">instalacoes_galeria</t>
+          <t xml:space="preserve">contatos_adicionais</t>
         </is>
       </c>
       <c r="B626" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C626" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D626" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E626" s="2"/>
       <c r="F626" s="2"/>
-      <c r="G626" s="2"/>
+      <c r="G626" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="627">
       <c r="A627" t="inlineStr" s="2">
@@ -17715,7 +17719,7 @@
       </c>
       <c r="B627" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cidade</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C627" t="inlineStr" s="2">
@@ -17725,7 +17729,7 @@
       </c>
       <c r="D627" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E627" s="2"/>
@@ -17740,12 +17744,12 @@
       </c>
       <c r="B628" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">potencia_kwp</t>
+          <t xml:space="preserve">cidade</t>
         </is>
       </c>
       <c r="C628" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D628" t="inlineStr" s="2">
@@ -17765,12 +17769,12 @@
       </c>
       <c r="B629" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">foto</t>
+          <t xml:space="preserve">potencia_kwp</t>
         </is>
       </c>
       <c r="C629" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">file</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D629" t="inlineStr" s="2">
@@ -17780,11 +17784,7 @@
       </c>
       <c r="E629" s="2"/>
       <c r="F629" s="2"/>
-      <c r="G629" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
-        </is>
-      </c>
+      <c r="G629" s="2"/>
     </row>
     <row r="630">
       <c r="A630" t="inlineStr" s="2">
@@ -17794,12 +17794,12 @@
       </c>
       <c r="B630" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">foto_url</t>
+          <t xml:space="preserve">foto</t>
         </is>
       </c>
       <c r="C630" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="D630" t="inlineStr" s="2">
@@ -17809,7 +17809,11 @@
       </c>
       <c r="E630" s="2"/>
       <c r="F630" s="2"/>
-      <c r="G630" s="2"/>
+      <c r="G630" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
+        </is>
+      </c>
     </row>
     <row r="631">
       <c r="A631" t="inlineStr" s="2">
@@ -17819,12 +17823,12 @@
       </c>
       <c r="B631" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ordem</t>
+          <t xml:space="preserve">foto_url</t>
         </is>
       </c>
       <c r="C631" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D631" t="inlineStr" s="2">
@@ -17844,12 +17848,12 @@
       </c>
       <c r="B632" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">destaque</t>
+          <t xml:space="preserve">ordem</t>
         </is>
       </c>
       <c r="C632" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D632" t="inlineStr" s="2">
@@ -17857,11 +17861,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E632" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E632" s="2"/>
       <c r="F632" s="2"/>
       <c r="G632" s="2"/>
     </row>
@@ -17873,12 +17873,12 @@
       </c>
       <c r="B633" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">destaque</t>
         </is>
       </c>
       <c r="C633" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D633" t="inlineStr" s="2">
@@ -17886,13 +17886,13 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E633" s="2"/>
+      <c r="E633" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F633" s="2"/>
-      <c r="G633" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G633" s="2"/>
     </row>
     <row r="634">
       <c r="A634" t="inlineStr" s="2">
@@ -17902,7 +17902,7 @@
       </c>
       <c r="B634" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C634" t="inlineStr" s="2">
@@ -17919,34 +17919,38 @@
       <c r="F634" s="2"/>
       <c r="G634" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="635">
       <c r="A635" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">projecao_tarifaria</t>
+          <t xml:space="preserve">instalacoes_galeria</t>
         </is>
       </c>
       <c r="B635" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ano</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C635" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D635" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E635" s="2"/>
       <c r="F635" s="2"/>
-      <c r="G635" s="2"/>
+      <c r="G635" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="636">
       <c r="A636" t="inlineStr" s="2">
@@ -17956,12 +17960,12 @@
       </c>
       <c r="B636" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_cliente</t>
+          <t xml:space="preserve">ano</t>
         </is>
       </c>
       <c r="C636" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D636" t="inlineStr" s="2">
@@ -17969,11 +17973,7 @@
           <t xml:space="preserve">Sim</t>
         </is>
       </c>
-      <c r="E636" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">residencial | comercial</t>
-        </is>
-      </c>
+      <c r="E636" s="2"/>
       <c r="F636" s="2"/>
       <c r="G636" s="2"/>
     </row>
@@ -17985,20 +17985,24 @@
       </c>
       <c r="B637" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tarifa_kwh</t>
+          <t xml:space="preserve">tipo_cliente</t>
         </is>
       </c>
       <c r="C637" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D637" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E637" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">residencial | comercial</t>
+        </is>
+      </c>
       <c r="F637" s="2"/>
       <c r="G637" s="2"/>
     </row>
@@ -18010,7 +18014,7 @@
       </c>
       <c r="B638" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fio_b_kwh</t>
+          <t xml:space="preserve">tarifa_kwh</t>
         </is>
       </c>
       <c r="C638" t="inlineStr" s="2">
@@ -18035,7 +18039,7 @@
       </c>
       <c r="B639" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fs</t>
+          <t xml:space="preserve">fio_b_kwh</t>
         </is>
       </c>
       <c r="C639" t="inlineStr" s="2">
@@ -18060,7 +18064,7 @@
       </c>
       <c r="B640" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gd_eco_liquida</t>
+          <t xml:space="preserve">fs</t>
         </is>
       </c>
       <c r="C640" t="inlineStr" s="2">
@@ -18085,7 +18089,7 @@
       </c>
       <c r="B641" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">economia_acumulada</t>
+          <t xml:space="preserve">gd_eco_liquida</t>
         </is>
       </c>
       <c r="C641" t="inlineStr" s="2">
@@ -18110,7 +18114,7 @@
       </c>
       <c r="B642" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gasto_acumulado</t>
+          <t xml:space="preserve">economia_acumulada</t>
         </is>
       </c>
       <c r="C642" t="inlineStr" s="2">
@@ -18135,12 +18139,12 @@
       </c>
       <c r="B643" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">gasto_acumulado</t>
         </is>
       </c>
       <c r="C643" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D643" t="inlineStr" s="2">
@@ -18150,11 +18154,7 @@
       </c>
       <c r="E643" s="2"/>
       <c r="F643" s="2"/>
-      <c r="G643" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G643" s="2"/>
     </row>
     <row r="644">
       <c r="A644" t="inlineStr" s="2">
@@ -18164,7 +18164,7 @@
       </c>
       <c r="B644" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C644" t="inlineStr" s="2">
@@ -18181,38 +18181,38 @@
       <c r="F644" s="2"/>
       <c r="G644" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="645">
       <c r="A645" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">equipamentos</t>
+          <t xml:space="preserve">projecao_tarifaria</t>
         </is>
       </c>
       <c r="B645" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C645" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D645" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E645" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">inversor | modulo_fv</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E645" s="2"/>
       <c r="F645" s="2"/>
-      <c r="G645" s="2"/>
+      <c r="G645" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="646">
       <c r="A646" t="inlineStr" s="2">
@@ -18222,12 +18222,12 @@
       </c>
       <c r="B646" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">marca</t>
+          <t xml:space="preserve">tipo</t>
         </is>
       </c>
       <c r="C646" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D646" t="inlineStr" s="2">
@@ -18235,7 +18235,11 @@
           <t xml:space="preserve">Sim</t>
         </is>
       </c>
-      <c r="E646" s="2"/>
+      <c r="E646" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">inversor | modulo_fv</t>
+        </is>
+      </c>
       <c r="F646" s="2"/>
       <c r="G646" s="2"/>
     </row>
@@ -18247,7 +18251,7 @@
       </c>
       <c r="B647" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">modelo</t>
+          <t xml:space="preserve">marca</t>
         </is>
       </c>
       <c r="C647" t="inlineStr" s="2">
@@ -18272,12 +18276,12 @@
       </c>
       <c r="B648" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">potencia_w</t>
+          <t xml:space="preserve">modelo</t>
         </is>
       </c>
       <c r="C648" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D648" t="inlineStr" s="2">
@@ -18297,17 +18301,17 @@
       </c>
       <c r="B649" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">descricao_padrao</t>
+          <t xml:space="preserve">potencia_w</t>
         </is>
       </c>
       <c r="C649" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D649" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E649" s="2"/>
@@ -18322,12 +18326,12 @@
       </c>
       <c r="B650" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">garantia_anos</t>
+          <t xml:space="preserve">descricao_padrao</t>
         </is>
       </c>
       <c r="C650" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D650" t="inlineStr" s="2">
@@ -18347,12 +18351,12 @@
       </c>
       <c r="B651" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">foto</t>
+          <t xml:space="preserve">garantia_anos</t>
         </is>
       </c>
       <c r="C651" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">file</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D651" t="inlineStr" s="2">
@@ -18362,11 +18366,7 @@
       </c>
       <c r="E651" s="2"/>
       <c r="F651" s="2"/>
-      <c r="G651" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
-        </is>
-      </c>
+      <c r="G651" s="2"/>
     </row>
     <row r="652">
       <c r="A652" t="inlineStr" s="2">
@@ -18376,12 +18376,12 @@
       </c>
       <c r="B652" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">foto</t>
         </is>
       </c>
       <c r="C652" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="D652" t="inlineStr" s="2">
@@ -18393,7 +18393,7 @@
       <c r="F652" s="2"/>
       <c r="G652" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
+          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
         </is>
       </c>
     </row>
@@ -18405,7 +18405,7 @@
       </c>
       <c r="B653" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C653" t="inlineStr" s="2">
@@ -18422,7 +18422,7 @@
       <c r="F653" s="2"/>
       <c r="G653" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
@@ -18434,12 +18434,12 @@
       </c>
       <c r="B654" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">datasheet_pdf</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C654" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">file</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D654" t="inlineStr" s="2">
@@ -18451,34 +18451,38 @@
       <c r="F654" s="2"/>
       <c r="G654" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
         </is>
       </c>
     </row>
     <row r="655">
       <c r="A655" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">parametros_tarifarios</t>
+          <t xml:space="preserve">equipamentos</t>
         </is>
       </c>
       <c r="B655" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ano</t>
+          <t xml:space="preserve">datasheet_pdf</t>
         </is>
       </c>
       <c r="C655" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="D655" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E655" s="2"/>
       <c r="F655" s="2"/>
-      <c r="G655" s="2"/>
+      <c r="G655" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
+        </is>
+      </c>
     </row>
     <row r="656">
       <c r="A656" t="inlineStr" s="2">
@@ -18488,12 +18492,12 @@
       </c>
       <c r="B656" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">classe</t>
+          <t xml:space="preserve">ano</t>
         </is>
       </c>
       <c r="C656" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D656" t="inlineStr" s="2">
@@ -18501,11 +18505,7 @@
           <t xml:space="preserve">Sim</t>
         </is>
       </c>
-      <c r="E656" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">residencial | comercial</t>
-        </is>
-      </c>
+      <c r="E656" s="2"/>
       <c r="F656" s="2"/>
       <c r="G656" s="2"/>
     </row>
@@ -18517,20 +18517,24 @@
       </c>
       <c r="B657" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tarifa</t>
+          <t xml:space="preserve">classe</t>
         </is>
       </c>
       <c r="C657" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D657" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E657" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">residencial | comercial</t>
+        </is>
+      </c>
       <c r="F657" s="2"/>
       <c r="G657" s="2"/>
     </row>
@@ -18542,7 +18546,7 @@
       </c>
       <c r="B658" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fio_b</t>
+          <t xml:space="preserve">tarifa</t>
         </is>
       </c>
       <c r="C658" t="inlineStr" s="2">
@@ -18567,7 +18571,7 @@
       </c>
       <c r="B659" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fs</t>
+          <t xml:space="preserve">fio_b</t>
         </is>
       </c>
       <c r="C659" t="inlineStr" s="2">
@@ -18592,7 +18596,7 @@
       </c>
       <c r="B660" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gd_eco_liquida</t>
+          <t xml:space="preserve">fs</t>
         </is>
       </c>
       <c r="C660" t="inlineStr" s="2">
@@ -18617,12 +18621,12 @@
       </c>
       <c r="B661" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">gd_eco_liquida</t>
         </is>
       </c>
       <c r="C661" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D661" t="inlineStr" s="2">
@@ -18632,11 +18636,7 @@
       </c>
       <c r="E661" s="2"/>
       <c r="F661" s="2"/>
-      <c r="G661" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G661" s="2"/>
     </row>
     <row r="662">
       <c r="A662" t="inlineStr" s="2">
@@ -18646,7 +18646,7 @@
       </c>
       <c r="B662" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C662" t="inlineStr" s="2">
@@ -18663,34 +18663,38 @@
       <c r="F662" s="2"/>
       <c r="G662" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="663">
       <c r="A663" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">parametros_tarifarios</t>
         </is>
       </c>
       <c r="B663" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">nome</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C663" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D663" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E663" s="2"/>
       <c r="F663" s="2"/>
-      <c r="G663" s="2"/>
+      <c r="G663" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="664">
       <c r="A664" t="inlineStr" s="2">
@@ -18700,12 +18704,12 @@
       </c>
       <c r="B664" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gatilho</t>
+          <t xml:space="preserve">nome</t>
         </is>
       </c>
       <c r="C664" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D664" t="inlineStr" s="2">
@@ -18713,11 +18717,7 @@
           <t xml:space="preserve">Sim</t>
         </is>
       </c>
-      <c r="E664" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">status_mudou | instalacao_concluida | atividade_concluida | data_especifica | dias_apos_evento</t>
-        </is>
-      </c>
+      <c r="E664" s="2"/>
       <c r="F664" s="2"/>
       <c r="G664" s="2"/>
     </row>
@@ -18729,26 +18729,26 @@
       </c>
       <c r="B665" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">configuracao_gatilho</t>
+          <t xml:space="preserve">gatilho</t>
         </is>
       </c>
       <c r="C665" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D665" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E665" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">status_mudou | instalacao_concluida | atividade_concluida | data_especifica | dias_apos_evento</t>
+        </is>
+      </c>
       <c r="F665" s="2"/>
-      <c r="G665" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="G665" s="2"/>
     </row>
     <row r="666">
       <c r="A666" t="inlineStr" s="2">
@@ -18758,26 +18758,26 @@
       </c>
       <c r="B666" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">acao</t>
+          <t xml:space="preserve">configuracao_gatilho</t>
         </is>
       </c>
       <c r="C666" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D666" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E666" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">criar_atividade | enviar_whatsapp | enviar_email | mudar_status</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E666" s="2"/>
       <c r="F666" s="2"/>
-      <c r="G666" s="2"/>
+      <c r="G666" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Estrutura JSON livre</t>
+        </is>
+      </c>
     </row>
     <row r="667">
       <c r="A667" t="inlineStr" s="2">
@@ -18787,26 +18787,26 @@
       </c>
       <c r="B667" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">configuracao_acao</t>
+          <t xml:space="preserve">acao</t>
         </is>
       </c>
       <c r="C667" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D667" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E667" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">criar_atividade | enviar_whatsapp | enviar_email | mudar_status</t>
+        </is>
+      </c>
       <c r="F667" s="2"/>
-      <c r="G667" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="G667" s="2"/>
     </row>
     <row r="668">
       <c r="A668" t="inlineStr" s="2">
@@ -18816,26 +18816,26 @@
       </c>
       <c r="B668" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">destino</t>
+          <t xml:space="preserve">configuracao_acao</t>
         </is>
       </c>
       <c r="C668" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D668" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E668" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">cliente_evento | responsavel_empresa | cliente_especifico</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E668" s="2"/>
       <c r="F668" s="2"/>
-      <c r="G668" s="2"/>
+      <c r="G668" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Estrutura JSON livre</t>
+        </is>
+      </c>
     </row>
     <row r="669">
       <c r="A669" t="inlineStr" s="2">
@@ -18845,25 +18845,25 @@
       </c>
       <c r="B669" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_especifico_id</t>
+          <t xml:space="preserve">destino</t>
         </is>
       </c>
       <c r="C669" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D669" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E669" s="2"/>
-      <c r="F669" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">cliente_evento | responsavel_empresa | cliente_especifico</t>
+        </is>
+      </c>
+      <c r="F669" s="2"/>
       <c r="G669" s="2"/>
     </row>
     <row r="670">
@@ -18874,12 +18874,12 @@
       </c>
       <c r="B670" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ativa</t>
+          <t xml:space="preserve">cliente_especifico_id</t>
         </is>
       </c>
       <c r="C670" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D670" t="inlineStr" s="2">
@@ -18887,12 +18887,12 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E670" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
-      <c r="F670" s="2"/>
+      <c r="E670" s="2"/>
+      <c r="F670" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G670" s="2"/>
     </row>
     <row r="671">
@@ -18903,12 +18903,12 @@
       </c>
       <c r="B671" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">ativa</t>
         </is>
       </c>
       <c r="C671" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D671" t="inlineStr" s="2">
@@ -18916,13 +18916,13 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E671" s="2"/>
+      <c r="E671" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F671" s="2"/>
-      <c r="G671" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G671" s="2"/>
     </row>
     <row r="672">
       <c r="A672" t="inlineStr" s="2">
@@ -18932,7 +18932,7 @@
       </c>
       <c r="B672" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C672" t="inlineStr" s="2">
@@ -18949,38 +18949,38 @@
       <c r="F672" s="2"/>
       <c r="G672" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="673">
       <c r="A673" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes_execucoes</t>
+          <t xml:space="preserve">automacoes</t>
         </is>
       </c>
       <c r="B673" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacao</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C673" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D673" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E673" s="2"/>
-      <c r="F673" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">automacoes</t>
-        </is>
-      </c>
-      <c r="G673" s="2"/>
+      <c r="F673" s="2"/>
+      <c r="G673" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="674">
       <c r="A674" t="inlineStr" s="2">
@@ -18990,12 +18990,12 @@
       </c>
       <c r="B674" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_execucao</t>
+          <t xml:space="preserve">automacao</t>
         </is>
       </c>
       <c r="C674" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D674" t="inlineStr" s="2">
@@ -19004,7 +19004,11 @@
         </is>
       </c>
       <c r="E674" s="2"/>
-      <c r="F674" s="2"/>
+      <c r="F674" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">automacoes</t>
+        </is>
+      </c>
       <c r="G674" s="2"/>
     </row>
     <row r="675">
@@ -19015,24 +19019,20 @@
       </c>
       <c r="B675" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">sucesso</t>
+          <t xml:space="preserve">data_execucao</t>
         </is>
       </c>
       <c r="C675" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D675" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E675" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E675" s="2"/>
       <c r="F675" s="2"/>
       <c r="G675" s="2"/>
     </row>
@@ -19044,12 +19044,12 @@
       </c>
       <c r="B676" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mensagem</t>
+          <t xml:space="preserve">sucesso</t>
         </is>
       </c>
       <c r="C676" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D676" t="inlineStr" s="2">
@@ -19057,7 +19057,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E676" s="2"/>
+      <c r="E676" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F676" s="2"/>
       <c r="G676" s="2"/>
     </row>
@@ -19069,7 +19073,7 @@
       </c>
       <c r="B677" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">referencia_registro</t>
+          <t xml:space="preserve">mensagem</t>
         </is>
       </c>
       <c r="C677" t="inlineStr" s="2">
@@ -19094,12 +19098,12 @@
       </c>
       <c r="B678" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente</t>
+          <t xml:space="preserve">referencia_registro</t>
         </is>
       </c>
       <c r="C678" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D678" t="inlineStr" s="2">
@@ -19108,11 +19112,7 @@
         </is>
       </c>
       <c r="E678" s="2"/>
-      <c r="F678" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+      <c r="F678" s="2"/>
       <c r="G678" s="2"/>
     </row>
     <row r="679">
@@ -19123,12 +19123,12 @@
       </c>
       <c r="B679" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">dados_execucao</t>
+          <t xml:space="preserve">cliente</t>
         </is>
       </c>
       <c r="C679" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D679" t="inlineStr" s="2">
@@ -19137,12 +19137,12 @@
         </is>
       </c>
       <c r="E679" s="2"/>
-      <c r="F679" s="2"/>
-      <c r="G679" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="F679" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
+      <c r="G679" s="2"/>
     </row>
     <row r="680">
       <c r="A680" t="inlineStr" s="2">
@@ -19152,12 +19152,12 @@
       </c>
       <c r="B680" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">dados_execucao</t>
         </is>
       </c>
       <c r="C680" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D680" t="inlineStr" s="2">
@@ -19169,7 +19169,7 @@
       <c r="F680" s="2"/>
       <c r="G680" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
+          <t xml:space="preserve">Estrutura JSON livre</t>
         </is>
       </c>
     </row>
@@ -19181,7 +19181,7 @@
       </c>
       <c r="B681" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C681" t="inlineStr" s="2">
@@ -19198,38 +19198,38 @@
       <c r="F681" s="2"/>
       <c r="G681" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="682">
       <c r="A682" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">automacoes_execucoes</t>
         </is>
       </c>
       <c r="B682" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C682" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D682" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E682" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">atividade_atrasada | lembrete | sistema</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E682" s="2"/>
       <c r="F682" s="2"/>
-      <c r="G682" s="2"/>
+      <c r="G682" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="683">
       <c r="A683" t="inlineStr" s="2">
@@ -19239,12 +19239,12 @@
       </c>
       <c r="B683" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">tipo</t>
         </is>
       </c>
       <c r="C683" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D683" t="inlineStr" s="2">
@@ -19252,7 +19252,11 @@
           <t xml:space="preserve">Sim</t>
         </is>
       </c>
-      <c r="E683" s="2"/>
+      <c r="E683" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">atividade_atrasada | lembrete | sistema</t>
+        </is>
+      </c>
       <c r="F683" s="2"/>
       <c r="G683" s="2"/>
     </row>
@@ -19264,7 +19268,7 @@
       </c>
       <c r="B684" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mensagem</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C684" t="inlineStr" s="2">
@@ -19274,7 +19278,7 @@
       </c>
       <c r="D684" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E684" s="2"/>
@@ -19289,12 +19293,12 @@
       </c>
       <c r="B685" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">atividade_id</t>
+          <t xml:space="preserve">mensagem</t>
         </is>
       </c>
       <c r="C685" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D685" t="inlineStr" s="2">
@@ -19303,11 +19307,7 @@
         </is>
       </c>
       <c r="E685" s="2"/>
-      <c r="F685" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">atividades</t>
-        </is>
-      </c>
+      <c r="F685" s="2"/>
       <c r="G685" s="2"/>
     </row>
     <row r="686">
@@ -19318,7 +19318,7 @@
       </c>
       <c r="B686" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_id</t>
+          <t xml:space="preserve">atividade_id</t>
         </is>
       </c>
       <c r="C686" t="inlineStr" s="2">
@@ -19334,7 +19334,7 @@
       <c r="E686" s="2"/>
       <c r="F686" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">clientes</t>
+          <t xml:space="preserve">atividades</t>
         </is>
       </c>
       <c r="G686" s="2"/>
@@ -19347,12 +19347,12 @@
       </c>
       <c r="B687" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_nome</t>
+          <t xml:space="preserve">cliente_id</t>
         </is>
       </c>
       <c r="C687" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D687" t="inlineStr" s="2">
@@ -19361,7 +19361,11 @@
         </is>
       </c>
       <c r="E687" s="2"/>
-      <c r="F687" s="2"/>
+      <c r="F687" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G687" s="2"/>
     </row>
     <row r="688">
@@ -19372,12 +19376,12 @@
       </c>
       <c r="B688" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_prevista</t>
+          <t xml:space="preserve">cliente_nome</t>
         </is>
       </c>
       <c r="C688" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D688" t="inlineStr" s="2">
@@ -19397,12 +19401,12 @@
       </c>
       <c r="B689" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">dias_atraso</t>
+          <t xml:space="preserve">data_prevista</t>
         </is>
       </c>
       <c r="C689" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D689" t="inlineStr" s="2">
@@ -19422,12 +19426,12 @@
       </c>
       <c r="B690" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">lida</t>
+          <t xml:space="preserve">dias_atraso</t>
         </is>
       </c>
       <c r="C690" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D690" t="inlineStr" s="2">
@@ -19435,11 +19439,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E690" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E690" s="2"/>
       <c r="F690" s="2"/>
       <c r="G690" s="2"/>
     </row>
@@ -19451,12 +19451,12 @@
       </c>
       <c r="B691" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">lida_em</t>
+          <t xml:space="preserve">lida</t>
         </is>
       </c>
       <c r="C691" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D691" t="inlineStr" s="2">
@@ -19464,7 +19464,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E691" s="2"/>
+      <c r="E691" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F691" s="2"/>
       <c r="G691" s="2"/>
     </row>
@@ -19476,24 +19480,20 @@
       </c>
       <c r="B692" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">lida_em</t>
         </is>
       </c>
       <c r="C692" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D692" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E692" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">ativa | resolvida | arquivada</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E692" s="2"/>
       <c r="F692" s="2"/>
       <c r="G692" s="2"/>
     </row>
@@ -19505,20 +19505,24 @@
       </c>
       <c r="B693" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">resolvida_em</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="C693" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D693" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E693" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativa | resolvida | arquivada</t>
+        </is>
+      </c>
       <c r="F693" s="2"/>
       <c r="G693" s="2"/>
     </row>
@@ -19530,12 +19534,12 @@
       </c>
       <c r="B694" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">resolvida_em</t>
         </is>
       </c>
       <c r="C694" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D694" t="inlineStr" s="2">
@@ -19545,11 +19549,7 @@
       </c>
       <c r="E694" s="2"/>
       <c r="F694" s="2"/>
-      <c r="G694" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G694" s="2"/>
     </row>
     <row r="695">
       <c r="A695" t="inlineStr" s="2">
@@ -19559,7 +19559,7 @@
       </c>
       <c r="B695" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C695" t="inlineStr" s="2">
@@ -19576,38 +19576,38 @@
       <c r="F695" s="2"/>
       <c r="G695" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="696">
       <c r="A696" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">notificacoes_internas</t>
         </is>
       </c>
       <c r="B696" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_id</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C696" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D696" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E696" s="2"/>
-      <c r="F696" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
-      <c r="G696" s="2"/>
+      <c r="F696" s="2"/>
+      <c r="G696" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="697">
       <c r="A697" t="inlineStr" s="2">
@@ -19617,25 +19617,25 @@
       </c>
       <c r="B697" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_negocio</t>
+          <t xml:space="preserve">cliente_id</t>
         </is>
       </c>
       <c r="C697" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D697" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E697" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">venda usina | bateria | expansão | renovação | serviço | venda bateria</t>
-        </is>
-      </c>
-      <c r="F697" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E697" s="2"/>
+      <c r="F697" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G697" s="2"/>
     </row>
     <row r="698">
@@ -19646,12 +19646,12 @@
       </c>
       <c r="B698" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">valor_estimado</t>
+          <t xml:space="preserve">tipo_negocio</t>
         </is>
       </c>
       <c r="C698" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D698" t="inlineStr" s="2">
@@ -19659,7 +19659,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E698" s="2"/>
+      <c r="E698" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">venda usina | bateria | expansão | renovação | serviço | venda bateria</t>
+        </is>
+      </c>
       <c r="F698" s="2"/>
       <c r="G698" s="2"/>
     </row>
@@ -19671,7 +19675,7 @@
       </c>
       <c r="B699" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">valor_final</t>
+          <t xml:space="preserve">valor_estimado</t>
         </is>
       </c>
       <c r="C699" t="inlineStr" s="2">
@@ -19696,12 +19700,12 @@
       </c>
       <c r="B700" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">etapa_funil</t>
+          <t xml:space="preserve">valor_final</t>
         </is>
       </c>
       <c r="C700" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D700" t="inlineStr" s="2">
@@ -19709,11 +19713,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E700" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">novo lead | qualificado | proposta enviada | negociação | contrato assinado</t>
-        </is>
-      </c>
+      <c r="E700" s="2"/>
       <c r="F700" s="2"/>
       <c r="G700" s="2"/>
     </row>
@@ -19725,12 +19725,12 @@
       </c>
       <c r="B701" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">probabilidade</t>
+          <t xml:space="preserve">etapa_funil</t>
         </is>
       </c>
       <c r="C701" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D701" t="inlineStr" s="2">
@@ -19738,7 +19738,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E701" s="2"/>
+      <c r="E701" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">novo lead | qualificado | proposta enviada | negociação | contrato assinado</t>
+        </is>
+      </c>
       <c r="F701" s="2"/>
       <c r="G701" s="2"/>
     </row>
@@ -19750,12 +19754,12 @@
       </c>
       <c r="B702" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_previsao_fechamento</t>
+          <t xml:space="preserve">probabilidade</t>
         </is>
       </c>
       <c r="C702" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D702" t="inlineStr" s="2">
@@ -19775,7 +19779,7 @@
       </c>
       <c r="B703" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_fechamento</t>
+          <t xml:space="preserve">data_previsao_fechamento</t>
         </is>
       </c>
       <c r="C703" t="inlineStr" s="2">
@@ -19800,12 +19804,12 @@
       </c>
       <c r="B704" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">data_fechamento</t>
         </is>
       </c>
       <c r="C704" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D704" t="inlineStr" s="2">
@@ -19813,11 +19817,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E704" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">em andamento | ganho | perdido</t>
-        </is>
-      </c>
+      <c r="E704" s="2"/>
       <c r="F704" s="2"/>
       <c r="G704" s="2"/>
     </row>
@@ -19829,12 +19829,12 @@
       </c>
       <c r="B705" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">motivo_perda</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="C705" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D705" t="inlineStr" s="2">
@@ -19842,7 +19842,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E705" s="2"/>
+      <c r="E705" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">em andamento | ganho | perdido</t>
+        </is>
+      </c>
       <c r="F705" s="2"/>
       <c r="G705" s="2"/>
     </row>
@@ -19854,12 +19858,12 @@
       </c>
       <c r="B706" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">reabertura</t>
+          <t xml:space="preserve">motivo_perda</t>
         </is>
       </c>
       <c r="C706" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D706" t="inlineStr" s="2">
@@ -19867,11 +19871,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E706" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E706" s="2"/>
       <c r="F706" s="2"/>
       <c r="G706" s="2"/>
     </row>
@@ -19883,12 +19883,12 @@
       </c>
       <c r="B707" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">motivo_reabertura</t>
+          <t xml:space="preserve">reabertura</t>
         </is>
       </c>
       <c r="C707" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D707" t="inlineStr" s="2">
@@ -19896,7 +19896,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E707" s="2"/>
+      <c r="E707" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F707" s="2"/>
       <c r="G707" s="2"/>
     </row>
@@ -19908,7 +19912,7 @@
       </c>
       <c r="B708" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">condicao_pagamento</t>
+          <t xml:space="preserve">motivo_reabertura</t>
         </is>
       </c>
       <c r="C708" t="inlineStr" s="2">
@@ -19933,12 +19937,12 @@
       </c>
       <c r="B709" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">condicao_pagamento</t>
         </is>
       </c>
       <c r="C709" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D709" t="inlineStr" s="2">
@@ -19948,11 +19952,7 @@
       </c>
       <c r="E709" s="2"/>
       <c r="F709" s="2"/>
-      <c r="G709" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G709" s="2"/>
     </row>
     <row r="710">
       <c r="A710" t="inlineStr" s="2">
@@ -19962,7 +19962,7 @@
       </c>
       <c r="B710" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C710" t="inlineStr" s="2">
@@ -19979,7 +19979,7 @@
       <c r="F710" s="2"/>
       <c r="G710" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
@@ -19991,12 +19991,12 @@
       </c>
       <c r="B711" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_venda</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C711" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D711" t="inlineStr" s="2">
@@ -20004,13 +20004,13 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E711" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Energia Solar | O&amp;M (Operação e Manutenção) | Baterias | Carregadores Veículos Elétricos</t>
-        </is>
-      </c>
+      <c r="E711" s="2"/>
       <c r="F711" s="2"/>
-      <c r="G711" s="2"/>
+      <c r="G711" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="712">
       <c r="A712" t="inlineStr" s="2">
@@ -20020,12 +20020,12 @@
       </c>
       <c r="B712" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">tipo_venda</t>
         </is>
       </c>
       <c r="C712" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D712" t="inlineStr" s="2">
@@ -20033,7 +20033,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E712" s="2"/>
+      <c r="E712" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Energia Solar | O&amp;M (Operação e Manutenção) | Baterias | Carregadores Veículos Elétricos</t>
+        </is>
+      </c>
       <c r="F712" s="2"/>
       <c r="G712" s="2"/>
     </row>
@@ -20045,12 +20049,12 @@
       </c>
       <c r="B713" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">valor</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C713" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D713" t="inlineStr" s="2">
@@ -20070,12 +20074,12 @@
       </c>
       <c r="B714" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">consultor_responsavel</t>
+          <t xml:space="preserve">valor</t>
         </is>
       </c>
       <c r="C714" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D714" t="inlineStr" s="2">
@@ -20084,11 +20088,7 @@
         </is>
       </c>
       <c r="E714" s="2"/>
-      <c r="F714" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">users</t>
-        </is>
-      </c>
+      <c r="F714" s="2"/>
       <c r="G714" s="2"/>
     </row>
     <row r="715">
@@ -20099,26 +20099,55 @@
       </c>
       <c r="B715" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">consultor_responsavel</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">relation</t>
+        </is>
+      </c>
+      <c r="D715" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E715" s="2"/>
+      <c r="F715" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">users</t>
+        </is>
+      </c>
+      <c r="G715" s="2"/>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">recorrencia_mensal</t>
         </is>
       </c>
-      <c r="C715" t="inlineStr" s="2">
+      <c r="C716" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">bool</t>
         </is>
       </c>
-      <c r="D715" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E715" t="inlineStr" s="2">
+      <c r="D716" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">true / false</t>
         </is>
       </c>
-      <c r="F715" s="2"/>
-      <c r="G715" s="2"/>
+      <c r="F716" s="2"/>
+      <c r="G716" s="2"/>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>

<commit_message>
feat: criar atividade administrativa Análise de Fatura com IA Gemini, relatório interativo e envio via WhatsApp
</commit_message>
<xml_diff>
--- a/public/schema-delfos-solar.xlsx
+++ b/public/schema-delfos-solar.xlsx
@@ -1216,22 +1216,50 @@
     <row r="41">
       <c r="A41" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TOTAL: 39 coleções</t>
+          <t xml:space="preserve">analises_fatura</t>
         </is>
       </c>
       <c r="B41" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Coleção de dados do sistema.</t>
+        </is>
+      </c>
+      <c r="C41" s="2">
+        <v>21</v>
+      </c>
+      <c r="D41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">base</t>
+        </is>
+      </c>
+      <c r="E41" s="2">
+        <v>1</v>
+      </c>
+      <c r="F41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Regras RLS configuradas (autenticado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TOTAL: 40 coleções</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Total geral de campos e relacionamentos no banco PocketBase Delfos Solar</t>
         </is>
       </c>
-      <c r="C41" s="2">
-        <v>747</v>
-      </c>
-      <c r="D41" s="2"/>
-      <c r="E41" s="2">
-        <v>47</v>
-      </c>
-      <c r="F41" s="2"/>
+      <c r="C42" s="2">
+        <v>768</v>
+      </c>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2">
+        <v>48</v>
+      </c>
+      <c r="F42" s="2"/>
     </row>
   </sheetData>
 </worksheet>
@@ -4429,7 +4457,7 @@
       </c>
       <c r="E122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contato_ligacao | reuniao_presencial | follow_up | instalacao | proposta | limpeza_manutencao | auto_leitura_rge | ligar_indicacao | configuracao_datalogger | garantia_equipamento | relatorio_solarview | contato_reativacao | anotacao | ligacao | reuniao | visita_tecnica | mudanca_estagio | anexo_g | troca_titularidade | transferencia_creditos | custom | gerar_procuracao | gerar_contrato | oferecer_limpeza_avulsa | solicitar_contas_rge | mensagem_enviada</t>
+          <t xml:space="preserve">contato_ligacao | reuniao_presencial | follow_up | instalacao | proposta | limpeza_manutencao | auto_leitura_rge | ligar_indicacao | configuracao_datalogger | garantia_equipamento | relatorio_solarview | contato_reativacao | anotacao | ligacao | reuniao | visita_tecnica | mudanca_estagio | anexo_g | troca_titularidade | transferencia_creditos | custom | gerar_procuracao | gerar_contrato | oferecer_limpeza_avulsa | solicitar_contas_rge | mensagem_enviada | analise_fatura</t>
         </is>
       </c>
       <c r="F122" s="2"/>
@@ -20960,6 +20988,555 @@
       </c>
       <c r="F748" s="2"/>
       <c r="G748" s="2"/>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">analises_fatura</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">token</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D749" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E749" s="2"/>
+      <c r="F749" s="2"/>
+      <c r="G749" s="2"/>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">analises_fatura</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">cliente_id</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">relation</t>
+        </is>
+      </c>
+      <c r="D750" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E750" s="2"/>
+      <c r="F750" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
+      <c r="G750" s="2"/>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">analises_fatura</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">cliente_nome</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D751" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E751" s="2"/>
+      <c r="F751" s="2"/>
+      <c r="G751" s="2"/>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">analises_fatura</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">uc</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E752" s="2"/>
+      <c r="F752" s="2"/>
+      <c r="G752" s="2"/>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">analises_fatura</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">competencia</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D753" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E753" s="2"/>
+      <c r="F753" s="2"/>
+      <c r="G753" s="2"/>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">analises_fatura</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">vencimento</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D754" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E754" s="2"/>
+      <c r="F754" s="2"/>
+      <c r="G754" s="2"/>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">analises_fatura</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">total_pagar</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E755" s="2"/>
+      <c r="F755" s="2"/>
+      <c r="G755" s="2"/>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">analises_fatura</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">consumo_kwh</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D756" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E756" s="2"/>
+      <c r="F756" s="2"/>
+      <c r="G756" s="2"/>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">analises_fatura</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">energia_injetada_kwh</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D757" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E757" s="2"/>
+      <c r="F757" s="2"/>
+      <c r="G757" s="2"/>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">analises_fatura</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">creditos_compensados_kwh</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D758" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E758" s="2"/>
+      <c r="F758" s="2"/>
+      <c r="G758" s="2"/>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">analises_fatura</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">saldo_energia_kwh</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D759" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E759" s="2"/>
+      <c r="F759" s="2"/>
+      <c r="G759" s="2"/>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">analises_fatura</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">saldo_expirar_kwh</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D760" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E760" s="2"/>
+      <c r="F760" s="2"/>
+      <c r="G760" s="2"/>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">analises_fatura</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">economia_estimada_rs</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D761" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E761" s="2"/>
+      <c r="F761" s="2"/>
+      <c r="G761" s="2"/>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">analises_fatura</t>
+        </is>
+      </c>
+      <c r="B762" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">papel_uc</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D762" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E762" s="2"/>
+      <c r="F762" s="2"/>
+      <c r="G762" s="2"/>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">analises_fatura</t>
+        </is>
+      </c>
+      <c r="B763" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">arquivos_nomes</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">json</t>
+        </is>
+      </c>
+      <c r="D763" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E763" s="2"/>
+      <c r="F763" s="2"/>
+      <c r="G763" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Estrutura JSON livre</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">analises_fatura</t>
+        </is>
+      </c>
+      <c r="B764" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">dados_completos</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">json</t>
+        </is>
+      </c>
+      <c r="D764" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E764" s="2"/>
+      <c r="F764" s="2"/>
+      <c r="G764" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Estrutura JSON livre</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">analises_fatura</t>
+        </is>
+      </c>
+      <c r="B765" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">atividade_id</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D765" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E765" s="2"/>
+      <c r="F765" s="2"/>
+      <c r="G765" s="2"/>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">analises_fatura</t>
+        </is>
+      </c>
+      <c r="B766" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">whatsapp_enviado</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">bool</t>
+        </is>
+      </c>
+      <c r="D766" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E766" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
+      <c r="F766" s="2"/>
+      <c r="G766" s="2"/>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">analises_fatura</t>
+        </is>
+      </c>
+      <c r="B767" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">whatsapp_enviado_em</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D767" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E767" s="2"/>
+      <c r="F767" s="2"/>
+      <c r="G767" s="2"/>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">analises_fatura</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">created</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D768" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E768" s="2"/>
+      <c r="F768" s="2"/>
+      <c r="G768" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">analises_fatura</t>
+        </is>
+      </c>
+      <c r="B769" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">updated</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D769" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E769" s="2"/>
+      <c r="F769" s="2"/>
+      <c r="G769" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
   </sheetData>
 </worksheet>
@@ -22512,6 +23089,38 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">analises_fatura</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">cliente_id</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Vínculo do registro ao cliente proprietário</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: funcionalidade completa de Base de Conhecimento e Assistente Delfos com Gemini
</commit_message>
<xml_diff>
--- a/public/schema-delfos-solar.xlsx
+++ b/public/schema-delfos-solar.xlsx
@@ -1244,22 +1244,78 @@
     <row r="42">
       <c r="A42" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TOTAL: 40 coleções</t>
+          <t xml:space="preserve">knowledge_categories</t>
         </is>
       </c>
       <c r="B42" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Coleção de dados do sistema.</t>
+        </is>
+      </c>
+      <c r="C42" s="2">
+        <v>6</v>
+      </c>
+      <c r="D42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">base</t>
+        </is>
+      </c>
+      <c r="E42" s="2">
+        <v>0</v>
+      </c>
+      <c r="F42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Regras RLS configuradas (autenticado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_articles</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Coleção de dados do sistema.</t>
+        </is>
+      </c>
+      <c r="C43" s="2">
+        <v>10</v>
+      </c>
+      <c r="D43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">base</t>
+        </is>
+      </c>
+      <c r="E43" s="2">
+        <v>2</v>
+      </c>
+      <c r="F43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Regras RLS configuradas (autenticado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TOTAL: 42 coleções</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Total geral de campos e relacionamentos no banco PocketBase Delfos Solar</t>
         </is>
       </c>
-      <c r="C42" s="2">
-        <v>768</v>
-      </c>
-      <c r="D42" s="2"/>
-      <c r="E42" s="2">
-        <v>48</v>
-      </c>
-      <c r="F42" s="2"/>
+      <c r="C44" s="2">
+        <v>784</v>
+      </c>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2">
+        <v>50</v>
+      </c>
+      <c r="F44" s="2"/>
     </row>
   </sheetData>
 </worksheet>
@@ -21538,6 +21594,434 @@
         </is>
       </c>
     </row>
+    <row r="770">
+      <c r="A770" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_categories</t>
+        </is>
+      </c>
+      <c r="B770" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">titulo</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D770" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E770" s="2"/>
+      <c r="F770" s="2"/>
+      <c r="G770" s="2"/>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_categories</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">descricao</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D771" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E771" s="2"/>
+      <c r="F771" s="2"/>
+      <c r="G771" s="2"/>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_categories</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">icone</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D772" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E772" s="2"/>
+      <c r="F772" s="2"/>
+      <c r="G772" s="2"/>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_categories</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ordem</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D773" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E773" s="2"/>
+      <c r="F773" s="2"/>
+      <c r="G773" s="2"/>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_categories</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">created</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D774" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E774" s="2"/>
+      <c r="F774" s="2"/>
+      <c r="G774" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_categories</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">updated</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D775" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E775" s="2"/>
+      <c r="F775" s="2"/>
+      <c r="G775" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_articles</t>
+        </is>
+      </c>
+      <c r="B776" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">categoria_id</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">relation</t>
+        </is>
+      </c>
+      <c r="D776" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E776" s="2"/>
+      <c r="F776" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_categories</t>
+        </is>
+      </c>
+      <c r="G776" s="2"/>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_articles</t>
+        </is>
+      </c>
+      <c r="B777" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">titulo</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D777" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E777" s="2"/>
+      <c r="F777" s="2"/>
+      <c r="G777" s="2"/>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_articles</t>
+        </is>
+      </c>
+      <c r="B778" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">conteudo</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D778" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E778" s="2"/>
+      <c r="F778" s="2"/>
+      <c r="G778" s="2"/>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_articles</t>
+        </is>
+      </c>
+      <c r="B779" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">texto_extraido</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D779" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E779" s="2"/>
+      <c r="F779" s="2"/>
+      <c r="G779" s="2"/>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_articles</t>
+        </is>
+      </c>
+      <c r="B780" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">anexos</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">file</t>
+        </is>
+      </c>
+      <c r="D780" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E780" s="2"/>
+      <c r="F780" s="2"/>
+      <c r="G780" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_articles</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">criado_por</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">relation</t>
+        </is>
+      </c>
+      <c r="D781" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E781" s="2"/>
+      <c r="F781" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">users</t>
+        </is>
+      </c>
+      <c r="G781" s="2"/>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_articles</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autor_nome</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D782" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E782" s="2"/>
+      <c r="F782" s="2"/>
+      <c r="G782" s="2"/>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_articles</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">tags</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D783" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E783" s="2"/>
+      <c r="F783" s="2"/>
+      <c r="G783" s="2"/>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_articles</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">created</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D784" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E784" s="2"/>
+      <c r="F784" s="2"/>
+      <c r="G784" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_articles</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">updated</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D785" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E785" s="2"/>
+      <c r="F785" s="2"/>
+      <c r="G785" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -23121,6 +23605,70 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_articles</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">categoria_id</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_categories</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Relaciona o registro de knowledge_articles com knowledge_categories</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_articles</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">criado_por</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">users</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Relaciona o registro de knowledge_articles com users</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
IMPLEMENTE de fato — a tentativa anterior terminou sem escrever nenhum …
</commit_message>
<xml_diff>
--- a/public/schema-delfos-solar.xlsx
+++ b/public/schema-delfos-solar.xlsx
@@ -1300,22 +1300,50 @@
     <row r="44">
       <c r="A44" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TOTAL: 42 coleções</t>
+          <t xml:space="preserve">contratos_usinas</t>
         </is>
       </c>
       <c r="B44" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Coleção de dados do sistema.</t>
+        </is>
+      </c>
+      <c r="C44" s="2">
+        <v>8</v>
+      </c>
+      <c r="D44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">base</t>
+        </is>
+      </c>
+      <c r="E44" s="2">
+        <v>2</v>
+      </c>
+      <c r="F44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Regras RLS configuradas (autenticado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TOTAL: 43 coleções</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Total geral de campos e relacionamentos no banco PocketBase Delfos Solar</t>
         </is>
       </c>
-      <c r="C44" s="2">
-        <v>790</v>
-      </c>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2">
-        <v>51</v>
-      </c>
-      <c r="F44" s="2"/>
+      <c r="C45" s="2">
+        <v>798</v>
+      </c>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2">
+        <v>53</v>
+      </c>
+      <c r="F45" s="2"/>
     </row>
   </sheetData>
 </worksheet>
@@ -22184,6 +22212,226 @@
         </is>
       </c>
     </row>
+    <row r="792">
+      <c r="A792" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contratos_usinas</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contrato_id</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">relation</t>
+        </is>
+      </c>
+      <c r="D792" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E792" s="2"/>
+      <c r="F792" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contratos_om</t>
+        </is>
+      </c>
+      <c r="G792" s="2"/>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contratos_usinas</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usina_id</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">relation</t>
+        </is>
+      </c>
+      <c r="D793" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E793" s="2"/>
+      <c r="F793" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usinas</t>
+        </is>
+      </c>
+      <c r="G793" s="2"/>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contratos_usinas</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativo</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">bool</t>
+        </is>
+      </c>
+      <c r="D794" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E794" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
+      <c r="F794" s="2"/>
+      <c r="G794" s="2"/>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contratos_usinas</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">data_vinculo</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">date</t>
+        </is>
+      </c>
+      <c r="D795" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E795" s="2"/>
+      <c r="F795" s="2"/>
+      <c r="G795" s="2"/>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contratos_usinas</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">data_desvinculo</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">date</t>
+        </is>
+      </c>
+      <c r="D796" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E796" s="2"/>
+      <c r="F796" s="2"/>
+      <c r="G796" s="2"/>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contratos_usinas</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">observacoes</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D797" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E797" s="2"/>
+      <c r="F797" s="2"/>
+      <c r="G797" s="2"/>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contratos_usinas</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">created</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D798" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E798" s="2"/>
+      <c r="F798" s="2"/>
+      <c r="G798" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contratos_usinas</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">updated</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D799" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E799" s="2"/>
+      <c r="F799" s="2"/>
+      <c r="G799" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -23863,6 +24111,70 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contratos_usinas</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contrato_id</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contratos_om</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Vínculo do serviço ou anomalia ao contrato de O&amp;M vigente</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contratos_usinas</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usina_id</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usinas</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Vínculo da atividade à usina fotovoltaica correspondente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: adicionar visão consolidada de contatos e campos aditivos de papel e WhatsApp
</commit_message>
<xml_diff>
--- a/public/schema-delfos-solar.xlsx
+++ b/public/schema-delfos-solar.xlsx
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="C32" s="2">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D32" t="inlineStr" s="2">
         <is>
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="C45" s="2">
-        <v>798</v>
+        <v>800</v>
       </c>
       <c r="D45" s="2"/>
       <c r="E45" s="2">
@@ -18800,42 +18800,46 @@
     <row r="665">
       <c r="A665" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">instalacoes_galeria</t>
+          <t xml:space="preserve">contatos_adicionais</t>
         </is>
       </c>
       <c r="B665" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">papel</t>
         </is>
       </c>
       <c r="C665" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D665" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E665" s="2"/>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">principal | financeiro | tecnico | responsavel | outro</t>
+        </is>
+      </c>
       <c r="F665" s="2"/>
       <c r="G665" s="2"/>
     </row>
     <row r="666">
       <c r="A666" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">instalacoes_galeria</t>
+          <t xml:space="preserve">contatos_adicionais</t>
         </is>
       </c>
       <c r="B666" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cidade</t>
+          <t xml:space="preserve">is_whatsapp</t>
         </is>
       </c>
       <c r="C666" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D666" t="inlineStr" s="2">
@@ -18843,7 +18847,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E666" s="2"/>
+      <c r="E666" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F666" s="2"/>
       <c r="G666" s="2"/>
     </row>
@@ -18855,17 +18863,17 @@
       </c>
       <c r="B667" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">potencia_kwp</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C667" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D667" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E667" s="2"/>
@@ -18880,12 +18888,12 @@
       </c>
       <c r="B668" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">foto</t>
+          <t xml:space="preserve">cidade</t>
         </is>
       </c>
       <c r="C668" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">file</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D668" t="inlineStr" s="2">
@@ -18895,11 +18903,7 @@
       </c>
       <c r="E668" s="2"/>
       <c r="F668" s="2"/>
-      <c r="G668" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
-        </is>
-      </c>
+      <c r="G668" s="2"/>
     </row>
     <row r="669">
       <c r="A669" t="inlineStr" s="2">
@@ -18909,12 +18913,12 @@
       </c>
       <c r="B669" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">foto_url</t>
+          <t xml:space="preserve">potencia_kwp</t>
         </is>
       </c>
       <c r="C669" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D669" t="inlineStr" s="2">
@@ -18934,12 +18938,12 @@
       </c>
       <c r="B670" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ordem</t>
+          <t xml:space="preserve">foto</t>
         </is>
       </c>
       <c r="C670" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="D670" t="inlineStr" s="2">
@@ -18949,7 +18953,11 @@
       </c>
       <c r="E670" s="2"/>
       <c r="F670" s="2"/>
-      <c r="G670" s="2"/>
+      <c r="G670" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
+        </is>
+      </c>
     </row>
     <row r="671">
       <c r="A671" t="inlineStr" s="2">
@@ -18959,12 +18967,12 @@
       </c>
       <c r="B671" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">destaque</t>
+          <t xml:space="preserve">foto_url</t>
         </is>
       </c>
       <c r="C671" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D671" t="inlineStr" s="2">
@@ -18972,11 +18980,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E671" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E671" s="2"/>
       <c r="F671" s="2"/>
       <c r="G671" s="2"/>
     </row>
@@ -18988,12 +18992,12 @@
       </c>
       <c r="B672" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">ordem</t>
         </is>
       </c>
       <c r="C672" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D672" t="inlineStr" s="2">
@@ -19003,11 +19007,7 @@
       </c>
       <c r="E672" s="2"/>
       <c r="F672" s="2"/>
-      <c r="G672" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G672" s="2"/>
     </row>
     <row r="673">
       <c r="A673" t="inlineStr" s="2">
@@ -19017,12 +19017,12 @@
       </c>
       <c r="B673" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">destaque</t>
         </is>
       </c>
       <c r="C673" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D673" t="inlineStr" s="2">
@@ -19030,67 +19030,71 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E673" s="2"/>
+      <c r="E673" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F673" s="2"/>
-      <c r="G673" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G673" s="2"/>
     </row>
     <row r="674">
       <c r="A674" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">projecao_tarifaria</t>
+          <t xml:space="preserve">instalacoes_galeria</t>
         </is>
       </c>
       <c r="B674" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ano</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C674" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D674" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E674" s="2"/>
       <c r="F674" s="2"/>
-      <c r="G674" s="2"/>
+      <c r="G674" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="675">
       <c r="A675" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">projecao_tarifaria</t>
+          <t xml:space="preserve">instalacoes_galeria</t>
         </is>
       </c>
       <c r="B675" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_cliente</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C675" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D675" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E675" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">residencial | comercial</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E675" s="2"/>
       <c r="F675" s="2"/>
-      <c r="G675" s="2"/>
+      <c r="G675" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="676">
       <c r="A676" t="inlineStr" s="2">
@@ -19100,7 +19104,7 @@
       </c>
       <c r="B676" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tarifa_kwh</t>
+          <t xml:space="preserve">ano</t>
         </is>
       </c>
       <c r="C676" t="inlineStr" s="2">
@@ -19110,7 +19114,7 @@
       </c>
       <c r="D676" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E676" s="2"/>
@@ -19125,20 +19129,24 @@
       </c>
       <c r="B677" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fio_b_kwh</t>
+          <t xml:space="preserve">tipo_cliente</t>
         </is>
       </c>
       <c r="C677" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D677" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E677" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">residencial | comercial</t>
+        </is>
+      </c>
       <c r="F677" s="2"/>
       <c r="G677" s="2"/>
     </row>
@@ -19150,7 +19158,7 @@
       </c>
       <c r="B678" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fs</t>
+          <t xml:space="preserve">tarifa_kwh</t>
         </is>
       </c>
       <c r="C678" t="inlineStr" s="2">
@@ -19175,7 +19183,7 @@
       </c>
       <c r="B679" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gd_eco_liquida</t>
+          <t xml:space="preserve">fio_b_kwh</t>
         </is>
       </c>
       <c r="C679" t="inlineStr" s="2">
@@ -19200,7 +19208,7 @@
       </c>
       <c r="B680" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">economia_acumulada</t>
+          <t xml:space="preserve">fs</t>
         </is>
       </c>
       <c r="C680" t="inlineStr" s="2">
@@ -19225,7 +19233,7 @@
       </c>
       <c r="B681" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gasto_acumulado</t>
+          <t xml:space="preserve">gd_eco_liquida</t>
         </is>
       </c>
       <c r="C681" t="inlineStr" s="2">
@@ -19250,12 +19258,12 @@
       </c>
       <c r="B682" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">economia_acumulada</t>
         </is>
       </c>
       <c r="C682" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D682" t="inlineStr" s="2">
@@ -19265,11 +19273,7 @@
       </c>
       <c r="E682" s="2"/>
       <c r="F682" s="2"/>
-      <c r="G682" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G682" s="2"/>
     </row>
     <row r="683">
       <c r="A683" t="inlineStr" s="2">
@@ -19279,12 +19283,12 @@
       </c>
       <c r="B683" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">gasto_acumulado</t>
         </is>
       </c>
       <c r="C683" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D683" t="inlineStr" s="2">
@@ -19294,65 +19298,65 @@
       </c>
       <c r="E683" s="2"/>
       <c r="F683" s="2"/>
-      <c r="G683" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G683" s="2"/>
     </row>
     <row r="684">
       <c r="A684" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">equipamentos</t>
+          <t xml:space="preserve">projecao_tarifaria</t>
         </is>
       </c>
       <c r="B684" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C684" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D684" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E684" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">inversor | modulo_fv</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E684" s="2"/>
       <c r="F684" s="2"/>
-      <c r="G684" s="2"/>
+      <c r="G684" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="685">
       <c r="A685" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">equipamentos</t>
+          <t xml:space="preserve">projecao_tarifaria</t>
         </is>
       </c>
       <c r="B685" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">marca</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C685" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D685" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E685" s="2"/>
       <c r="F685" s="2"/>
-      <c r="G685" s="2"/>
+      <c r="G685" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="686">
       <c r="A686" t="inlineStr" s="2">
@@ -19362,12 +19366,12 @@
       </c>
       <c r="B686" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">modelo</t>
+          <t xml:space="preserve">tipo</t>
         </is>
       </c>
       <c r="C686" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D686" t="inlineStr" s="2">
@@ -19375,7 +19379,11 @@
           <t xml:space="preserve">Sim</t>
         </is>
       </c>
-      <c r="E686" s="2"/>
+      <c r="E686" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">inversor | modulo_fv</t>
+        </is>
+      </c>
       <c r="F686" s="2"/>
       <c r="G686" s="2"/>
     </row>
@@ -19387,12 +19395,12 @@
       </c>
       <c r="B687" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">potencia_w</t>
+          <t xml:space="preserve">marca</t>
         </is>
       </c>
       <c r="C687" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D687" t="inlineStr" s="2">
@@ -19412,7 +19420,7 @@
       </c>
       <c r="B688" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">descricao_padrao</t>
+          <t xml:space="preserve">modelo</t>
         </is>
       </c>
       <c r="C688" t="inlineStr" s="2">
@@ -19422,7 +19430,7 @@
       </c>
       <c r="D688" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E688" s="2"/>
@@ -19437,7 +19445,7 @@
       </c>
       <c r="B689" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">garantia_anos</t>
+          <t xml:space="preserve">potencia_w</t>
         </is>
       </c>
       <c r="C689" t="inlineStr" s="2">
@@ -19447,7 +19455,7 @@
       </c>
       <c r="D689" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E689" s="2"/>
@@ -19462,12 +19470,12 @@
       </c>
       <c r="B690" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">foto</t>
+          <t xml:space="preserve">descricao_padrao</t>
         </is>
       </c>
       <c r="C690" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">file</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D690" t="inlineStr" s="2">
@@ -19477,11 +19485,7 @@
       </c>
       <c r="E690" s="2"/>
       <c r="F690" s="2"/>
-      <c r="G690" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
-        </is>
-      </c>
+      <c r="G690" s="2"/>
     </row>
     <row r="691">
       <c r="A691" t="inlineStr" s="2">
@@ -19491,12 +19495,12 @@
       </c>
       <c r="B691" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">garantia_anos</t>
         </is>
       </c>
       <c r="C691" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D691" t="inlineStr" s="2">
@@ -19506,11 +19510,7 @@
       </c>
       <c r="E691" s="2"/>
       <c r="F691" s="2"/>
-      <c r="G691" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G691" s="2"/>
     </row>
     <row r="692">
       <c r="A692" t="inlineStr" s="2">
@@ -19520,12 +19520,12 @@
       </c>
       <c r="B692" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">foto</t>
         </is>
       </c>
       <c r="C692" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="D692" t="inlineStr" s="2">
@@ -19537,7 +19537,7 @@
       <c r="F692" s="2"/>
       <c r="G692" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
         </is>
       </c>
     </row>
@@ -19549,12 +19549,12 @@
       </c>
       <c r="B693" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">datasheet_pdf</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C693" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">file</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D693" t="inlineStr" s="2">
@@ -19566,63 +19566,67 @@
       <c r="F693" s="2"/>
       <c r="G693" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="694">
       <c r="A694" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">parametros_tarifarios</t>
+          <t xml:space="preserve">equipamentos</t>
         </is>
       </c>
       <c r="B694" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ano</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C694" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D694" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E694" s="2"/>
       <c r="F694" s="2"/>
-      <c r="G694" s="2"/>
+      <c r="G694" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="695">
       <c r="A695" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">parametros_tarifarios</t>
+          <t xml:space="preserve">equipamentos</t>
         </is>
       </c>
       <c r="B695" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">classe</t>
+          <t xml:space="preserve">datasheet_pdf</t>
         </is>
       </c>
       <c r="C695" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="D695" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E695" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">residencial | comercial</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E695" s="2"/>
       <c r="F695" s="2"/>
-      <c r="G695" s="2"/>
+      <c r="G695" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
+        </is>
+      </c>
     </row>
     <row r="696">
       <c r="A696" t="inlineStr" s="2">
@@ -19632,7 +19636,7 @@
       </c>
       <c r="B696" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tarifa</t>
+          <t xml:space="preserve">ano</t>
         </is>
       </c>
       <c r="C696" t="inlineStr" s="2">
@@ -19642,7 +19646,7 @@
       </c>
       <c r="D696" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E696" s="2"/>
@@ -19657,20 +19661,24 @@
       </c>
       <c r="B697" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fio_b</t>
+          <t xml:space="preserve">classe</t>
         </is>
       </c>
       <c r="C697" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D697" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E697" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">residencial | comercial</t>
+        </is>
+      </c>
       <c r="F697" s="2"/>
       <c r="G697" s="2"/>
     </row>
@@ -19682,7 +19690,7 @@
       </c>
       <c r="B698" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fs</t>
+          <t xml:space="preserve">tarifa</t>
         </is>
       </c>
       <c r="C698" t="inlineStr" s="2">
@@ -19707,7 +19715,7 @@
       </c>
       <c r="B699" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gd_eco_liquida</t>
+          <t xml:space="preserve">fio_b</t>
         </is>
       </c>
       <c r="C699" t="inlineStr" s="2">
@@ -19732,12 +19740,12 @@
       </c>
       <c r="B700" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">fs</t>
         </is>
       </c>
       <c r="C700" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D700" t="inlineStr" s="2">
@@ -19747,11 +19755,7 @@
       </c>
       <c r="E700" s="2"/>
       <c r="F700" s="2"/>
-      <c r="G700" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G700" s="2"/>
     </row>
     <row r="701">
       <c r="A701" t="inlineStr" s="2">
@@ -19761,12 +19765,12 @@
       </c>
       <c r="B701" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">gd_eco_liquida</t>
         </is>
       </c>
       <c r="C701" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D701" t="inlineStr" s="2">
@@ -19776,65 +19780,65 @@
       </c>
       <c r="E701" s="2"/>
       <c r="F701" s="2"/>
-      <c r="G701" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G701" s="2"/>
     </row>
     <row r="702">
       <c r="A702" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">parametros_tarifarios</t>
         </is>
       </c>
       <c r="B702" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">nome</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C702" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D702" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E702" s="2"/>
       <c r="F702" s="2"/>
-      <c r="G702" s="2"/>
+      <c r="G702" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="703">
       <c r="A703" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">parametros_tarifarios</t>
         </is>
       </c>
       <c r="B703" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gatilho</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C703" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D703" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E703" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">status_mudou | instalacao_concluida | atividade_concluida | data_especifica | dias_apos_evento</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E703" s="2"/>
       <c r="F703" s="2"/>
-      <c r="G703" s="2"/>
+      <c r="G703" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="704">
       <c r="A704" t="inlineStr" s="2">
@@ -19844,26 +19848,22 @@
       </c>
       <c r="B704" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">configuracao_gatilho</t>
+          <t xml:space="preserve">nome</t>
         </is>
       </c>
       <c r="C704" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D704" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E704" s="2"/>
       <c r="F704" s="2"/>
-      <c r="G704" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="G704" s="2"/>
     </row>
     <row r="705">
       <c r="A705" t="inlineStr" s="2">
@@ -19873,7 +19873,7 @@
       </c>
       <c r="B705" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">acao</t>
+          <t xml:space="preserve">gatilho</t>
         </is>
       </c>
       <c r="C705" t="inlineStr" s="2">
@@ -19888,7 +19888,7 @@
       </c>
       <c r="E705" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">criar_atividade | enviar_whatsapp | enviar_email | mudar_status</t>
+          <t xml:space="preserve">status_mudou | instalacao_concluida | atividade_concluida | data_especifica | dias_apos_evento</t>
         </is>
       </c>
       <c r="F705" s="2"/>
@@ -19902,7 +19902,7 @@
       </c>
       <c r="B706" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">configuracao_acao</t>
+          <t xml:space="preserve">configuracao_gatilho</t>
         </is>
       </c>
       <c r="C706" t="inlineStr" s="2">
@@ -19931,7 +19931,7 @@
       </c>
       <c r="B707" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">destino</t>
+          <t xml:space="preserve">acao</t>
         </is>
       </c>
       <c r="C707" t="inlineStr" s="2">
@@ -19946,7 +19946,7 @@
       </c>
       <c r="E707" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_evento | responsavel_empresa | cliente_especifico</t>
+          <t xml:space="preserve">criar_atividade | enviar_whatsapp | enviar_email | mudar_status</t>
         </is>
       </c>
       <c r="F707" s="2"/>
@@ -19960,12 +19960,12 @@
       </c>
       <c r="B708" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_especifico_id</t>
+          <t xml:space="preserve">configuracao_acao</t>
         </is>
       </c>
       <c r="C708" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D708" t="inlineStr" s="2">
@@ -19974,12 +19974,12 @@
         </is>
       </c>
       <c r="E708" s="2"/>
-      <c r="F708" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
-      <c r="G708" s="2"/>
+      <c r="F708" s="2"/>
+      <c r="G708" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Estrutura JSON livre</t>
+        </is>
+      </c>
     </row>
     <row r="709">
       <c r="A709" t="inlineStr" s="2">
@@ -19989,22 +19989,22 @@
       </c>
       <c r="B709" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ativa</t>
+          <t xml:space="preserve">destino</t>
         </is>
       </c>
       <c r="C709" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D709" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E709" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">true / false</t>
+          <t xml:space="preserve">cliente_evento | responsavel_empresa | cliente_especifico</t>
         </is>
       </c>
       <c r="F709" s="2"/>
@@ -20018,12 +20018,12 @@
       </c>
       <c r="B710" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">cliente_especifico_id</t>
         </is>
       </c>
       <c r="C710" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D710" t="inlineStr" s="2">
@@ -20032,12 +20032,12 @@
         </is>
       </c>
       <c r="E710" s="2"/>
-      <c r="F710" s="2"/>
-      <c r="G710" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="F710" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
+      <c r="G710" s="2"/>
     </row>
     <row r="711">
       <c r="A711" t="inlineStr" s="2">
@@ -20047,12 +20047,12 @@
       </c>
       <c r="B711" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">ativa</t>
         </is>
       </c>
       <c r="C711" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D711" t="inlineStr" s="2">
@@ -20060,67 +20060,71 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E711" s="2"/>
+      <c r="E711" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F711" s="2"/>
-      <c r="G711" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G711" s="2"/>
     </row>
     <row r="712">
       <c r="A712" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes_execucoes</t>
+          <t xml:space="preserve">automacoes</t>
         </is>
       </c>
       <c r="B712" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacao</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C712" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D712" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E712" s="2"/>
-      <c r="F712" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">automacoes</t>
-        </is>
-      </c>
-      <c r="G712" s="2"/>
+      <c r="F712" s="2"/>
+      <c r="G712" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="713">
       <c r="A713" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes_execucoes</t>
+          <t xml:space="preserve">automacoes</t>
         </is>
       </c>
       <c r="B713" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_execucao</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C713" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D713" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E713" s="2"/>
       <c r="F713" s="2"/>
-      <c r="G713" s="2"/>
+      <c r="G713" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="714">
       <c r="A714" t="inlineStr" s="2">
@@ -20130,25 +20134,25 @@
       </c>
       <c r="B714" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">sucesso</t>
+          <t xml:space="preserve">automacao</t>
         </is>
       </c>
       <c r="C714" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D714" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E714" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
-      <c r="F714" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E714" s="2"/>
+      <c r="F714" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">automacoes</t>
+        </is>
+      </c>
       <c r="G714" s="2"/>
     </row>
     <row r="715">
@@ -20159,17 +20163,17 @@
       </c>
       <c r="B715" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mensagem</t>
+          <t xml:space="preserve">data_execucao</t>
         </is>
       </c>
       <c r="C715" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D715" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E715" s="2"/>
@@ -20184,12 +20188,12 @@
       </c>
       <c r="B716" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">referencia_registro</t>
+          <t xml:space="preserve">sucesso</t>
         </is>
       </c>
       <c r="C716" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D716" t="inlineStr" s="2">
@@ -20197,7 +20201,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E716" s="2"/>
+      <c r="E716" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F716" s="2"/>
       <c r="G716" s="2"/>
     </row>
@@ -20209,12 +20217,12 @@
       </c>
       <c r="B717" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente</t>
+          <t xml:space="preserve">mensagem</t>
         </is>
       </c>
       <c r="C717" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D717" t="inlineStr" s="2">
@@ -20223,11 +20231,7 @@
         </is>
       </c>
       <c r="E717" s="2"/>
-      <c r="F717" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+      <c r="F717" s="2"/>
       <c r="G717" s="2"/>
     </row>
     <row r="718">
@@ -20238,12 +20242,12 @@
       </c>
       <c r="B718" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">dados_execucao</t>
+          <t xml:space="preserve">referencia_registro</t>
         </is>
       </c>
       <c r="C718" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D718" t="inlineStr" s="2">
@@ -20253,11 +20257,7 @@
       </c>
       <c r="E718" s="2"/>
       <c r="F718" s="2"/>
-      <c r="G718" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="G718" s="2"/>
     </row>
     <row r="719">
       <c r="A719" t="inlineStr" s="2">
@@ -20267,12 +20267,12 @@
       </c>
       <c r="B719" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">cliente</t>
         </is>
       </c>
       <c r="C719" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D719" t="inlineStr" s="2">
@@ -20281,12 +20281,12 @@
         </is>
       </c>
       <c r="E719" s="2"/>
-      <c r="F719" s="2"/>
-      <c r="G719" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="F719" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
+      <c r="G719" s="2"/>
     </row>
     <row r="720">
       <c r="A720" t="inlineStr" s="2">
@@ -20296,12 +20296,12 @@
       </c>
       <c r="B720" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">dados_execucao</t>
         </is>
       </c>
       <c r="C720" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D720" t="inlineStr" s="2">
@@ -20313,63 +20313,67 @@
       <c r="F720" s="2"/>
       <c r="G720" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Estrutura JSON livre</t>
         </is>
       </c>
     </row>
     <row r="721">
       <c r="A721" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">automacoes_execucoes</t>
         </is>
       </c>
       <c r="B721" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C721" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D721" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E721" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">atividade_atrasada | lembrete | sistema</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E721" s="2"/>
       <c r="F721" s="2"/>
-      <c r="G721" s="2"/>
+      <c r="G721" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="722">
       <c r="A722" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">automacoes_execucoes</t>
         </is>
       </c>
       <c r="B722" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C722" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D722" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E722" s="2"/>
       <c r="F722" s="2"/>
-      <c r="G722" s="2"/>
+      <c r="G722" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="723">
       <c r="A723" t="inlineStr" s="2">
@@ -20379,20 +20383,24 @@
       </c>
       <c r="B723" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mensagem</t>
+          <t xml:space="preserve">tipo</t>
         </is>
       </c>
       <c r="C723" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D723" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E723" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E723" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">atividade_atrasada | lembrete | sistema</t>
+        </is>
+      </c>
       <c r="F723" s="2"/>
       <c r="G723" s="2"/>
     </row>
@@ -20404,25 +20412,21 @@
       </c>
       <c r="B724" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">atividade_id</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C724" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D724" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E724" s="2"/>
-      <c r="F724" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">atividades</t>
-        </is>
-      </c>
+      <c r="F724" s="2"/>
       <c r="G724" s="2"/>
     </row>
     <row r="725">
@@ -20433,12 +20437,12 @@
       </c>
       <c r="B725" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_id</t>
+          <t xml:space="preserve">mensagem</t>
         </is>
       </c>
       <c r="C725" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D725" t="inlineStr" s="2">
@@ -20447,11 +20451,7 @@
         </is>
       </c>
       <c r="E725" s="2"/>
-      <c r="F725" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+      <c r="F725" s="2"/>
       <c r="G725" s="2"/>
     </row>
     <row r="726">
@@ -20462,12 +20462,12 @@
       </c>
       <c r="B726" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_nome</t>
+          <t xml:space="preserve">atividade_id</t>
         </is>
       </c>
       <c r="C726" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D726" t="inlineStr" s="2">
@@ -20476,7 +20476,11 @@
         </is>
       </c>
       <c r="E726" s="2"/>
-      <c r="F726" s="2"/>
+      <c r="F726" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">atividades</t>
+        </is>
+      </c>
       <c r="G726" s="2"/>
     </row>
     <row r="727">
@@ -20487,12 +20491,12 @@
       </c>
       <c r="B727" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_prevista</t>
+          <t xml:space="preserve">cliente_id</t>
         </is>
       </c>
       <c r="C727" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D727" t="inlineStr" s="2">
@@ -20501,7 +20505,11 @@
         </is>
       </c>
       <c r="E727" s="2"/>
-      <c r="F727" s="2"/>
+      <c r="F727" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G727" s="2"/>
     </row>
     <row r="728">
@@ -20512,12 +20520,12 @@
       </c>
       <c r="B728" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">dias_atraso</t>
+          <t xml:space="preserve">cliente_nome</t>
         </is>
       </c>
       <c r="C728" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D728" t="inlineStr" s="2">
@@ -20537,12 +20545,12 @@
       </c>
       <c r="B729" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">lida</t>
+          <t xml:space="preserve">data_prevista</t>
         </is>
       </c>
       <c r="C729" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D729" t="inlineStr" s="2">
@@ -20550,11 +20558,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E729" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E729" s="2"/>
       <c r="F729" s="2"/>
       <c r="G729" s="2"/>
     </row>
@@ -20566,12 +20570,12 @@
       </c>
       <c r="B730" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">lida_em</t>
+          <t xml:space="preserve">dias_atraso</t>
         </is>
       </c>
       <c r="C730" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D730" t="inlineStr" s="2">
@@ -20591,22 +20595,22 @@
       </c>
       <c r="B731" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">lida</t>
         </is>
       </c>
       <c r="C731" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D731" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E731" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ativa | resolvida | arquivada</t>
+          <t xml:space="preserve">true / false</t>
         </is>
       </c>
       <c r="F731" s="2"/>
@@ -20620,7 +20624,7 @@
       </c>
       <c r="B732" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">resolvida_em</t>
+          <t xml:space="preserve">lida_em</t>
         </is>
       </c>
       <c r="C732" t="inlineStr" s="2">
@@ -20645,26 +20649,26 @@
       </c>
       <c r="B733" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="C733" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D733" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E733" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativa | resolvida | arquivada</t>
+        </is>
+      </c>
       <c r="F733" s="2"/>
-      <c r="G733" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G733" s="2"/>
     </row>
     <row r="734">
       <c r="A734" t="inlineStr" s="2">
@@ -20674,12 +20678,12 @@
       </c>
       <c r="B734" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">resolvida_em</t>
         </is>
       </c>
       <c r="C734" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D734" t="inlineStr" s="2">
@@ -20689,55 +20693,51 @@
       </c>
       <c r="E734" s="2"/>
       <c r="F734" s="2"/>
-      <c r="G734" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G734" s="2"/>
     </row>
     <row r="735">
       <c r="A735" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">notificacoes_internas</t>
         </is>
       </c>
       <c r="B735" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_id</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C735" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D735" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E735" s="2"/>
-      <c r="F735" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
-      <c r="G735" s="2"/>
+      <c r="F735" s="2"/>
+      <c r="G735" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="736">
       <c r="A736" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">notificacoes_internas</t>
         </is>
       </c>
       <c r="B736" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_negocio</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C736" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D736" t="inlineStr" s="2">
@@ -20745,13 +20745,13 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E736" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">venda usina | bateria | expansão | renovação | serviço | venda bateria</t>
-        </is>
-      </c>
+      <c r="E736" s="2"/>
       <c r="F736" s="2"/>
-      <c r="G736" s="2"/>
+      <c r="G736" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="737">
       <c r="A737" t="inlineStr" s="2">
@@ -20761,21 +20761,25 @@
       </c>
       <c r="B737" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">valor_estimado</t>
+          <t xml:space="preserve">cliente_id</t>
         </is>
       </c>
       <c r="C737" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D737" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E737" s="2"/>
-      <c r="F737" s="2"/>
+      <c r="F737" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G737" s="2"/>
     </row>
     <row r="738">
@@ -20786,12 +20790,12 @@
       </c>
       <c r="B738" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">valor_final</t>
+          <t xml:space="preserve">tipo_negocio</t>
         </is>
       </c>
       <c r="C738" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D738" t="inlineStr" s="2">
@@ -20799,7 +20803,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E738" s="2"/>
+      <c r="E738" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">venda usina | bateria | expansão | renovação | serviço | venda bateria</t>
+        </is>
+      </c>
       <c r="F738" s="2"/>
       <c r="G738" s="2"/>
     </row>
@@ -20811,12 +20819,12 @@
       </c>
       <c r="B739" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">etapa_funil</t>
+          <t xml:space="preserve">valor_estimado</t>
         </is>
       </c>
       <c r="C739" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D739" t="inlineStr" s="2">
@@ -20824,11 +20832,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E739" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">novo lead | qualificado | proposta enviada | negociação | contrato assinado</t>
-        </is>
-      </c>
+      <c r="E739" s="2"/>
       <c r="F739" s="2"/>
       <c r="G739" s="2"/>
     </row>
@@ -20840,7 +20844,7 @@
       </c>
       <c r="B740" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">probabilidade</t>
+          <t xml:space="preserve">valor_final</t>
         </is>
       </c>
       <c r="C740" t="inlineStr" s="2">
@@ -20865,12 +20869,12 @@
       </c>
       <c r="B741" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_previsao_fechamento</t>
+          <t xml:space="preserve">etapa_funil</t>
         </is>
       </c>
       <c r="C741" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D741" t="inlineStr" s="2">
@@ -20878,7 +20882,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E741" s="2"/>
+      <c r="E741" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">novo lead | qualificado | proposta enviada | negociação | contrato assinado</t>
+        </is>
+      </c>
       <c r="F741" s="2"/>
       <c r="G741" s="2"/>
     </row>
@@ -20890,12 +20898,12 @@
       </c>
       <c r="B742" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_fechamento</t>
+          <t xml:space="preserve">probabilidade</t>
         </is>
       </c>
       <c r="C742" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D742" t="inlineStr" s="2">
@@ -20915,12 +20923,12 @@
       </c>
       <c r="B743" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">data_previsao_fechamento</t>
         </is>
       </c>
       <c r="C743" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D743" t="inlineStr" s="2">
@@ -20928,11 +20936,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E743" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">em andamento | ganho | perdido</t>
-        </is>
-      </c>
+      <c r="E743" s="2"/>
       <c r="F743" s="2"/>
       <c r="G743" s="2"/>
     </row>
@@ -20944,12 +20948,12 @@
       </c>
       <c r="B744" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">motivo_perda</t>
+          <t xml:space="preserve">data_fechamento</t>
         </is>
       </c>
       <c r="C744" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D744" t="inlineStr" s="2">
@@ -20969,12 +20973,12 @@
       </c>
       <c r="B745" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">reabertura</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="C745" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D745" t="inlineStr" s="2">
@@ -20984,7 +20988,7 @@
       </c>
       <c r="E745" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">true / false</t>
+          <t xml:space="preserve">em andamento | ganho | perdido</t>
         </is>
       </c>
       <c r="F745" s="2"/>
@@ -20998,7 +21002,7 @@
       </c>
       <c r="B746" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">motivo_reabertura</t>
+          <t xml:space="preserve">motivo_perda</t>
         </is>
       </c>
       <c r="C746" t="inlineStr" s="2">
@@ -21023,12 +21027,12 @@
       </c>
       <c r="B747" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">condicao_pagamento</t>
+          <t xml:space="preserve">reabertura</t>
         </is>
       </c>
       <c r="C747" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D747" t="inlineStr" s="2">
@@ -21036,7 +21040,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E747" s="2"/>
+      <c r="E747" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F747" s="2"/>
       <c r="G747" s="2"/>
     </row>
@@ -21048,12 +21056,12 @@
       </c>
       <c r="B748" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">motivo_reabertura</t>
         </is>
       </c>
       <c r="C748" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D748" t="inlineStr" s="2">
@@ -21063,11 +21071,7 @@
       </c>
       <c r="E748" s="2"/>
       <c r="F748" s="2"/>
-      <c r="G748" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G748" s="2"/>
     </row>
     <row r="749">
       <c r="A749" t="inlineStr" s="2">
@@ -21077,12 +21081,12 @@
       </c>
       <c r="B749" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">condicao_pagamento</t>
         </is>
       </c>
       <c r="C749" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D749" t="inlineStr" s="2">
@@ -21092,11 +21096,7 @@
       </c>
       <c r="E749" s="2"/>
       <c r="F749" s="2"/>
-      <c r="G749" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G749" s="2"/>
     </row>
     <row r="750">
       <c r="A750" t="inlineStr" s="2">
@@ -21106,12 +21106,12 @@
       </c>
       <c r="B750" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_venda</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C750" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D750" t="inlineStr" s="2">
@@ -21119,13 +21119,13 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E750" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Energia Solar | O&amp;M (Operação e Manutenção) | Baterias | Carregadores Veículos Elétricos</t>
-        </is>
-      </c>
+      <c r="E750" s="2"/>
       <c r="F750" s="2"/>
-      <c r="G750" s="2"/>
+      <c r="G750" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="751">
       <c r="A751" t="inlineStr" s="2">
@@ -21135,12 +21135,12 @@
       </c>
       <c r="B751" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C751" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D751" t="inlineStr" s="2">
@@ -21150,7 +21150,11 @@
       </c>
       <c r="E751" s="2"/>
       <c r="F751" s="2"/>
-      <c r="G751" s="2"/>
+      <c r="G751" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="752">
       <c r="A752" t="inlineStr" s="2">
@@ -21160,12 +21164,12 @@
       </c>
       <c r="B752" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">valor</t>
+          <t xml:space="preserve">tipo_venda</t>
         </is>
       </c>
       <c r="C752" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D752" t="inlineStr" s="2">
@@ -21173,7 +21177,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E752" s="2"/>
+      <c r="E752" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Energia Solar | O&amp;M (Operação e Manutenção) | Baterias | Carregadores Veículos Elétricos</t>
+        </is>
+      </c>
       <c r="F752" s="2"/>
       <c r="G752" s="2"/>
     </row>
@@ -21185,12 +21193,12 @@
       </c>
       <c r="B753" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">consultor_responsavel</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C753" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D753" t="inlineStr" s="2">
@@ -21199,11 +21207,7 @@
         </is>
       </c>
       <c r="E753" s="2"/>
-      <c r="F753" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">users</t>
-        </is>
-      </c>
+      <c r="F753" s="2"/>
       <c r="G753" s="2"/>
     </row>
     <row r="754">
@@ -21214,12 +21218,12 @@
       </c>
       <c r="B754" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">recorrencia_mensal</t>
+          <t xml:space="preserve">valor</t>
         </is>
       </c>
       <c r="C754" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D754" t="inlineStr" s="2">
@@ -21227,53 +21231,53 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E754" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E754" s="2"/>
       <c r="F754" s="2"/>
       <c r="G754" s="2"/>
     </row>
     <row r="755">
       <c r="A755" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">analises_fatura</t>
+          <t xml:space="preserve">negocios</t>
         </is>
       </c>
       <c r="B755" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">token</t>
+          <t xml:space="preserve">consultor_responsavel</t>
         </is>
       </c>
       <c r="C755" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D755" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E755" s="2"/>
-      <c r="F755" s="2"/>
+      <c r="F755" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">users</t>
+        </is>
+      </c>
       <c r="G755" s="2"/>
     </row>
     <row r="756">
       <c r="A756" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">analises_fatura</t>
+          <t xml:space="preserve">negocios</t>
         </is>
       </c>
       <c r="B756" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_id</t>
+          <t xml:space="preserve">recorrencia_mensal</t>
         </is>
       </c>
       <c r="C756" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D756" t="inlineStr" s="2">
@@ -21281,12 +21285,12 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E756" s="2"/>
-      <c r="F756" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+      <c r="E756" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
+      <c r="F756" s="2"/>
       <c r="G756" s="2"/>
     </row>
     <row r="757">
@@ -21297,7 +21301,7 @@
       </c>
       <c r="B757" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_nome</t>
+          <t xml:space="preserve">token</t>
         </is>
       </c>
       <c r="C757" t="inlineStr" s="2">
@@ -21307,7 +21311,7 @@
       </c>
       <c r="D757" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E757" s="2"/>
@@ -21322,12 +21326,12 @@
       </c>
       <c r="B758" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">uc</t>
+          <t xml:space="preserve">cliente_id</t>
         </is>
       </c>
       <c r="C758" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D758" t="inlineStr" s="2">
@@ -21336,7 +21340,11 @@
         </is>
       </c>
       <c r="E758" s="2"/>
-      <c r="F758" s="2"/>
+      <c r="F758" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G758" s="2"/>
     </row>
     <row r="759">
@@ -21347,7 +21355,7 @@
       </c>
       <c r="B759" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">competencia</t>
+          <t xml:space="preserve">cliente_nome</t>
         </is>
       </c>
       <c r="C759" t="inlineStr" s="2">
@@ -21372,7 +21380,7 @@
       </c>
       <c r="B760" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">vencimento</t>
+          <t xml:space="preserve">uc</t>
         </is>
       </c>
       <c r="C760" t="inlineStr" s="2">
@@ -21397,12 +21405,12 @@
       </c>
       <c r="B761" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">total_pagar</t>
+          <t xml:space="preserve">competencia</t>
         </is>
       </c>
       <c r="C761" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D761" t="inlineStr" s="2">
@@ -21422,12 +21430,12 @@
       </c>
       <c r="B762" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">consumo_kwh</t>
+          <t xml:space="preserve">vencimento</t>
         </is>
       </c>
       <c r="C762" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D762" t="inlineStr" s="2">
@@ -21447,7 +21455,7 @@
       </c>
       <c r="B763" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">energia_injetada_kwh</t>
+          <t xml:space="preserve">total_pagar</t>
         </is>
       </c>
       <c r="C763" t="inlineStr" s="2">
@@ -21472,7 +21480,7 @@
       </c>
       <c r="B764" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">creditos_compensados_kwh</t>
+          <t xml:space="preserve">consumo_kwh</t>
         </is>
       </c>
       <c r="C764" t="inlineStr" s="2">
@@ -21497,7 +21505,7 @@
       </c>
       <c r="B765" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">saldo_energia_kwh</t>
+          <t xml:space="preserve">energia_injetada_kwh</t>
         </is>
       </c>
       <c r="C765" t="inlineStr" s="2">
@@ -21522,7 +21530,7 @@
       </c>
       <c r="B766" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">saldo_expirar_kwh</t>
+          <t xml:space="preserve">creditos_compensados_kwh</t>
         </is>
       </c>
       <c r="C766" t="inlineStr" s="2">
@@ -21547,7 +21555,7 @@
       </c>
       <c r="B767" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">economia_estimada_rs</t>
+          <t xml:space="preserve">saldo_energia_kwh</t>
         </is>
       </c>
       <c r="C767" t="inlineStr" s="2">
@@ -21572,12 +21580,12 @@
       </c>
       <c r="B768" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">papel_uc</t>
+          <t xml:space="preserve">saldo_expirar_kwh</t>
         </is>
       </c>
       <c r="C768" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D768" t="inlineStr" s="2">
@@ -21597,12 +21605,12 @@
       </c>
       <c r="B769" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">arquivos_nomes</t>
+          <t xml:space="preserve">economia_estimada_rs</t>
         </is>
       </c>
       <c r="C769" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D769" t="inlineStr" s="2">
@@ -21612,11 +21620,7 @@
       </c>
       <c r="E769" s="2"/>
       <c r="F769" s="2"/>
-      <c r="G769" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="G769" s="2"/>
     </row>
     <row r="770">
       <c r="A770" t="inlineStr" s="2">
@@ -21626,12 +21630,12 @@
       </c>
       <c r="B770" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">dados_completos</t>
+          <t xml:space="preserve">papel_uc</t>
         </is>
       </c>
       <c r="C770" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D770" t="inlineStr" s="2">
@@ -21641,11 +21645,7 @@
       </c>
       <c r="E770" s="2"/>
       <c r="F770" s="2"/>
-      <c r="G770" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="G770" s="2"/>
     </row>
     <row r="771">
       <c r="A771" t="inlineStr" s="2">
@@ -21655,12 +21655,12 @@
       </c>
       <c r="B771" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">atividade_id</t>
+          <t xml:space="preserve">arquivos_nomes</t>
         </is>
       </c>
       <c r="C771" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D771" t="inlineStr" s="2">
@@ -21670,7 +21670,11 @@
       </c>
       <c r="E771" s="2"/>
       <c r="F771" s="2"/>
-      <c r="G771" s="2"/>
+      <c r="G771" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Estrutura JSON livre</t>
+        </is>
+      </c>
     </row>
     <row r="772">
       <c r="A772" t="inlineStr" s="2">
@@ -21680,12 +21684,12 @@
       </c>
       <c r="B772" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">whatsapp_enviado</t>
+          <t xml:space="preserve">dados_completos</t>
         </is>
       </c>
       <c r="C772" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D772" t="inlineStr" s="2">
@@ -21693,13 +21697,13 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E772" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E772" s="2"/>
       <c r="F772" s="2"/>
-      <c r="G772" s="2"/>
+      <c r="G772" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Estrutura JSON livre</t>
+        </is>
+      </c>
     </row>
     <row r="773">
       <c r="A773" t="inlineStr" s="2">
@@ -21709,7 +21713,7 @@
       </c>
       <c r="B773" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">whatsapp_enviado_em</t>
+          <t xml:space="preserve">atividade_id</t>
         </is>
       </c>
       <c r="C773" t="inlineStr" s="2">
@@ -21734,12 +21738,12 @@
       </c>
       <c r="B774" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">whatsapp_enviado</t>
         </is>
       </c>
       <c r="C774" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D774" t="inlineStr" s="2">
@@ -21747,13 +21751,13 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E774" s="2"/>
+      <c r="E774" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F774" s="2"/>
-      <c r="G774" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G774" s="2"/>
     </row>
     <row r="775">
       <c r="A775" t="inlineStr" s="2">
@@ -21763,12 +21767,12 @@
       </c>
       <c r="B775" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">whatsapp_enviado_em</t>
         </is>
       </c>
       <c r="C775" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D775" t="inlineStr" s="2">
@@ -21778,51 +21782,51 @@
       </c>
       <c r="E775" s="2"/>
       <c r="F775" s="2"/>
-      <c r="G775" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G775" s="2"/>
     </row>
     <row r="776">
       <c r="A776" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">knowledge_categories</t>
+          <t xml:space="preserve">analises_fatura</t>
         </is>
       </c>
       <c r="B776" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C776" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D776" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E776" s="2"/>
       <c r="F776" s="2"/>
-      <c r="G776" s="2"/>
+      <c r="G776" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="777">
       <c r="A777" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">knowledge_categories</t>
+          <t xml:space="preserve">analises_fatura</t>
         </is>
       </c>
       <c r="B777" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">descricao</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C777" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D777" t="inlineStr" s="2">
@@ -21832,7 +21836,11 @@
       </c>
       <c r="E777" s="2"/>
       <c r="F777" s="2"/>
-      <c r="G777" s="2"/>
+      <c r="G777" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="778">
       <c r="A778" t="inlineStr" s="2">
@@ -21842,7 +21850,7 @@
       </c>
       <c r="B778" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">icone</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C778" t="inlineStr" s="2">
@@ -21852,7 +21860,7 @@
       </c>
       <c r="D778" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E778" s="2"/>
@@ -21867,12 +21875,12 @@
       </c>
       <c r="B779" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ordem</t>
+          <t xml:space="preserve">descricao</t>
         </is>
       </c>
       <c r="C779" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D779" t="inlineStr" s="2">
@@ -21892,12 +21900,12 @@
       </c>
       <c r="B780" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">icone</t>
         </is>
       </c>
       <c r="C780" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D780" t="inlineStr" s="2">
@@ -21907,11 +21915,7 @@
       </c>
       <c r="E780" s="2"/>
       <c r="F780" s="2"/>
-      <c r="G780" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G780" s="2"/>
     </row>
     <row r="781">
       <c r="A781" t="inlineStr" s="2">
@@ -21921,12 +21925,12 @@
       </c>
       <c r="B781" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">ordem</t>
         </is>
       </c>
       <c r="C781" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D781" t="inlineStr" s="2">
@@ -21936,65 +21940,65 @@
       </c>
       <c r="E781" s="2"/>
       <c r="F781" s="2"/>
-      <c r="G781" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G781" s="2"/>
     </row>
     <row r="782">
       <c r="A782" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">knowledge_articles</t>
+          <t xml:space="preserve">knowledge_categories</t>
         </is>
       </c>
       <c r="B782" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">categoria_id</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C782" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D782" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E782" s="2"/>
-      <c r="F782" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">knowledge_categories</t>
-        </is>
-      </c>
-      <c r="G782" s="2"/>
+      <c r="F782" s="2"/>
+      <c r="G782" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="783">
       <c r="A783" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">knowledge_articles</t>
+          <t xml:space="preserve">knowledge_categories</t>
         </is>
       </c>
       <c r="B783" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C783" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D783" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E783" s="2"/>
       <c r="F783" s="2"/>
-      <c r="G783" s="2"/>
+      <c r="G783" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="784">
       <c r="A784" t="inlineStr" s="2">
@@ -22004,12 +22008,12 @@
       </c>
       <c r="B784" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">conteudo</t>
+          <t xml:space="preserve">categoria_id</t>
         </is>
       </c>
       <c r="C784" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D784" t="inlineStr" s="2">
@@ -22018,7 +22022,11 @@
         </is>
       </c>
       <c r="E784" s="2"/>
-      <c r="F784" s="2"/>
+      <c r="F784" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_categories</t>
+        </is>
+      </c>
       <c r="G784" s="2"/>
     </row>
     <row r="785">
@@ -22029,7 +22037,7 @@
       </c>
       <c r="B785" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">texto_extraido</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C785" t="inlineStr" s="2">
@@ -22039,7 +22047,7 @@
       </c>
       <c r="D785" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E785" s="2"/>
@@ -22054,26 +22062,22 @@
       </c>
       <c r="B786" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">anexos</t>
+          <t xml:space="preserve">conteudo</t>
         </is>
       </c>
       <c r="C786" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">file</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D786" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E786" s="2"/>
       <c r="F786" s="2"/>
-      <c r="G786" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
-        </is>
-      </c>
+      <c r="G786" s="2"/>
     </row>
     <row r="787">
       <c r="A787" t="inlineStr" s="2">
@@ -22083,12 +22087,12 @@
       </c>
       <c r="B787" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">criado_por</t>
+          <t xml:space="preserve">texto_extraido</t>
         </is>
       </c>
       <c r="C787" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D787" t="inlineStr" s="2">
@@ -22097,11 +22101,7 @@
         </is>
       </c>
       <c r="E787" s="2"/>
-      <c r="F787" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">users</t>
-        </is>
-      </c>
+      <c r="F787" s="2"/>
       <c r="G787" s="2"/>
     </row>
     <row r="788">
@@ -22112,12 +22112,12 @@
       </c>
       <c r="B788" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autor_nome</t>
+          <t xml:space="preserve">anexos</t>
         </is>
       </c>
       <c r="C788" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="D788" t="inlineStr" s="2">
@@ -22127,7 +22127,11 @@
       </c>
       <c r="E788" s="2"/>
       <c r="F788" s="2"/>
-      <c r="G788" s="2"/>
+      <c r="G788" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
+        </is>
+      </c>
     </row>
     <row r="789">
       <c r="A789" t="inlineStr" s="2">
@@ -22137,12 +22141,12 @@
       </c>
       <c r="B789" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tags</t>
+          <t xml:space="preserve">criado_por</t>
         </is>
       </c>
       <c r="C789" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D789" t="inlineStr" s="2">
@@ -22151,7 +22155,11 @@
         </is>
       </c>
       <c r="E789" s="2"/>
-      <c r="F789" s="2"/>
+      <c r="F789" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">users</t>
+        </is>
+      </c>
       <c r="G789" s="2"/>
     </row>
     <row r="790">
@@ -22162,12 +22170,12 @@
       </c>
       <c r="B790" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">autor_nome</t>
         </is>
       </c>
       <c r="C790" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D790" t="inlineStr" s="2">
@@ -22177,11 +22185,7 @@
       </c>
       <c r="E790" s="2"/>
       <c r="F790" s="2"/>
-      <c r="G790" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G790" s="2"/>
     </row>
     <row r="791">
       <c r="A791" t="inlineStr" s="2">
@@ -22191,12 +22195,12 @@
       </c>
       <c r="B791" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">tags</t>
         </is>
       </c>
       <c r="C791" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D791" t="inlineStr" s="2">
@@ -22206,69 +22210,65 @@
       </c>
       <c r="E791" s="2"/>
       <c r="F791" s="2"/>
-      <c r="G791" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G791" s="2"/>
     </row>
     <row r="792">
       <c r="A792" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contratos_usinas</t>
+          <t xml:space="preserve">knowledge_articles</t>
         </is>
       </c>
       <c r="B792" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contrato_id</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C792" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D792" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E792" s="2"/>
-      <c r="F792" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">contratos_om</t>
-        </is>
-      </c>
-      <c r="G792" s="2"/>
+      <c r="F792" s="2"/>
+      <c r="G792" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="793">
       <c r="A793" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contratos_usinas</t>
+          <t xml:space="preserve">knowledge_articles</t>
         </is>
       </c>
       <c r="B793" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">usina_id</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C793" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D793" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E793" s="2"/>
-      <c r="F793" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">usinas</t>
-        </is>
-      </c>
-      <c r="G793" s="2"/>
+      <c r="F793" s="2"/>
+      <c r="G793" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="794">
       <c r="A794" t="inlineStr" s="2">
@@ -22278,25 +22278,25 @@
       </c>
       <c r="B794" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ativo</t>
+          <t xml:space="preserve">contrato_id</t>
         </is>
       </c>
       <c r="C794" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D794" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E794" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
-      <c r="F794" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E794" s="2"/>
+      <c r="F794" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contratos_om</t>
+        </is>
+      </c>
       <c r="G794" s="2"/>
     </row>
     <row r="795">
@@ -22307,21 +22307,25 @@
       </c>
       <c r="B795" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_vinculo</t>
+          <t xml:space="preserve">usina_id</t>
         </is>
       </c>
       <c r="C795" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D795" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E795" s="2"/>
-      <c r="F795" s="2"/>
+      <c r="F795" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usinas</t>
+        </is>
+      </c>
       <c r="G795" s="2"/>
     </row>
     <row r="796">
@@ -22332,12 +22336,12 @@
       </c>
       <c r="B796" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_desvinculo</t>
+          <t xml:space="preserve">ativo</t>
         </is>
       </c>
       <c r="C796" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D796" t="inlineStr" s="2">
@@ -22345,7 +22349,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E796" s="2"/>
+      <c r="E796" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F796" s="2"/>
       <c r="G796" s="2"/>
     </row>
@@ -22357,12 +22365,12 @@
       </c>
       <c r="B797" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">observacoes</t>
+          <t xml:space="preserve">data_vinculo</t>
         </is>
       </c>
       <c r="C797" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D797" t="inlineStr" s="2">
@@ -22382,12 +22390,12 @@
       </c>
       <c r="B798" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">data_desvinculo</t>
         </is>
       </c>
       <c r="C798" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D798" t="inlineStr" s="2">
@@ -22397,11 +22405,7 @@
       </c>
       <c r="E798" s="2"/>
       <c r="F798" s="2"/>
-      <c r="G798" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G798" s="2"/>
     </row>
     <row r="799">
       <c r="A799" t="inlineStr" s="2">
@@ -22411,12 +22415,12 @@
       </c>
       <c r="B799" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">observacoes</t>
         </is>
       </c>
       <c r="C799" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D799" t="inlineStr" s="2">
@@ -22426,7 +22430,61 @@
       </c>
       <c r="E799" s="2"/>
       <c r="F799" s="2"/>
-      <c r="G799" t="inlineStr" s="2">
+      <c r="G799" s="2"/>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contratos_usinas</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">created</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D800" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E800" s="2"/>
+      <c r="F800" s="2"/>
+      <c r="G800" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contratos_usinas</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">updated</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D801" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E801" s="2"/>
+      <c r="F801" s="2"/>
+      <c r="G801" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
         </is>

</xml_diff>

<commit_message>
feat: cadastro aditivo de ativos das usinas com acompanhamento de garantias e integracao na ficha da usina
</commit_message>
<xml_diff>
--- a/public/schema-delfos-solar.xlsx
+++ b/public/schema-delfos-solar.xlsx
@@ -1328,22 +1328,50 @@
     <row r="45">
       <c r="A45" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TOTAL: 43 coleções</t>
+          <t xml:space="preserve">ativos</t>
         </is>
       </c>
       <c r="B45" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Coleção de dados do sistema.</t>
+        </is>
+      </c>
+      <c r="C45" s="2">
+        <v>13</v>
+      </c>
+      <c r="D45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">base</t>
+        </is>
+      </c>
+      <c r="E45" s="2">
+        <v>2</v>
+      </c>
+      <c r="F45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Regras RLS configuradas (autenticado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TOTAL: 44 coleções</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Total geral de campos e relacionamentos no banco PocketBase Delfos Solar</t>
         </is>
       </c>
-      <c r="C45" s="2">
-        <v>800</v>
-      </c>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2">
-        <v>53</v>
-      </c>
-      <c r="F45" s="2"/>
+      <c r="C46" s="2">
+        <v>813</v>
+      </c>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2">
+        <v>55</v>
+      </c>
+      <c r="F46" s="2"/>
     </row>
   </sheetData>
 </worksheet>
@@ -22490,6 +22518,355 @@
         </is>
       </c>
     </row>
+    <row r="802">
+      <c r="A802" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativos</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usina_id</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">relation</t>
+        </is>
+      </c>
+      <c r="D802" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E802" s="2"/>
+      <c r="F802" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usinas</t>
+        </is>
+      </c>
+      <c r="G802" s="2"/>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativos</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">tipo</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">select</t>
+        </is>
+      </c>
+      <c r="D803" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E803" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">inversor | placa_solar | bateria | string_box | outros</t>
+        </is>
+      </c>
+      <c r="F803" s="2"/>
+      <c r="G803" s="2"/>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativos</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">tipo_outro_descricao</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D804" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E804" s="2"/>
+      <c r="F804" s="2"/>
+      <c r="G804" s="2"/>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativos</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">fabricante</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D805" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E805" s="2"/>
+      <c r="F805" s="2"/>
+      <c r="G805" s="2"/>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativos</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">modelo</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D806" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E806" s="2"/>
+      <c r="F806" s="2"/>
+      <c r="G806" s="2"/>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativos</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">numero_serie</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D807" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E807" s="2"/>
+      <c r="F807" s="2"/>
+      <c r="G807" s="2"/>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativos</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">data_instalacao</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">date</t>
+        </is>
+      </c>
+      <c r="D808" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E808" s="2"/>
+      <c r="F808" s="2"/>
+      <c r="G808" s="2"/>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativos</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">data_fim_garantia</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">date</t>
+        </is>
+      </c>
+      <c r="D809" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E809" s="2"/>
+      <c r="F809" s="2"/>
+      <c r="G809" s="2"/>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativos</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">responsavel_id</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">relation</t>
+        </is>
+      </c>
+      <c r="D810" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E810" s="2"/>
+      <c r="F810" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">users</t>
+        </is>
+      </c>
+      <c r="G810" s="2"/>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativos</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">observacoes</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D811" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E811" s="2"/>
+      <c r="F811" s="2"/>
+      <c r="G811" s="2"/>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativos</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">status_operacional</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">select</t>
+        </is>
+      </c>
+      <c r="D812" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E812" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">operacional | em_alerta | manutencao | desativado</t>
+        </is>
+      </c>
+      <c r="F812" s="2"/>
+      <c r="G812" s="2"/>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativos</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">created</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D813" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E813" s="2"/>
+      <c r="F813" s="2"/>
+      <c r="G813" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativos</t>
+        </is>
+      </c>
+      <c r="B814" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">updated</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D814" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E814" s="2"/>
+      <c r="F814" s="2"/>
+      <c r="G814" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -24233,6 +24610,70 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativos</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usina_id</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usinas</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Vínculo da atividade à usina fotovoltaica correspondente</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativos</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">responsavel_id</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">users</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Relaciona o registro de ativos com users</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: importar/copiar inversores de cliente_inversores para ativos com idempotencia e relatorio
</commit_message>
<xml_diff>
--- a/public/schema-delfos-solar.xlsx
+++ b/public/schema-delfos-solar.xlsx
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="C45" s="2">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D45" t="inlineStr" s="2">
         <is>
@@ -1365,7 +1365,7 @@
         </is>
       </c>
       <c r="C46" s="2">
-        <v>818</v>
+        <v>820</v>
       </c>
       <c r="D46" s="2"/>
       <c r="E46" s="2">
@@ -22661,7 +22661,7 @@
       </c>
       <c r="D807" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E807" s="2"/>
@@ -22991,6 +22991,56 @@
           <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
         </is>
       </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativos</t>
+        </is>
+      </c>
+      <c r="B820" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">chave_importacao</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D820" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E820" s="2"/>
+      <c r="F820" s="2"/>
+      <c r="G820" s="2"/>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativos</t>
+        </is>
+      </c>
+      <c r="B821" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">cliente_inversor_id</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D821" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E821" s="2"/>
+      <c r="F821" s="2"/>
+      <c r="G821" s="2"/>
     </row>
   </sheetData>
 </worksheet>
@@ -24753,7 +24803,7 @@
       </c>
       <c r="D55" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E55" t="inlineStr" s="2">

</xml_diff>

<commit_message>
feat: reorganiza cadastro em area unica de contatos com relacao N:N e regra autoritativa do WhatsApp
</commit_message>
<xml_diff>
--- a/public/schema-delfos-solar.xlsx
+++ b/public/schema-delfos-solar.xlsx
@@ -1356,22 +1356,50 @@
     <row r="46">
       <c r="A46" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TOTAL: 44 coleções</t>
+          <t xml:space="preserve">contatos</t>
         </is>
       </c>
       <c r="B46" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Coleção de dados do sistema.</t>
+        </is>
+      </c>
+      <c r="C46" s="2">
+        <v>13</v>
+      </c>
+      <c r="D46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">base</t>
+        </is>
+      </c>
+      <c r="E46" s="2">
+        <v>2</v>
+      </c>
+      <c r="F46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Regras RLS configuradas (autenticado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TOTAL: 45 coleções</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Total geral de campos e relacionamentos no banco PocketBase Delfos Solar</t>
         </is>
       </c>
-      <c r="C46" s="2">
-        <v>820</v>
-      </c>
-      <c r="D46" s="2"/>
-      <c r="E46" s="2">
-        <v>55</v>
-      </c>
-      <c r="F46" s="2"/>
+      <c r="C47" s="2">
+        <v>833</v>
+      </c>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2">
+        <v>57</v>
+      </c>
+      <c r="F47" s="2"/>
     </row>
   </sheetData>
 </worksheet>
@@ -23042,6 +23070,351 @@
       <c r="F821" s="2"/>
       <c r="G821" s="2"/>
     </row>
+    <row r="822">
+      <c r="A822" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contatos</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">nome</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E822" s="2"/>
+      <c r="F822" s="2"/>
+      <c r="G822" s="2"/>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contatos</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">telefone</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D823" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E823" s="2"/>
+      <c r="F823" s="2"/>
+      <c r="G823" s="2"/>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contatos</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">whatsapp</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D824" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E824" s="2"/>
+      <c r="F824" s="2"/>
+      <c r="G824" s="2"/>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contatos</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">email</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">email</t>
+        </is>
+      </c>
+      <c r="D825" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E825" s="2"/>
+      <c r="F825" s="2"/>
+      <c r="G825" s="2"/>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contatos</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">papel</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">select</t>
+        </is>
+      </c>
+      <c r="D826" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E826" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">cliente | lead | fornecedor | tecnico | parceiro | familiar | responsavel | financeiro | outro</t>
+        </is>
+      </c>
+      <c r="F826" s="2"/>
+      <c r="G826" s="2"/>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contatos</t>
+        </is>
+      </c>
+      <c r="B827" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">cargo</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D827" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E827" s="2"/>
+      <c r="F827" s="2"/>
+      <c r="G827" s="2"/>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contatos</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">observacoes</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D828" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E828" s="2"/>
+      <c r="F828" s="2"/>
+      <c r="G828" s="2"/>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contatos</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes_vinculados</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">relation</t>
+        </is>
+      </c>
+      <c r="D829" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E829" s="2"/>
+      <c r="F829" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
+      <c r="G829" s="2"/>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contatos</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios_vinculados</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">relation</t>
+        </is>
+      </c>
+      <c r="D830" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E830" s="2"/>
+      <c r="F830" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="G830" s="2"/>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contatos</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">conversa_id</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D831" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E831" s="2"/>
+      <c r="F831" s="2"/>
+      <c r="G831" s="2"/>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contatos</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">origem_registro</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D832" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E832" s="2"/>
+      <c r="F832" s="2"/>
+      <c r="G832" s="2"/>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contatos</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">created</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D833" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E833" s="2"/>
+      <c r="F833" s="2"/>
+      <c r="G833" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contatos</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">updated</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D834" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E834" s="2"/>
+      <c r="F834" s="2"/>
+      <c r="G834" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -24849,6 +25222,70 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contatos</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes_vinculados</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Relaciona o registro de contatos com clientes</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contatos</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios_vinculados</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Relaciona o registro de contatos com negocios</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: gestão de equipamentos como ativos da usina e importação inteligente (v0.0.747)
</commit_message>
<xml_diff>
--- a/public/schema-delfos-solar.xlsx
+++ b/public/schema-delfos-solar.xlsx
@@ -1057,7 +1057,7 @@
         </is>
       </c>
       <c r="C35" s="2">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D35" t="inlineStr" s="2">
         <is>
@@ -1065,7 +1065,7 @@
         </is>
       </c>
       <c r="E35" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F35" t="inlineStr" s="2">
         <is>
@@ -1384,22 +1384,50 @@
     <row r="47">
       <c r="A47" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TOTAL: 45 coleções</t>
+          <t xml:space="preserve">usina_equipamentos</t>
         </is>
       </c>
       <c r="B47" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Coleção de dados do sistema.</t>
+        </is>
+      </c>
+      <c r="C47" s="2">
+        <v>7</v>
+      </c>
+      <c r="D47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">base</t>
+        </is>
+      </c>
+      <c r="E47" s="2">
+        <v>2</v>
+      </c>
+      <c r="F47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Regras RLS configuradas (autenticado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TOTAL: 46 coleções</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Total geral de campos e relacionamentos no banco PocketBase Delfos Solar</t>
         </is>
       </c>
-      <c r="C47" s="2">
-        <v>847</v>
-      </c>
-      <c r="D47" s="2"/>
-      <c r="E47" s="2">
-        <v>57</v>
-      </c>
-      <c r="F47" s="2"/>
+      <c r="C48" s="2">
+        <v>858</v>
+      </c>
+      <c r="D48" s="2"/>
+      <c r="E48" s="2">
+        <v>60</v>
+      </c>
+      <c r="F48" s="2"/>
     </row>
   </sheetData>
 </worksheet>
@@ -19912,7 +19940,7 @@
       </c>
       <c r="E705" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">inversor | modulo_fv</t>
+          <t xml:space="preserve">inversor | modulo_fv | outro</t>
         </is>
       </c>
       <c r="F705" s="2"/>
@@ -20162,22 +20190,22 @@
     <row r="715">
       <c r="A715" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">parametros_tarifarios</t>
+          <t xml:space="preserve">equipamentos</t>
         </is>
       </c>
       <c r="B715" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ano</t>
+          <t xml:space="preserve">datasheet_url</t>
         </is>
       </c>
       <c r="C715" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">url</t>
         </is>
       </c>
       <c r="D715" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E715" s="2"/>
@@ -20187,46 +20215,42 @@
     <row r="716">
       <c r="A716" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">parametros_tarifarios</t>
+          <t xml:space="preserve">equipamentos</t>
         </is>
       </c>
       <c r="B716" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">classe</t>
+          <t xml:space="preserve">datalogger_url</t>
         </is>
       </c>
       <c r="C716" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">url</t>
         </is>
       </c>
       <c r="D716" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E716" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">residencial | comercial</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E716" s="2"/>
       <c r="F716" s="2"/>
       <c r="G716" s="2"/>
     </row>
     <row r="717">
       <c r="A717" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">parametros_tarifarios</t>
+          <t xml:space="preserve">equipamentos</t>
         </is>
       </c>
       <c r="B717" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tarifa</t>
+          <t xml:space="preserve">fornecedor_id</t>
         </is>
       </c>
       <c r="C717" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D717" t="inlineStr" s="2">
@@ -20235,23 +20259,27 @@
         </is>
       </c>
       <c r="E717" s="2"/>
-      <c r="F717" s="2"/>
+      <c r="F717" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">fornecedores</t>
+        </is>
+      </c>
       <c r="G717" s="2"/>
     </row>
     <row r="718">
       <c r="A718" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">parametros_tarifarios</t>
+          <t xml:space="preserve">equipamentos</t>
         </is>
       </c>
       <c r="B718" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fio_b</t>
+          <t xml:space="preserve">telefone_suporte_fornecedor</t>
         </is>
       </c>
       <c r="C718" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D718" t="inlineStr" s="2">
@@ -20271,7 +20299,7 @@
       </c>
       <c r="B719" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fs</t>
+          <t xml:space="preserve">ano</t>
         </is>
       </c>
       <c r="C719" t="inlineStr" s="2">
@@ -20281,7 +20309,7 @@
       </c>
       <c r="D719" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E719" s="2"/>
@@ -20296,20 +20324,24 @@
       </c>
       <c r="B720" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gd_eco_liquida</t>
+          <t xml:space="preserve">classe</t>
         </is>
       </c>
       <c r="C720" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D720" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E720" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">residencial | comercial</t>
+        </is>
+      </c>
       <c r="F720" s="2"/>
       <c r="G720" s="2"/>
     </row>
@@ -20321,12 +20353,12 @@
       </c>
       <c r="B721" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">tarifa</t>
         </is>
       </c>
       <c r="C721" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D721" t="inlineStr" s="2">
@@ -20336,11 +20368,7 @@
       </c>
       <c r="E721" s="2"/>
       <c r="F721" s="2"/>
-      <c r="G721" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G721" s="2"/>
     </row>
     <row r="722">
       <c r="A722" t="inlineStr" s="2">
@@ -20350,12 +20378,12 @@
       </c>
       <c r="B722" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">fio_b</t>
         </is>
       </c>
       <c r="C722" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D722" t="inlineStr" s="2">
@@ -20365,31 +20393,27 @@
       </c>
       <c r="E722" s="2"/>
       <c r="F722" s="2"/>
-      <c r="G722" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G722" s="2"/>
     </row>
     <row r="723">
       <c r="A723" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">parametros_tarifarios</t>
         </is>
       </c>
       <c r="B723" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">nome</t>
+          <t xml:space="preserve">fs</t>
         </is>
       </c>
       <c r="C723" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D723" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E723" s="2"/>
@@ -20399,46 +20423,42 @@
     <row r="724">
       <c r="A724" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">parametros_tarifarios</t>
         </is>
       </c>
       <c r="B724" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gatilho</t>
+          <t xml:space="preserve">gd_eco_liquida</t>
         </is>
       </c>
       <c r="C724" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D724" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E724" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">status_mudou | instalacao_concluida | atividade_concluida | data_especifica | dias_apos_evento</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E724" s="2"/>
       <c r="F724" s="2"/>
       <c r="G724" s="2"/>
     </row>
     <row r="725">
       <c r="A725" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">parametros_tarifarios</t>
         </is>
       </c>
       <c r="B725" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">configuracao_gatilho</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C725" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D725" t="inlineStr" s="2">
@@ -20450,38 +20470,38 @@
       <c r="F725" s="2"/>
       <c r="G725" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="726">
       <c r="A726" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">parametros_tarifarios</t>
         </is>
       </c>
       <c r="B726" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">acao</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C726" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D726" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E726" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">criar_atividade | enviar_whatsapp | enviar_email | mudar_status</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E726" s="2"/>
       <c r="F726" s="2"/>
-      <c r="G726" s="2"/>
+      <c r="G726" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="727">
       <c r="A727" t="inlineStr" s="2">
@@ -20491,26 +20511,22 @@
       </c>
       <c r="B727" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">configuracao_acao</t>
+          <t xml:space="preserve">nome</t>
         </is>
       </c>
       <c r="C727" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D727" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E727" s="2"/>
       <c r="F727" s="2"/>
-      <c r="G727" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="G727" s="2"/>
     </row>
     <row r="728">
       <c r="A728" t="inlineStr" s="2">
@@ -20520,7 +20536,7 @@
       </c>
       <c r="B728" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">destino</t>
+          <t xml:space="preserve">gatilho</t>
         </is>
       </c>
       <c r="C728" t="inlineStr" s="2">
@@ -20535,7 +20551,7 @@
       </c>
       <c r="E728" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_evento | responsavel_empresa | cliente_especifico</t>
+          <t xml:space="preserve">status_mudou | instalacao_concluida | atividade_concluida | data_especifica | dias_apos_evento</t>
         </is>
       </c>
       <c r="F728" s="2"/>
@@ -20549,12 +20565,12 @@
       </c>
       <c r="B729" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_especifico_id</t>
+          <t xml:space="preserve">configuracao_gatilho</t>
         </is>
       </c>
       <c r="C729" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D729" t="inlineStr" s="2">
@@ -20563,12 +20579,12 @@
         </is>
       </c>
       <c r="E729" s="2"/>
-      <c r="F729" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
-      <c r="G729" s="2"/>
+      <c r="F729" s="2"/>
+      <c r="G729" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Estrutura JSON livre</t>
+        </is>
+      </c>
     </row>
     <row r="730">
       <c r="A730" t="inlineStr" s="2">
@@ -20578,22 +20594,22 @@
       </c>
       <c r="B730" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ativa</t>
+          <t xml:space="preserve">acao</t>
         </is>
       </c>
       <c r="C730" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D730" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E730" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">true / false</t>
+          <t xml:space="preserve">criar_atividade | enviar_whatsapp | enviar_email | mudar_status</t>
         </is>
       </c>
       <c r="F730" s="2"/>
@@ -20607,12 +20623,12 @@
       </c>
       <c r="B731" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">configuracao_acao</t>
         </is>
       </c>
       <c r="C731" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D731" t="inlineStr" s="2">
@@ -20624,7 +20640,7 @@
       <c r="F731" s="2"/>
       <c r="G731" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
+          <t xml:space="preserve">Estrutura JSON livre</t>
         </is>
       </c>
     </row>
@@ -20636,36 +20652,36 @@
       </c>
       <c r="B732" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">destino</t>
         </is>
       </c>
       <c r="C732" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D732" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E732" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E732" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">cliente_evento | responsavel_empresa | cliente_especifico</t>
+        </is>
+      </c>
       <c r="F732" s="2"/>
-      <c r="G732" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G732" s="2"/>
     </row>
     <row r="733">
       <c r="A733" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes_execucoes</t>
+          <t xml:space="preserve">automacoes</t>
         </is>
       </c>
       <c r="B733" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacao</t>
+          <t xml:space="preserve">cliente_especifico_id</t>
         </is>
       </c>
       <c r="C733" t="inlineStr" s="2">
@@ -20675,13 +20691,13 @@
       </c>
       <c r="D733" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E733" s="2"/>
       <c r="F733" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">clientes</t>
         </is>
       </c>
       <c r="G733" s="2"/>
@@ -20689,42 +20705,46 @@
     <row r="734">
       <c r="A734" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes_execucoes</t>
+          <t xml:space="preserve">automacoes</t>
         </is>
       </c>
       <c r="B734" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_execucao</t>
+          <t xml:space="preserve">ativa</t>
         </is>
       </c>
       <c r="C734" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D734" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E734" s="2"/>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E734" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F734" s="2"/>
       <c r="G734" s="2"/>
     </row>
     <row r="735">
       <c r="A735" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes_execucoes</t>
+          <t xml:space="preserve">automacoes</t>
         </is>
       </c>
       <c r="B735" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">sucesso</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C735" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D735" t="inlineStr" s="2">
@@ -20732,28 +20752,28 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E735" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E735" s="2"/>
       <c r="F735" s="2"/>
-      <c r="G735" s="2"/>
+      <c r="G735" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="736">
       <c r="A736" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes_execucoes</t>
+          <t xml:space="preserve">automacoes</t>
         </is>
       </c>
       <c r="B736" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mensagem</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C736" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D736" t="inlineStr" s="2">
@@ -20763,7 +20783,11 @@
       </c>
       <c r="E736" s="2"/>
       <c r="F736" s="2"/>
-      <c r="G736" s="2"/>
+      <c r="G736" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="737">
       <c r="A737" t="inlineStr" s="2">
@@ -20773,21 +20797,25 @@
       </c>
       <c r="B737" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">referencia_registro</t>
+          <t xml:space="preserve">automacao</t>
         </is>
       </c>
       <c r="C737" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D737" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E737" s="2"/>
-      <c r="F737" s="2"/>
+      <c r="F737" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">automacoes</t>
+        </is>
+      </c>
       <c r="G737" s="2"/>
     </row>
     <row r="738">
@@ -20798,25 +20826,21 @@
       </c>
       <c r="B738" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente</t>
+          <t xml:space="preserve">data_execucao</t>
         </is>
       </c>
       <c r="C738" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D738" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E738" s="2"/>
-      <c r="F738" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+      <c r="F738" s="2"/>
       <c r="G738" s="2"/>
     </row>
     <row r="739">
@@ -20827,12 +20851,12 @@
       </c>
       <c r="B739" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">dados_execucao</t>
+          <t xml:space="preserve">sucesso</t>
         </is>
       </c>
       <c r="C739" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D739" t="inlineStr" s="2">
@@ -20840,13 +20864,13 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E739" s="2"/>
+      <c r="E739" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F739" s="2"/>
-      <c r="G739" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="G739" s="2"/>
     </row>
     <row r="740">
       <c r="A740" t="inlineStr" s="2">
@@ -20856,12 +20880,12 @@
       </c>
       <c r="B740" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">mensagem</t>
         </is>
       </c>
       <c r="C740" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D740" t="inlineStr" s="2">
@@ -20871,11 +20895,7 @@
       </c>
       <c r="E740" s="2"/>
       <c r="F740" s="2"/>
-      <c r="G740" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G740" s="2"/>
     </row>
     <row r="741">
       <c r="A741" t="inlineStr" s="2">
@@ -20885,12 +20905,12 @@
       </c>
       <c r="B741" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">referencia_registro</t>
         </is>
       </c>
       <c r="C741" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D741" t="inlineStr" s="2">
@@ -20900,80 +20920,80 @@
       </c>
       <c r="E741" s="2"/>
       <c r="F741" s="2"/>
-      <c r="G741" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G741" s="2"/>
     </row>
     <row r="742">
       <c r="A742" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">automacoes_execucoes</t>
         </is>
       </c>
       <c r="B742" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo</t>
+          <t xml:space="preserve">cliente</t>
         </is>
       </c>
       <c r="C742" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D742" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E742" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">atividade_atrasada | lembrete | sistema</t>
-        </is>
-      </c>
-      <c r="F742" s="2"/>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E742" s="2"/>
+      <c r="F742" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G742" s="2"/>
     </row>
     <row r="743">
       <c r="A743" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">automacoes_execucoes</t>
         </is>
       </c>
       <c r="B743" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">dados_execucao</t>
         </is>
       </c>
       <c r="C743" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D743" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E743" s="2"/>
       <c r="F743" s="2"/>
-      <c r="G743" s="2"/>
+      <c r="G743" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Estrutura JSON livre</t>
+        </is>
+      </c>
     </row>
     <row r="744">
       <c r="A744" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">automacoes_execucoes</t>
         </is>
       </c>
       <c r="B744" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mensagem</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C744" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D744" t="inlineStr" s="2">
@@ -20983,22 +21003,26 @@
       </c>
       <c r="E744" s="2"/>
       <c r="F744" s="2"/>
-      <c r="G744" s="2"/>
+      <c r="G744" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="745">
       <c r="A745" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">automacoes_execucoes</t>
         </is>
       </c>
       <c r="B745" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">atividade_id</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C745" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D745" t="inlineStr" s="2">
@@ -21007,12 +21031,12 @@
         </is>
       </c>
       <c r="E745" s="2"/>
-      <c r="F745" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">atividades</t>
-        </is>
-      </c>
-      <c r="G745" s="2"/>
+      <c r="F745" s="2"/>
+      <c r="G745" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="746">
       <c r="A746" t="inlineStr" s="2">
@@ -21022,25 +21046,25 @@
       </c>
       <c r="B746" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_id</t>
+          <t xml:space="preserve">tipo</t>
         </is>
       </c>
       <c r="C746" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D746" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E746" s="2"/>
-      <c r="F746" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E746" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">atividade_atrasada | lembrete | sistema</t>
+        </is>
+      </c>
+      <c r="F746" s="2"/>
       <c r="G746" s="2"/>
     </row>
     <row r="747">
@@ -21051,7 +21075,7 @@
       </c>
       <c r="B747" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_nome</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C747" t="inlineStr" s="2">
@@ -21061,7 +21085,7 @@
       </c>
       <c r="D747" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E747" s="2"/>
@@ -21076,12 +21100,12 @@
       </c>
       <c r="B748" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_prevista</t>
+          <t xml:space="preserve">mensagem</t>
         </is>
       </c>
       <c r="C748" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D748" t="inlineStr" s="2">
@@ -21101,12 +21125,12 @@
       </c>
       <c r="B749" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">dias_atraso</t>
+          <t xml:space="preserve">atividade_id</t>
         </is>
       </c>
       <c r="C749" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D749" t="inlineStr" s="2">
@@ -21115,7 +21139,11 @@
         </is>
       </c>
       <c r="E749" s="2"/>
-      <c r="F749" s="2"/>
+      <c r="F749" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">atividades</t>
+        </is>
+      </c>
       <c r="G749" s="2"/>
     </row>
     <row r="750">
@@ -21126,12 +21154,12 @@
       </c>
       <c r="B750" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">lida</t>
+          <t xml:space="preserve">cliente_id</t>
         </is>
       </c>
       <c r="C750" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D750" t="inlineStr" s="2">
@@ -21139,12 +21167,12 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E750" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
-      <c r="F750" s="2"/>
+      <c r="E750" s="2"/>
+      <c r="F750" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G750" s="2"/>
     </row>
     <row r="751">
@@ -21155,12 +21183,12 @@
       </c>
       <c r="B751" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">lida_em</t>
+          <t xml:space="preserve">cliente_nome</t>
         </is>
       </c>
       <c r="C751" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D751" t="inlineStr" s="2">
@@ -21180,24 +21208,20 @@
       </c>
       <c r="B752" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">data_prevista</t>
         </is>
       </c>
       <c r="C752" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D752" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E752" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">ativa | resolvida | arquivada</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E752" s="2"/>
       <c r="F752" s="2"/>
       <c r="G752" s="2"/>
     </row>
@@ -21209,12 +21233,12 @@
       </c>
       <c r="B753" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">resolvida_em</t>
+          <t xml:space="preserve">dias_atraso</t>
         </is>
       </c>
       <c r="C753" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D753" t="inlineStr" s="2">
@@ -21234,12 +21258,12 @@
       </c>
       <c r="B754" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">lida</t>
         </is>
       </c>
       <c r="C754" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D754" t="inlineStr" s="2">
@@ -21247,13 +21271,13 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E754" s="2"/>
+      <c r="E754" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F754" s="2"/>
-      <c r="G754" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G754" s="2"/>
     </row>
     <row r="755">
       <c r="A755" t="inlineStr" s="2">
@@ -21263,12 +21287,12 @@
       </c>
       <c r="B755" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">lida_em</t>
         </is>
       </c>
       <c r="C755" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D755" t="inlineStr" s="2">
@@ -21278,26 +21302,22 @@
       </c>
       <c r="E755" s="2"/>
       <c r="F755" s="2"/>
-      <c r="G755" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G755" s="2"/>
     </row>
     <row r="756">
       <c r="A756" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">notificacoes_internas</t>
         </is>
       </c>
       <c r="B756" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_id</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="C756" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D756" t="inlineStr" s="2">
@@ -21305,28 +21325,28 @@
           <t xml:space="preserve">Sim</t>
         </is>
       </c>
-      <c r="E756" s="2"/>
-      <c r="F756" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+      <c r="E756" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativa | resolvida | arquivada</t>
+        </is>
+      </c>
+      <c r="F756" s="2"/>
       <c r="G756" s="2"/>
     </row>
     <row r="757">
       <c r="A757" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">notificacoes_internas</t>
         </is>
       </c>
       <c r="B757" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_negocio</t>
+          <t xml:space="preserve">resolvida_em</t>
         </is>
       </c>
       <c r="C757" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D757" t="inlineStr" s="2">
@@ -21334,28 +21354,24 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E757" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">venda usina | bateria | expansão | renovação | serviço | venda bateria</t>
-        </is>
-      </c>
+      <c r="E757" s="2"/>
       <c r="F757" s="2"/>
       <c r="G757" s="2"/>
     </row>
     <row r="758">
       <c r="A758" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">notificacoes_internas</t>
         </is>
       </c>
       <c r="B758" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">valor_estimado</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C758" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D758" t="inlineStr" s="2">
@@ -21365,22 +21381,26 @@
       </c>
       <c r="E758" s="2"/>
       <c r="F758" s="2"/>
-      <c r="G758" s="2"/>
+      <c r="G758" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="759">
       <c r="A759" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">notificacoes_internas</t>
         </is>
       </c>
       <c r="B759" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">valor_final</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C759" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D759" t="inlineStr" s="2">
@@ -21390,7 +21410,11 @@
       </c>
       <c r="E759" s="2"/>
       <c r="F759" s="2"/>
-      <c r="G759" s="2"/>
+      <c r="G759" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="760">
       <c r="A760" t="inlineStr" s="2">
@@ -21400,25 +21424,25 @@
       </c>
       <c r="B760" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">etapa_funil</t>
+          <t xml:space="preserve">cliente_id</t>
         </is>
       </c>
       <c r="C760" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D760" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E760" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">novo lead | qualificado | proposta enviada | negociação | contrato assinado</t>
-        </is>
-      </c>
-      <c r="F760" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E760" s="2"/>
+      <c r="F760" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G760" s="2"/>
     </row>
     <row r="761">
@@ -21429,12 +21453,12 @@
       </c>
       <c r="B761" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">probabilidade</t>
+          <t xml:space="preserve">tipo_negocio</t>
         </is>
       </c>
       <c r="C761" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D761" t="inlineStr" s="2">
@@ -21442,7 +21466,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E761" s="2"/>
+      <c r="E761" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">venda usina | bateria | expansão | renovação | serviço | venda bateria</t>
+        </is>
+      </c>
       <c r="F761" s="2"/>
       <c r="G761" s="2"/>
     </row>
@@ -21454,12 +21482,12 @@
       </c>
       <c r="B762" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_previsao_fechamento</t>
+          <t xml:space="preserve">valor_estimado</t>
         </is>
       </c>
       <c r="C762" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D762" t="inlineStr" s="2">
@@ -21479,12 +21507,12 @@
       </c>
       <c r="B763" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_fechamento</t>
+          <t xml:space="preserve">valor_final</t>
         </is>
       </c>
       <c r="C763" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D763" t="inlineStr" s="2">
@@ -21504,7 +21532,7 @@
       </c>
       <c r="B764" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">etapa_funil</t>
         </is>
       </c>
       <c r="C764" t="inlineStr" s="2">
@@ -21519,7 +21547,7 @@
       </c>
       <c r="E764" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">em andamento | ganho | perdido</t>
+          <t xml:space="preserve">novo lead | qualificado | proposta enviada | negociação | contrato assinado</t>
         </is>
       </c>
       <c r="F764" s="2"/>
@@ -21533,12 +21561,12 @@
       </c>
       <c r="B765" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">motivo_perda</t>
+          <t xml:space="preserve">probabilidade</t>
         </is>
       </c>
       <c r="C765" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D765" t="inlineStr" s="2">
@@ -21558,12 +21586,12 @@
       </c>
       <c r="B766" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">reabertura</t>
+          <t xml:space="preserve">data_previsao_fechamento</t>
         </is>
       </c>
       <c r="C766" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D766" t="inlineStr" s="2">
@@ -21571,11 +21599,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E766" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E766" s="2"/>
       <c r="F766" s="2"/>
       <c r="G766" s="2"/>
     </row>
@@ -21587,12 +21611,12 @@
       </c>
       <c r="B767" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">motivo_reabertura</t>
+          <t xml:space="preserve">data_fechamento</t>
         </is>
       </c>
       <c r="C767" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D767" t="inlineStr" s="2">
@@ -21612,12 +21636,12 @@
       </c>
       <c r="B768" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">condicao_pagamento</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="C768" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D768" t="inlineStr" s="2">
@@ -21625,7 +21649,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E768" s="2"/>
+      <c r="E768" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">em andamento | ganho | perdido</t>
+        </is>
+      </c>
       <c r="F768" s="2"/>
       <c r="G768" s="2"/>
     </row>
@@ -21637,12 +21665,12 @@
       </c>
       <c r="B769" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">motivo_perda</t>
         </is>
       </c>
       <c r="C769" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D769" t="inlineStr" s="2">
@@ -21652,11 +21680,7 @@
       </c>
       <c r="E769" s="2"/>
       <c r="F769" s="2"/>
-      <c r="G769" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G769" s="2"/>
     </row>
     <row r="770">
       <c r="A770" t="inlineStr" s="2">
@@ -21666,12 +21690,12 @@
       </c>
       <c r="B770" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">reabertura</t>
         </is>
       </c>
       <c r="C770" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D770" t="inlineStr" s="2">
@@ -21679,13 +21703,13 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E770" s="2"/>
+      <c r="E770" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F770" s="2"/>
-      <c r="G770" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G770" s="2"/>
     </row>
     <row r="771">
       <c r="A771" t="inlineStr" s="2">
@@ -21695,12 +21719,12 @@
       </c>
       <c r="B771" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_venda</t>
+          <t xml:space="preserve">motivo_reabertura</t>
         </is>
       </c>
       <c r="C771" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D771" t="inlineStr" s="2">
@@ -21708,11 +21732,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E771" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Energia Solar | O&amp;M (Operação e Manutenção) | Baterias | Carregadores Veículos Elétricos</t>
-        </is>
-      </c>
+      <c r="E771" s="2"/>
       <c r="F771" s="2"/>
       <c r="G771" s="2"/>
     </row>
@@ -21724,7 +21744,7 @@
       </c>
       <c r="B772" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">condicao_pagamento</t>
         </is>
       </c>
       <c r="C772" t="inlineStr" s="2">
@@ -21749,12 +21769,12 @@
       </c>
       <c r="B773" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">valor</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C773" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D773" t="inlineStr" s="2">
@@ -21764,7 +21784,11 @@
       </c>
       <c r="E773" s="2"/>
       <c r="F773" s="2"/>
-      <c r="G773" s="2"/>
+      <c r="G773" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="774">
       <c r="A774" t="inlineStr" s="2">
@@ -21774,12 +21798,12 @@
       </c>
       <c r="B774" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">consultor_responsavel</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C774" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D774" t="inlineStr" s="2">
@@ -21788,12 +21812,12 @@
         </is>
       </c>
       <c r="E774" s="2"/>
-      <c r="F774" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">users</t>
-        </is>
-      </c>
-      <c r="G774" s="2"/>
+      <c r="F774" s="2"/>
+      <c r="G774" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="775">
       <c r="A775" t="inlineStr" s="2">
@@ -21803,12 +21827,12 @@
       </c>
       <c r="B775" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">recorrencia_mensal</t>
+          <t xml:space="preserve">tipo_venda</t>
         </is>
       </c>
       <c r="C775" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D775" t="inlineStr" s="2">
@@ -21818,7 +21842,7 @@
       </c>
       <c r="E775" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">true / false</t>
+          <t xml:space="preserve">Energia Solar | O&amp;M (Operação e Manutenção) | Baterias | Carregadores Veículos Elétricos</t>
         </is>
       </c>
       <c r="F775" s="2"/>
@@ -21827,12 +21851,12 @@
     <row r="776">
       <c r="A776" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">analises_fatura</t>
+          <t xml:space="preserve">negocios</t>
         </is>
       </c>
       <c r="B776" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">token</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C776" t="inlineStr" s="2">
@@ -21842,7 +21866,7 @@
       </c>
       <c r="D776" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E776" s="2"/>
@@ -21852,17 +21876,17 @@
     <row r="777">
       <c r="A777" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">analises_fatura</t>
+          <t xml:space="preserve">negocios</t>
         </is>
       </c>
       <c r="B777" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_id</t>
+          <t xml:space="preserve">valor</t>
         </is>
       </c>
       <c r="C777" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D777" t="inlineStr" s="2">
@@ -21871,27 +21895,23 @@
         </is>
       </c>
       <c r="E777" s="2"/>
-      <c r="F777" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+      <c r="F777" s="2"/>
       <c r="G777" s="2"/>
     </row>
     <row r="778">
       <c r="A778" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">analises_fatura</t>
+          <t xml:space="preserve">negocios</t>
         </is>
       </c>
       <c r="B778" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_nome</t>
+          <t xml:space="preserve">consultor_responsavel</t>
         </is>
       </c>
       <c r="C778" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D778" t="inlineStr" s="2">
@@ -21900,23 +21920,27 @@
         </is>
       </c>
       <c r="E778" s="2"/>
-      <c r="F778" s="2"/>
+      <c r="F778" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">users</t>
+        </is>
+      </c>
       <c r="G778" s="2"/>
     </row>
     <row r="779">
       <c r="A779" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">analises_fatura</t>
+          <t xml:space="preserve">negocios</t>
         </is>
       </c>
       <c r="B779" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">uc</t>
+          <t xml:space="preserve">recorrencia_mensal</t>
         </is>
       </c>
       <c r="C779" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D779" t="inlineStr" s="2">
@@ -21924,7 +21948,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E779" s="2"/>
+      <c r="E779" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F779" s="2"/>
       <c r="G779" s="2"/>
     </row>
@@ -21936,7 +21964,7 @@
       </c>
       <c r="B780" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">competencia</t>
+          <t xml:space="preserve">token</t>
         </is>
       </c>
       <c r="C780" t="inlineStr" s="2">
@@ -21946,7 +21974,7 @@
       </c>
       <c r="D780" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E780" s="2"/>
@@ -21961,12 +21989,12 @@
       </c>
       <c r="B781" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">vencimento</t>
+          <t xml:space="preserve">cliente_id</t>
         </is>
       </c>
       <c r="C781" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D781" t="inlineStr" s="2">
@@ -21975,7 +22003,11 @@
         </is>
       </c>
       <c r="E781" s="2"/>
-      <c r="F781" s="2"/>
+      <c r="F781" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G781" s="2"/>
     </row>
     <row r="782">
@@ -21986,12 +22018,12 @@
       </c>
       <c r="B782" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">total_pagar</t>
+          <t xml:space="preserve">cliente_nome</t>
         </is>
       </c>
       <c r="C782" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D782" t="inlineStr" s="2">
@@ -22011,12 +22043,12 @@
       </c>
       <c r="B783" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">consumo_kwh</t>
+          <t xml:space="preserve">uc</t>
         </is>
       </c>
       <c r="C783" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D783" t="inlineStr" s="2">
@@ -22036,12 +22068,12 @@
       </c>
       <c r="B784" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">energia_injetada_kwh</t>
+          <t xml:space="preserve">competencia</t>
         </is>
       </c>
       <c r="C784" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D784" t="inlineStr" s="2">
@@ -22061,12 +22093,12 @@
       </c>
       <c r="B785" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">creditos_compensados_kwh</t>
+          <t xml:space="preserve">vencimento</t>
         </is>
       </c>
       <c r="C785" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D785" t="inlineStr" s="2">
@@ -22086,7 +22118,7 @@
       </c>
       <c r="B786" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">saldo_energia_kwh</t>
+          <t xml:space="preserve">total_pagar</t>
         </is>
       </c>
       <c r="C786" t="inlineStr" s="2">
@@ -22111,7 +22143,7 @@
       </c>
       <c r="B787" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">saldo_expirar_kwh</t>
+          <t xml:space="preserve">consumo_kwh</t>
         </is>
       </c>
       <c r="C787" t="inlineStr" s="2">
@@ -22136,7 +22168,7 @@
       </c>
       <c r="B788" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">economia_estimada_rs</t>
+          <t xml:space="preserve">energia_injetada_kwh</t>
         </is>
       </c>
       <c r="C788" t="inlineStr" s="2">
@@ -22161,12 +22193,12 @@
       </c>
       <c r="B789" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">papel_uc</t>
+          <t xml:space="preserve">creditos_compensados_kwh</t>
         </is>
       </c>
       <c r="C789" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D789" t="inlineStr" s="2">
@@ -22186,12 +22218,12 @@
       </c>
       <c r="B790" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">arquivos_nomes</t>
+          <t xml:space="preserve">saldo_energia_kwh</t>
         </is>
       </c>
       <c r="C790" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D790" t="inlineStr" s="2">
@@ -22201,11 +22233,7 @@
       </c>
       <c r="E790" s="2"/>
       <c r="F790" s="2"/>
-      <c r="G790" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="G790" s="2"/>
     </row>
     <row r="791">
       <c r="A791" t="inlineStr" s="2">
@@ -22215,12 +22243,12 @@
       </c>
       <c r="B791" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">dados_completos</t>
+          <t xml:space="preserve">saldo_expirar_kwh</t>
         </is>
       </c>
       <c r="C791" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D791" t="inlineStr" s="2">
@@ -22230,11 +22258,7 @@
       </c>
       <c r="E791" s="2"/>
       <c r="F791" s="2"/>
-      <c r="G791" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="G791" s="2"/>
     </row>
     <row r="792">
       <c r="A792" t="inlineStr" s="2">
@@ -22244,12 +22268,12 @@
       </c>
       <c r="B792" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">atividade_id</t>
+          <t xml:space="preserve">economia_estimada_rs</t>
         </is>
       </c>
       <c r="C792" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D792" t="inlineStr" s="2">
@@ -22269,12 +22293,12 @@
       </c>
       <c r="B793" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">whatsapp_enviado</t>
+          <t xml:space="preserve">papel_uc</t>
         </is>
       </c>
       <c r="C793" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D793" t="inlineStr" s="2">
@@ -22282,11 +22306,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E793" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E793" s="2"/>
       <c r="F793" s="2"/>
       <c r="G793" s="2"/>
     </row>
@@ -22298,12 +22318,12 @@
       </c>
       <c r="B794" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">whatsapp_enviado_em</t>
+          <t xml:space="preserve">arquivos_nomes</t>
         </is>
       </c>
       <c r="C794" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D794" t="inlineStr" s="2">
@@ -22313,7 +22333,11 @@
       </c>
       <c r="E794" s="2"/>
       <c r="F794" s="2"/>
-      <c r="G794" s="2"/>
+      <c r="G794" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Estrutura JSON livre</t>
+        </is>
+      </c>
     </row>
     <row r="795">
       <c r="A795" t="inlineStr" s="2">
@@ -22323,12 +22347,12 @@
       </c>
       <c r="B795" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">dados_completos</t>
         </is>
       </c>
       <c r="C795" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D795" t="inlineStr" s="2">
@@ -22340,7 +22364,7 @@
       <c r="F795" s="2"/>
       <c r="G795" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
+          <t xml:space="preserve">Estrutura JSON livre</t>
         </is>
       </c>
     </row>
@@ -22352,12 +22376,12 @@
       </c>
       <c r="B796" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">atividade_id</t>
         </is>
       </c>
       <c r="C796" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D796" t="inlineStr" s="2">
@@ -22367,46 +22391,46 @@
       </c>
       <c r="E796" s="2"/>
       <c r="F796" s="2"/>
-      <c r="G796" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G796" s="2"/>
     </row>
     <row r="797">
       <c r="A797" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">knowledge_categories</t>
+          <t xml:space="preserve">analises_fatura</t>
         </is>
       </c>
       <c r="B797" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">whatsapp_enviado</t>
         </is>
       </c>
       <c r="C797" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D797" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E797" s="2"/>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E797" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F797" s="2"/>
       <c r="G797" s="2"/>
     </row>
     <row r="798">
       <c r="A798" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">knowledge_categories</t>
+          <t xml:space="preserve">analises_fatura</t>
         </is>
       </c>
       <c r="B798" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">descricao</t>
+          <t xml:space="preserve">whatsapp_enviado_em</t>
         </is>
       </c>
       <c r="C798" t="inlineStr" s="2">
@@ -22426,17 +22450,17 @@
     <row r="799">
       <c r="A799" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">knowledge_categories</t>
+          <t xml:space="preserve">analises_fatura</t>
         </is>
       </c>
       <c r="B799" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">icone</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C799" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D799" t="inlineStr" s="2">
@@ -22446,22 +22470,26 @@
       </c>
       <c r="E799" s="2"/>
       <c r="F799" s="2"/>
-      <c r="G799" s="2"/>
+      <c r="G799" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="800">
       <c r="A800" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">knowledge_categories</t>
+          <t xml:space="preserve">analises_fatura</t>
         </is>
       </c>
       <c r="B800" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ordem</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C800" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D800" t="inlineStr" s="2">
@@ -22471,7 +22499,11 @@
       </c>
       <c r="E800" s="2"/>
       <c r="F800" s="2"/>
-      <c r="G800" s="2"/>
+      <c r="G800" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="801">
       <c r="A801" t="inlineStr" s="2">
@@ -22481,26 +22513,22 @@
       </c>
       <c r="B801" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C801" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D801" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E801" s="2"/>
       <c r="F801" s="2"/>
-      <c r="G801" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G801" s="2"/>
     </row>
     <row r="802">
       <c r="A802" t="inlineStr" s="2">
@@ -22510,12 +22538,12 @@
       </c>
       <c r="B802" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">descricao</t>
         </is>
       </c>
       <c r="C802" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D802" t="inlineStr" s="2">
@@ -22525,60 +22553,52 @@
       </c>
       <c r="E802" s="2"/>
       <c r="F802" s="2"/>
-      <c r="G802" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G802" s="2"/>
     </row>
     <row r="803">
       <c r="A803" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">knowledge_articles</t>
+          <t xml:space="preserve">knowledge_categories</t>
         </is>
       </c>
       <c r="B803" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">categoria_id</t>
+          <t xml:space="preserve">icone</t>
         </is>
       </c>
       <c r="C803" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D803" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E803" s="2"/>
-      <c r="F803" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">knowledge_categories</t>
-        </is>
-      </c>
+      <c r="F803" s="2"/>
       <c r="G803" s="2"/>
     </row>
     <row r="804">
       <c r="A804" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">knowledge_articles</t>
+          <t xml:space="preserve">knowledge_categories</t>
         </is>
       </c>
       <c r="B804" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">ordem</t>
         </is>
       </c>
       <c r="C804" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D804" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E804" s="2"/>
@@ -22588,42 +22608,46 @@
     <row r="805">
       <c r="A805" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">knowledge_articles</t>
+          <t xml:space="preserve">knowledge_categories</t>
         </is>
       </c>
       <c r="B805" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">conteudo</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C805" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D805" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E805" s="2"/>
       <c r="F805" s="2"/>
-      <c r="G805" s="2"/>
+      <c r="G805" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="806">
       <c r="A806" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">knowledge_articles</t>
+          <t xml:space="preserve">knowledge_categories</t>
         </is>
       </c>
       <c r="B806" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">texto_extraido</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C806" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D806" t="inlineStr" s="2">
@@ -22633,7 +22657,11 @@
       </c>
       <c r="E806" s="2"/>
       <c r="F806" s="2"/>
-      <c r="G806" s="2"/>
+      <c r="G806" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="807">
       <c r="A807" t="inlineStr" s="2">
@@ -22643,26 +22671,26 @@
       </c>
       <c r="B807" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">anexos</t>
+          <t xml:space="preserve">categoria_id</t>
         </is>
       </c>
       <c r="C807" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">file</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D807" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E807" s="2"/>
-      <c r="F807" s="2"/>
-      <c r="G807" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
-        </is>
-      </c>
+      <c r="F807" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_categories</t>
+        </is>
+      </c>
+      <c r="G807" s="2"/>
     </row>
     <row r="808">
       <c r="A808" t="inlineStr" s="2">
@@ -22672,25 +22700,21 @@
       </c>
       <c r="B808" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">criado_por</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C808" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D808" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E808" s="2"/>
-      <c r="F808" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">users</t>
-        </is>
-      </c>
+      <c r="F808" s="2"/>
       <c r="G808" s="2"/>
     </row>
     <row r="809">
@@ -22701,7 +22725,7 @@
       </c>
       <c r="B809" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autor_nome</t>
+          <t xml:space="preserve">conteudo</t>
         </is>
       </c>
       <c r="C809" t="inlineStr" s="2">
@@ -22711,7 +22735,7 @@
       </c>
       <c r="D809" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E809" s="2"/>
@@ -22726,7 +22750,7 @@
       </c>
       <c r="B810" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tags</t>
+          <t xml:space="preserve">texto_extraido</t>
         </is>
       </c>
       <c r="C810" t="inlineStr" s="2">
@@ -22751,12 +22775,12 @@
       </c>
       <c r="B811" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">anexos</t>
         </is>
       </c>
       <c r="C811" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="D811" t="inlineStr" s="2">
@@ -22768,7 +22792,7 @@
       <c r="F811" s="2"/>
       <c r="G811" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
+          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
         </is>
       </c>
     </row>
@@ -22780,12 +22804,12 @@
       </c>
       <c r="B812" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">criado_por</t>
         </is>
       </c>
       <c r="C812" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D812" t="inlineStr" s="2">
@@ -22794,85 +22818,77 @@
         </is>
       </c>
       <c r="E812" s="2"/>
-      <c r="F812" s="2"/>
-      <c r="G812" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="F812" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">users</t>
+        </is>
+      </c>
+      <c r="G812" s="2"/>
     </row>
     <row r="813">
       <c r="A813" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contratos_usinas</t>
+          <t xml:space="preserve">knowledge_articles</t>
         </is>
       </c>
       <c r="B813" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contrato_id</t>
+          <t xml:space="preserve">autor_nome</t>
         </is>
       </c>
       <c r="C813" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D813" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E813" s="2"/>
-      <c r="F813" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">contratos_om</t>
-        </is>
-      </c>
+      <c r="F813" s="2"/>
       <c r="G813" s="2"/>
     </row>
     <row r="814">
       <c r="A814" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contratos_usinas</t>
+          <t xml:space="preserve">knowledge_articles</t>
         </is>
       </c>
       <c r="B814" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">usina_id</t>
+          <t xml:space="preserve">tags</t>
         </is>
       </c>
       <c r="C814" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D814" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E814" s="2"/>
-      <c r="F814" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">usinas</t>
-        </is>
-      </c>
+      <c r="F814" s="2"/>
       <c r="G814" s="2"/>
     </row>
     <row r="815">
       <c r="A815" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contratos_usinas</t>
+          <t xml:space="preserve">knowledge_articles</t>
         </is>
       </c>
       <c r="B815" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ativo</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C815" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D815" t="inlineStr" s="2">
@@ -22880,28 +22896,28 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E815" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E815" s="2"/>
       <c r="F815" s="2"/>
-      <c r="G815" s="2"/>
+      <c r="G815" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="816">
       <c r="A816" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contratos_usinas</t>
+          <t xml:space="preserve">knowledge_articles</t>
         </is>
       </c>
       <c r="B816" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_vinculo</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C816" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D816" t="inlineStr" s="2">
@@ -22911,7 +22927,11 @@
       </c>
       <c r="E816" s="2"/>
       <c r="F816" s="2"/>
-      <c r="G816" s="2"/>
+      <c r="G816" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="817">
       <c r="A817" t="inlineStr" s="2">
@@ -22921,21 +22941,25 @@
       </c>
       <c r="B817" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_desvinculo</t>
+          <t xml:space="preserve">contrato_id</t>
         </is>
       </c>
       <c r="C817" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D817" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E817" s="2"/>
-      <c r="F817" s="2"/>
+      <c r="F817" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contratos_om</t>
+        </is>
+      </c>
       <c r="G817" s="2"/>
     </row>
     <row r="818">
@@ -22946,21 +22970,25 @@
       </c>
       <c r="B818" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">observacoes</t>
+          <t xml:space="preserve">usina_id</t>
         </is>
       </c>
       <c r="C818" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D818" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E818" s="2"/>
-      <c r="F818" s="2"/>
+      <c r="F818" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usinas</t>
+        </is>
+      </c>
       <c r="G818" s="2"/>
     </row>
     <row r="819">
@@ -22971,12 +22999,12 @@
       </c>
       <c r="B819" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">ativo</t>
         </is>
       </c>
       <c r="C819" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D819" t="inlineStr" s="2">
@@ -22984,13 +23012,13 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E819" s="2"/>
+      <c r="E819" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F819" s="2"/>
-      <c r="G819" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G819" s="2"/>
     </row>
     <row r="820">
       <c r="A820" t="inlineStr" s="2">
@@ -23000,12 +23028,12 @@
       </c>
       <c r="B820" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">data_vinculo</t>
         </is>
       </c>
       <c r="C820" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D820" t="inlineStr" s="2">
@@ -23015,26 +23043,22 @@
       </c>
       <c r="E820" s="2"/>
       <c r="F820" s="2"/>
-      <c r="G820" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="G820" s="2"/>
     </row>
     <row r="821">
       <c r="A821" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ativos</t>
+          <t xml:space="preserve">contratos_usinas</t>
         </is>
       </c>
       <c r="B821" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">usina_id</t>
+          <t xml:space="preserve">data_desvinculo</t>
         </is>
       </c>
       <c r="C821" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D821" t="inlineStr" s="2">
@@ -23043,56 +23067,48 @@
         </is>
       </c>
       <c r="E821" s="2"/>
-      <c r="F821" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">usinas</t>
-        </is>
-      </c>
+      <c r="F821" s="2"/>
       <c r="G821" s="2"/>
     </row>
     <row r="822">
       <c r="A822" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ativos</t>
+          <t xml:space="preserve">contratos_usinas</t>
         </is>
       </c>
       <c r="B822" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo</t>
+          <t xml:space="preserve">observacoes</t>
         </is>
       </c>
       <c r="C822" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D822" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E822" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">inversor | placa_solar | bateria | string_box | outros</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E822" s="2"/>
       <c r="F822" s="2"/>
       <c r="G822" s="2"/>
     </row>
     <row r="823">
       <c r="A823" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ativos</t>
+          <t xml:space="preserve">contratos_usinas</t>
         </is>
       </c>
       <c r="B823" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_outro_descricao</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C823" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D823" t="inlineStr" s="2">
@@ -23102,32 +23118,40 @@
       </c>
       <c r="E823" s="2"/>
       <c r="F823" s="2"/>
-      <c r="G823" s="2"/>
+      <c r="G823" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="824">
       <c r="A824" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ativos</t>
+          <t xml:space="preserve">contratos_usinas</t>
         </is>
       </c>
       <c r="B824" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fabricante</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C824" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D824" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E824" s="2"/>
       <c r="F824" s="2"/>
-      <c r="G824" s="2"/>
+      <c r="G824" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="825">
       <c r="A825" t="inlineStr" s="2">
@@ -23137,21 +23161,25 @@
       </c>
       <c r="B825" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">modelo</t>
+          <t xml:space="preserve">usina_id</t>
         </is>
       </c>
       <c r="C825" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D825" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E825" s="2"/>
-      <c r="F825" s="2"/>
+      <c r="F825" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usinas</t>
+        </is>
+      </c>
       <c r="G825" s="2"/>
     </row>
     <row r="826">
@@ -23162,20 +23190,24 @@
       </c>
       <c r="B826" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">numero_serie</t>
+          <t xml:space="preserve">tipo</t>
         </is>
       </c>
       <c r="C826" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D826" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E826" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E826" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">inversor | placa_solar | bateria | string_box | outros</t>
+        </is>
+      </c>
       <c r="F826" s="2"/>
       <c r="G826" s="2"/>
     </row>
@@ -23187,12 +23219,12 @@
       </c>
       <c r="B827" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_instalacao</t>
+          <t xml:space="preserve">tipo_outro_descricao</t>
         </is>
       </c>
       <c r="C827" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D827" t="inlineStr" s="2">
@@ -23212,17 +23244,17 @@
       </c>
       <c r="B828" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_fim_garantia</t>
+          <t xml:space="preserve">fabricante</t>
         </is>
       </c>
       <c r="C828" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D828" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E828" s="2"/>
@@ -23237,25 +23269,21 @@
       </c>
       <c r="B829" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">responsavel_id</t>
+          <t xml:space="preserve">modelo</t>
         </is>
       </c>
       <c r="C829" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D829" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E829" s="2"/>
-      <c r="F829" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">users</t>
-        </is>
-      </c>
+      <c r="F829" s="2"/>
       <c r="G829" s="2"/>
     </row>
     <row r="830">
@@ -23266,7 +23294,7 @@
       </c>
       <c r="B830" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">observacoes</t>
+          <t xml:space="preserve">numero_serie</t>
         </is>
       </c>
       <c r="C830" t="inlineStr" s="2">
@@ -23291,12 +23319,12 @@
       </c>
       <c r="B831" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">status_operacional</t>
+          <t xml:space="preserve">data_instalacao</t>
         </is>
       </c>
       <c r="C831" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D831" t="inlineStr" s="2">
@@ -23304,11 +23332,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E831" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">operacional | em_alerta | manutencao | desativado</t>
-        </is>
-      </c>
+      <c r="E831" s="2"/>
       <c r="F831" s="2"/>
       <c r="G831" s="2"/>
     </row>
@@ -23320,12 +23344,12 @@
       </c>
       <c r="B832" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">data_fim_garantia</t>
         </is>
       </c>
       <c r="C832" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D832" t="inlineStr" s="2">
@@ -23335,11 +23359,7 @@
       </c>
       <c r="E832" s="2"/>
       <c r="F832" s="2"/>
-      <c r="G832" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G832" s="2"/>
     </row>
     <row r="833">
       <c r="A833" t="inlineStr" s="2">
@@ -23349,12 +23369,12 @@
       </c>
       <c r="B833" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">responsavel_id</t>
         </is>
       </c>
       <c r="C833" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D833" t="inlineStr" s="2">
@@ -23363,12 +23383,12 @@
         </is>
       </c>
       <c r="E833" s="2"/>
-      <c r="F833" s="2"/>
-      <c r="G833" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
-        </is>
-      </c>
+      <c r="F833" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">users</t>
+        </is>
+      </c>
+      <c r="G833" s="2"/>
     </row>
     <row r="834">
       <c r="A834" t="inlineStr" s="2">
@@ -23378,7 +23398,7 @@
       </c>
       <c r="B834" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">chave_importacao</t>
+          <t xml:space="preserve">observacoes</t>
         </is>
       </c>
       <c r="C834" t="inlineStr" s="2">
@@ -23403,12 +23423,12 @@
       </c>
       <c r="B835" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_inversor_id</t>
+          <t xml:space="preserve">status_operacional</t>
         </is>
       </c>
       <c r="C835" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D835" t="inlineStr" s="2">
@@ -23416,49 +23436,57 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E835" s="2"/>
+      <c r="E835" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">operacional | em_alerta | manutencao | desativado</t>
+        </is>
+      </c>
       <c r="F835" s="2"/>
       <c r="G835" s="2"/>
     </row>
     <row r="836">
       <c r="A836" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contatos</t>
+          <t xml:space="preserve">ativos</t>
         </is>
       </c>
       <c r="B836" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">nome</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C836" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D836" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E836" s="2"/>
       <c r="F836" s="2"/>
-      <c r="G836" s="2"/>
+      <c r="G836" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
     </row>
     <row r="837">
       <c r="A837" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contatos</t>
+          <t xml:space="preserve">ativos</t>
         </is>
       </c>
       <c r="B837" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">telefone</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C837" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D837" t="inlineStr" s="2">
@@ -23468,17 +23496,21 @@
       </c>
       <c r="E837" s="2"/>
       <c r="F837" s="2"/>
-      <c r="G837" s="2"/>
+      <c r="G837" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="838">
       <c r="A838" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contatos</t>
+          <t xml:space="preserve">ativos</t>
         </is>
       </c>
       <c r="B838" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">whatsapp</t>
+          <t xml:space="preserve">chave_importacao</t>
         </is>
       </c>
       <c r="C838" t="inlineStr" s="2">
@@ -23498,17 +23530,17 @@
     <row r="839">
       <c r="A839" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contatos</t>
+          <t xml:space="preserve">ativos</t>
         </is>
       </c>
       <c r="B839" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">email</t>
+          <t xml:space="preserve">cliente_inversor_id</t>
         </is>
       </c>
       <c r="C839" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">email</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D839" t="inlineStr" s="2">
@@ -23528,24 +23560,20 @@
       </c>
       <c r="B840" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">papel</t>
+          <t xml:space="preserve">nome</t>
         </is>
       </c>
       <c r="C840" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D840" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E840" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">cliente | lead | fornecedor | tecnico | parceiro | familiar | responsavel | financeiro | outro</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E840" s="2"/>
       <c r="F840" s="2"/>
       <c r="G840" s="2"/>
     </row>
@@ -23557,7 +23585,7 @@
       </c>
       <c r="B841" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cargo</t>
+          <t xml:space="preserve">telefone</t>
         </is>
       </c>
       <c r="C841" t="inlineStr" s="2">
@@ -23582,7 +23610,7 @@
       </c>
       <c r="B842" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">observacoes</t>
+          <t xml:space="preserve">whatsapp</t>
         </is>
       </c>
       <c r="C842" t="inlineStr" s="2">
@@ -23607,12 +23635,12 @@
       </c>
       <c r="B843" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">clientes_vinculados</t>
+          <t xml:space="preserve">email</t>
         </is>
       </c>
       <c r="C843" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">email</t>
         </is>
       </c>
       <c r="D843" t="inlineStr" s="2">
@@ -23621,11 +23649,7 @@
         </is>
       </c>
       <c r="E843" s="2"/>
-      <c r="F843" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+      <c r="F843" s="2"/>
       <c r="G843" s="2"/>
     </row>
     <row r="844">
@@ -23636,12 +23660,12 @@
       </c>
       <c r="B844" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios_vinculados</t>
+          <t xml:space="preserve">papel</t>
         </is>
       </c>
       <c r="C844" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D844" t="inlineStr" s="2">
@@ -23649,12 +23673,12 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E844" s="2"/>
-      <c r="F844" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">negocios</t>
-        </is>
-      </c>
+      <c r="E844" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">cliente | lead | fornecedor | tecnico | parceiro | familiar | responsavel | financeiro | outro</t>
+        </is>
+      </c>
+      <c r="F844" s="2"/>
       <c r="G844" s="2"/>
     </row>
     <row r="845">
@@ -23665,7 +23689,7 @@
       </c>
       <c r="B845" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">conversa_id</t>
+          <t xml:space="preserve">cargo</t>
         </is>
       </c>
       <c r="C845" t="inlineStr" s="2">
@@ -23690,7 +23714,7 @@
       </c>
       <c r="B846" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">origem_registro</t>
+          <t xml:space="preserve">observacoes</t>
         </is>
       </c>
       <c r="C846" t="inlineStr" s="2">
@@ -23715,12 +23739,12 @@
       </c>
       <c r="B847" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">clientes_vinculados</t>
         </is>
       </c>
       <c r="C847" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D847" t="inlineStr" s="2">
@@ -23729,12 +23753,12 @@
         </is>
       </c>
       <c r="E847" s="2"/>
-      <c r="F847" s="2"/>
-      <c r="G847" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="F847" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
+      <c r="G847" s="2"/>
     </row>
     <row r="848">
       <c r="A848" t="inlineStr" s="2">
@@ -23744,22 +23768,321 @@
       </c>
       <c r="B848" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">negocios_vinculados</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">relation</t>
+        </is>
+      </c>
+      <c r="D848" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E848" s="2"/>
+      <c r="F848" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
+      <c r="G848" s="2"/>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contatos</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">conversa_id</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D849" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E849" s="2"/>
+      <c r="F849" s="2"/>
+      <c r="G849" s="2"/>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contatos</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">origem_registro</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D850" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E850" s="2"/>
+      <c r="F850" s="2"/>
+      <c r="G850" s="2"/>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contatos</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">created</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D851" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E851" s="2"/>
+      <c r="F851" s="2"/>
+      <c r="G851" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contatos</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">updated</t>
         </is>
       </c>
-      <c r="C848" t="inlineStr" s="2">
+      <c r="C852" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">autodate</t>
         </is>
       </c>
-      <c r="D848" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E848" s="2"/>
-      <c r="F848" s="2"/>
-      <c r="G848" t="inlineStr" s="2">
+      <c r="D852" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E852" s="2"/>
+      <c r="F852" s="2"/>
+      <c r="G852" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usina_equipamentos</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usina_id</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">relation</t>
+        </is>
+      </c>
+      <c r="D853" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E853" s="2"/>
+      <c r="F853" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usinas</t>
+        </is>
+      </c>
+      <c r="G853" s="2"/>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usina_equipamentos</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">equipamento_id</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">relation</t>
+        </is>
+      </c>
+      <c r="D854" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E854" s="2"/>
+      <c r="F854" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">equipamentos</t>
+        </is>
+      </c>
+      <c r="G854" s="2"/>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usina_equipamentos</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">quantidade</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D855" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E855" s="2"/>
+      <c r="F855" s="2"/>
+      <c r="G855" s="2"/>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usina_equipamentos</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">numero_serie</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D856" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E856" s="2"/>
+      <c r="F856" s="2"/>
+      <c r="G856" s="2"/>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usina_equipamentos</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">observacoes</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="D857" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E857" s="2"/>
+      <c r="F857" s="2"/>
+      <c r="G857" s="2"/>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usina_equipamentos</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">created</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D858" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E858" s="2"/>
+      <c r="F858" s="2"/>
+      <c r="G858" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usina_equipamentos</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">updated</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D859" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E859" s="2"/>
+      <c r="F859" s="2"/>
+      <c r="G859" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
         </is>
@@ -25127,17 +25450,17 @@
     <row r="43">
       <c r="A43" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">equipamentos</t>
         </is>
       </c>
       <c r="B43" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_especifico_id</t>
+          <t xml:space="preserve">fornecedor_id</t>
         </is>
       </c>
       <c r="C43" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">clientes</t>
+          <t xml:space="preserve">fornecedores</t>
         </is>
       </c>
       <c r="D43" t="inlineStr" s="2">
@@ -25152,29 +25475,29 @@
       </c>
       <c r="F43" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Relaciona o registro de automacoes com clientes</t>
+          <t xml:space="preserve">Fornecedor ou distribuidor solar associado</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes_execucoes</t>
+          <t xml:space="preserve">automacoes</t>
         </is>
       </c>
       <c r="B44" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacao</t>
+          <t xml:space="preserve">cliente_especifico_id</t>
         </is>
       </c>
       <c r="C44" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">clientes</t>
         </is>
       </c>
       <c r="D44" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E44" t="inlineStr" s="2">
@@ -25184,7 +25507,7 @@
       </c>
       <c r="F44" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Relaciona o registro de automacoes_execucoes com automacoes</t>
+          <t xml:space="preserve">Relaciona o registro de automacoes com clientes</t>
         </is>
       </c>
     </row>
@@ -25196,17 +25519,17 @@
       </c>
       <c r="B45" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente</t>
+          <t xml:space="preserve">automacao</t>
         </is>
       </c>
       <c r="C45" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">clientes</t>
+          <t xml:space="preserve">automacoes</t>
         </is>
       </c>
       <c r="D45" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E45" t="inlineStr" s="2">
@@ -25216,24 +25539,24 @@
       </c>
       <c r="F45" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Vínculo do registro ao cliente proprietário</t>
+          <t xml:space="preserve">Relaciona o registro de automacoes_execucoes com automacoes</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">automacoes_execucoes</t>
         </is>
       </c>
       <c r="B46" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">atividade_id</t>
+          <t xml:space="preserve">cliente</t>
         </is>
       </c>
       <c r="C46" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">atividades</t>
+          <t xml:space="preserve">clientes</t>
         </is>
       </c>
       <c r="D46" t="inlineStr" s="2">
@@ -25248,7 +25571,7 @@
       </c>
       <c r="F46" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Relaciona o registro de notificacoes_internas com atividades</t>
+          <t xml:space="preserve">Vínculo do registro ao cliente proprietário</t>
         </is>
       </c>
     </row>
@@ -25260,12 +25583,12 @@
       </c>
       <c r="B47" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_id</t>
+          <t xml:space="preserve">atividade_id</t>
         </is>
       </c>
       <c r="C47" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">clientes</t>
+          <t xml:space="preserve">atividades</t>
         </is>
       </c>
       <c r="D47" t="inlineStr" s="2">
@@ -25280,14 +25603,14 @@
       </c>
       <c r="F47" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Vínculo do registro ao cliente proprietário</t>
+          <t xml:space="preserve">Relaciona o registro de notificacoes_internas com atividades</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">notificacoes_internas</t>
         </is>
       </c>
       <c r="B48" t="inlineStr" s="2">
@@ -25302,7 +25625,7 @@
       </c>
       <c r="D48" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E48" t="inlineStr" s="2">
@@ -25324,17 +25647,17 @@
       </c>
       <c r="B49" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">consultor_responsavel</t>
+          <t xml:space="preserve">cliente_id</t>
         </is>
       </c>
       <c r="C49" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">users</t>
+          <t xml:space="preserve">clientes</t>
         </is>
       </c>
       <c r="D49" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E49" t="inlineStr" s="2">
@@ -25344,24 +25667,24 @@
       </c>
       <c r="F49" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Relaciona o registro de negocios com users</t>
+          <t xml:space="preserve">Vínculo do registro ao cliente proprietário</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">analises_fatura</t>
+          <t xml:space="preserve">negocios</t>
         </is>
       </c>
       <c r="B50" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_id</t>
+          <t xml:space="preserve">consultor_responsavel</t>
         </is>
       </c>
       <c r="C50" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">clientes</t>
+          <t xml:space="preserve">users</t>
         </is>
       </c>
       <c r="D50" t="inlineStr" s="2">
@@ -25376,29 +25699,29 @@
       </c>
       <c r="F50" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Vínculo do registro ao cliente proprietário</t>
+          <t xml:space="preserve">Relaciona o registro de negocios com users</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">knowledge_articles</t>
+          <t xml:space="preserve">analises_fatura</t>
         </is>
       </c>
       <c r="B51" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">categoria_id</t>
+          <t xml:space="preserve">cliente_id</t>
         </is>
       </c>
       <c r="C51" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">knowledge_categories</t>
+          <t xml:space="preserve">clientes</t>
         </is>
       </c>
       <c r="D51" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E51" t="inlineStr" s="2">
@@ -25408,7 +25731,7 @@
       </c>
       <c r="F51" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Relaciona o registro de knowledge_articles com knowledge_categories</t>
+          <t xml:space="preserve">Vínculo do registro ao cliente proprietário</t>
         </is>
       </c>
     </row>
@@ -25420,17 +25743,17 @@
       </c>
       <c r="B52" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">criado_por</t>
+          <t xml:space="preserve">categoria_id</t>
         </is>
       </c>
       <c r="C52" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">users</t>
+          <t xml:space="preserve">knowledge_categories</t>
         </is>
       </c>
       <c r="D52" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E52" t="inlineStr" s="2">
@@ -25440,29 +25763,29 @@
       </c>
       <c r="F52" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Relaciona o registro de knowledge_articles com users</t>
+          <t xml:space="preserve">Relaciona o registro de knowledge_articles com knowledge_categories</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contratos_usinas</t>
+          <t xml:space="preserve">knowledge_articles</t>
         </is>
       </c>
       <c r="B53" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contrato_id</t>
+          <t xml:space="preserve">criado_por</t>
         </is>
       </c>
       <c r="C53" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contratos_om</t>
+          <t xml:space="preserve">users</t>
         </is>
       </c>
       <c r="D53" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E53" t="inlineStr" s="2">
@@ -25472,7 +25795,7 @@
       </c>
       <c r="F53" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Vínculo do serviço ou anomalia ao contrato de O&amp;M vigente</t>
+          <t xml:space="preserve">Relaciona o registro de knowledge_articles com users</t>
         </is>
       </c>
     </row>
@@ -25484,12 +25807,12 @@
       </c>
       <c r="B54" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">usina_id</t>
+          <t xml:space="preserve">contrato_id</t>
         </is>
       </c>
       <c r="C54" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">usinas</t>
+          <t xml:space="preserve">contratos_om</t>
         </is>
       </c>
       <c r="D54" t="inlineStr" s="2">
@@ -25504,14 +25827,14 @@
       </c>
       <c r="F54" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Vínculo da atividade à usina fotovoltaica correspondente</t>
+          <t xml:space="preserve">Vínculo do serviço ou anomalia ao contrato de O&amp;M vigente</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ativos</t>
+          <t xml:space="preserve">contratos_usinas</t>
         </is>
       </c>
       <c r="B55" t="inlineStr" s="2">
@@ -25526,7 +25849,7 @@
       </c>
       <c r="D55" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E55" t="inlineStr" s="2">
@@ -25548,12 +25871,12 @@
       </c>
       <c r="B56" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">responsavel_id</t>
+          <t xml:space="preserve">usina_id</t>
         </is>
       </c>
       <c r="C56" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">users</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="D56" t="inlineStr" s="2">
@@ -25568,24 +25891,24 @@
       </c>
       <c r="F56" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Relaciona o registro de ativos com users</t>
+          <t xml:space="preserve">Vínculo da atividade à usina fotovoltaica correspondente</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contatos</t>
+          <t xml:space="preserve">ativos</t>
         </is>
       </c>
       <c r="B57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">clientes_vinculados</t>
+          <t xml:space="preserve">responsavel_id</t>
         </is>
       </c>
       <c r="C57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">clientes</t>
+          <t xml:space="preserve">users</t>
         </is>
       </c>
       <c r="D57" t="inlineStr" s="2">
@@ -25600,7 +25923,7 @@
       </c>
       <c r="F57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Relaciona o registro de contatos com clientes</t>
+          <t xml:space="preserve">Relaciona o registro de ativos com users</t>
         </is>
       </c>
     </row>
@@ -25612,27 +25935,123 @@
       </c>
       <c r="B58" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">clientes_vinculados</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Relaciona o registro de contatos com clientes</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">contatos</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">negocios_vinculados</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr" s="2">
+      <c r="C59" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">negocios</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr" s="2">
+      <c r="D59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Relaciona o registro de contatos com negocios</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usina_equipamentos</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usina_id</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usinas</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Vínculo da atividade à usina fotovoltaica correspondente</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usina_equipamentos</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">equipamento_id</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">equipamentos</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Relaciona o registro de usina_equipamentos com equipamentos</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(contatos): mesclagem com conversao em contato adicional, busca de pessoa existente e contato principal com roteamento whatsapp
</commit_message>
<xml_diff>
--- a/public/schema-delfos-solar.xlsx
+++ b/public/schema-delfos-solar.xlsx
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="C32" s="2">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D32" t="inlineStr" s="2">
         <is>
@@ -1421,7 +1421,7 @@
         </is>
       </c>
       <c r="C48" s="2">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="D48" s="2"/>
       <c r="E48" s="2">
@@ -19475,25 +19475,29 @@
     <row r="688">
       <c r="A688" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">instalacoes_galeria</t>
+          <t xml:space="preserve">contatos_adicionais</t>
         </is>
       </c>
       <c r="B688" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">is_principal</t>
         </is>
       </c>
       <c r="C688" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D688" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E688" s="2"/>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F688" s="2"/>
       <c r="G688" s="2"/>
     </row>
@@ -19505,7 +19509,7 @@
       </c>
       <c r="B689" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cidade</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C689" t="inlineStr" s="2">
@@ -19515,7 +19519,7 @@
       </c>
       <c r="D689" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E689" s="2"/>
@@ -19530,12 +19534,12 @@
       </c>
       <c r="B690" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">potencia_kwp</t>
+          <t xml:space="preserve">cidade</t>
         </is>
       </c>
       <c r="C690" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D690" t="inlineStr" s="2">
@@ -19555,12 +19559,12 @@
       </c>
       <c r="B691" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">foto</t>
+          <t xml:space="preserve">potencia_kwp</t>
         </is>
       </c>
       <c r="C691" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">file</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D691" t="inlineStr" s="2">
@@ -19570,11 +19574,7 @@
       </c>
       <c r="E691" s="2"/>
       <c r="F691" s="2"/>
-      <c r="G691" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
-        </is>
-      </c>
+      <c r="G691" s="2"/>
     </row>
     <row r="692">
       <c r="A692" t="inlineStr" s="2">
@@ -19584,12 +19584,12 @@
       </c>
       <c r="B692" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">foto_url</t>
+          <t xml:space="preserve">foto</t>
         </is>
       </c>
       <c r="C692" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="D692" t="inlineStr" s="2">
@@ -19599,7 +19599,11 @@
       </c>
       <c r="E692" s="2"/>
       <c r="F692" s="2"/>
-      <c r="G692" s="2"/>
+      <c r="G692" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
+        </is>
+      </c>
     </row>
     <row r="693">
       <c r="A693" t="inlineStr" s="2">
@@ -19609,12 +19613,12 @@
       </c>
       <c r="B693" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ordem</t>
+          <t xml:space="preserve">foto_url</t>
         </is>
       </c>
       <c r="C693" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D693" t="inlineStr" s="2">
@@ -19634,12 +19638,12 @@
       </c>
       <c r="B694" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">destaque</t>
+          <t xml:space="preserve">ordem</t>
         </is>
       </c>
       <c r="C694" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D694" t="inlineStr" s="2">
@@ -19647,11 +19651,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E694" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E694" s="2"/>
       <c r="F694" s="2"/>
       <c r="G694" s="2"/>
     </row>
@@ -19663,12 +19663,12 @@
       </c>
       <c r="B695" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">destaque</t>
         </is>
       </c>
       <c r="C695" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D695" t="inlineStr" s="2">
@@ -19676,13 +19676,13 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E695" s="2"/>
+      <c r="E695" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F695" s="2"/>
-      <c r="G695" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G695" s="2"/>
     </row>
     <row r="696">
       <c r="A696" t="inlineStr" s="2">
@@ -19692,7 +19692,7 @@
       </c>
       <c r="B696" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C696" t="inlineStr" s="2">
@@ -19709,34 +19709,38 @@
       <c r="F696" s="2"/>
       <c r="G696" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="697">
       <c r="A697" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">projecao_tarifaria</t>
+          <t xml:space="preserve">instalacoes_galeria</t>
         </is>
       </c>
       <c r="B697" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ano</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C697" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D697" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E697" s="2"/>
       <c r="F697" s="2"/>
-      <c r="G697" s="2"/>
+      <c r="G697" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="698">
       <c r="A698" t="inlineStr" s="2">
@@ -19746,12 +19750,12 @@
       </c>
       <c r="B698" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_cliente</t>
+          <t xml:space="preserve">ano</t>
         </is>
       </c>
       <c r="C698" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D698" t="inlineStr" s="2">
@@ -19759,11 +19763,7 @@
           <t xml:space="preserve">Sim</t>
         </is>
       </c>
-      <c r="E698" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">residencial | comercial</t>
-        </is>
-      </c>
+      <c r="E698" s="2"/>
       <c r="F698" s="2"/>
       <c r="G698" s="2"/>
     </row>
@@ -19775,20 +19775,24 @@
       </c>
       <c r="B699" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tarifa_kwh</t>
+          <t xml:space="preserve">tipo_cliente</t>
         </is>
       </c>
       <c r="C699" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D699" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E699" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">residencial | comercial</t>
+        </is>
+      </c>
       <c r="F699" s="2"/>
       <c r="G699" s="2"/>
     </row>
@@ -19800,7 +19804,7 @@
       </c>
       <c r="B700" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fio_b_kwh</t>
+          <t xml:space="preserve">tarifa_kwh</t>
         </is>
       </c>
       <c r="C700" t="inlineStr" s="2">
@@ -19825,7 +19829,7 @@
       </c>
       <c r="B701" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fs</t>
+          <t xml:space="preserve">fio_b_kwh</t>
         </is>
       </c>
       <c r="C701" t="inlineStr" s="2">
@@ -19850,7 +19854,7 @@
       </c>
       <c r="B702" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gd_eco_liquida</t>
+          <t xml:space="preserve">fs</t>
         </is>
       </c>
       <c r="C702" t="inlineStr" s="2">
@@ -19875,7 +19879,7 @@
       </c>
       <c r="B703" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">economia_acumulada</t>
+          <t xml:space="preserve">gd_eco_liquida</t>
         </is>
       </c>
       <c r="C703" t="inlineStr" s="2">
@@ -19900,7 +19904,7 @@
       </c>
       <c r="B704" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gasto_acumulado</t>
+          <t xml:space="preserve">economia_acumulada</t>
         </is>
       </c>
       <c r="C704" t="inlineStr" s="2">
@@ -19925,12 +19929,12 @@
       </c>
       <c r="B705" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">gasto_acumulado</t>
         </is>
       </c>
       <c r="C705" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D705" t="inlineStr" s="2">
@@ -19940,11 +19944,7 @@
       </c>
       <c r="E705" s="2"/>
       <c r="F705" s="2"/>
-      <c r="G705" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G705" s="2"/>
     </row>
     <row r="706">
       <c r="A706" t="inlineStr" s="2">
@@ -19954,7 +19954,7 @@
       </c>
       <c r="B706" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C706" t="inlineStr" s="2">
@@ -19971,38 +19971,38 @@
       <c r="F706" s="2"/>
       <c r="G706" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="707">
       <c r="A707" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">equipamentos</t>
+          <t xml:space="preserve">projecao_tarifaria</t>
         </is>
       </c>
       <c r="B707" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C707" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D707" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E707" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">inversor | modulo_fv | outro</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E707" s="2"/>
       <c r="F707" s="2"/>
-      <c r="G707" s="2"/>
+      <c r="G707" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="708">
       <c r="A708" t="inlineStr" s="2">
@@ -20012,12 +20012,12 @@
       </c>
       <c r="B708" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">marca</t>
+          <t xml:space="preserve">tipo</t>
         </is>
       </c>
       <c r="C708" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D708" t="inlineStr" s="2">
@@ -20025,7 +20025,11 @@
           <t xml:space="preserve">Sim</t>
         </is>
       </c>
-      <c r="E708" s="2"/>
+      <c r="E708" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">inversor | modulo_fv | outro</t>
+        </is>
+      </c>
       <c r="F708" s="2"/>
       <c r="G708" s="2"/>
     </row>
@@ -20037,7 +20041,7 @@
       </c>
       <c r="B709" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">modelo</t>
+          <t xml:space="preserve">marca</t>
         </is>
       </c>
       <c r="C709" t="inlineStr" s="2">
@@ -20062,12 +20066,12 @@
       </c>
       <c r="B710" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">potencia_w</t>
+          <t xml:space="preserve">modelo</t>
         </is>
       </c>
       <c r="C710" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D710" t="inlineStr" s="2">
@@ -20087,17 +20091,17 @@
       </c>
       <c r="B711" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">descricao_padrao</t>
+          <t xml:space="preserve">potencia_w</t>
         </is>
       </c>
       <c r="C711" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D711" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E711" s="2"/>
@@ -20112,12 +20116,12 @@
       </c>
       <c r="B712" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">garantia_anos</t>
+          <t xml:space="preserve">descricao_padrao</t>
         </is>
       </c>
       <c r="C712" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D712" t="inlineStr" s="2">
@@ -20137,12 +20141,12 @@
       </c>
       <c r="B713" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">foto</t>
+          <t xml:space="preserve">garantia_anos</t>
         </is>
       </c>
       <c r="C713" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">file</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D713" t="inlineStr" s="2">
@@ -20152,11 +20156,7 @@
       </c>
       <c r="E713" s="2"/>
       <c r="F713" s="2"/>
-      <c r="G713" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
-        </is>
-      </c>
+      <c r="G713" s="2"/>
     </row>
     <row r="714">
       <c r="A714" t="inlineStr" s="2">
@@ -20166,12 +20166,12 @@
       </c>
       <c r="B714" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">foto</t>
         </is>
       </c>
       <c r="C714" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="D714" t="inlineStr" s="2">
@@ -20183,7 +20183,7 @@
       <c r="F714" s="2"/>
       <c r="G714" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
+          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
         </is>
       </c>
     </row>
@@ -20195,7 +20195,7 @@
       </c>
       <c r="B715" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C715" t="inlineStr" s="2">
@@ -20212,7 +20212,7 @@
       <c r="F715" s="2"/>
       <c r="G715" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
@@ -20224,12 +20224,12 @@
       </c>
       <c r="B716" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">datasheet_pdf</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C716" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">file</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D716" t="inlineStr" s="2">
@@ -20241,7 +20241,7 @@
       <c r="F716" s="2"/>
       <c r="G716" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
         </is>
       </c>
     </row>
@@ -20253,12 +20253,12 @@
       </c>
       <c r="B717" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">datasheet_url</t>
+          <t xml:space="preserve">datasheet_pdf</t>
         </is>
       </c>
       <c r="C717" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">url</t>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="D717" t="inlineStr" s="2">
@@ -20268,7 +20268,11 @@
       </c>
       <c r="E717" s="2"/>
       <c r="F717" s="2"/>
-      <c r="G717" s="2"/>
+      <c r="G717" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
+        </is>
+      </c>
     </row>
     <row r="718">
       <c r="A718" t="inlineStr" s="2">
@@ -20278,7 +20282,7 @@
       </c>
       <c r="B718" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">datalogger_url</t>
+          <t xml:space="preserve">datasheet_url</t>
         </is>
       </c>
       <c r="C718" t="inlineStr" s="2">
@@ -20303,12 +20307,12 @@
       </c>
       <c r="B719" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fornecedor_id</t>
+          <t xml:space="preserve">datalogger_url</t>
         </is>
       </c>
       <c r="C719" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">url</t>
         </is>
       </c>
       <c r="D719" t="inlineStr" s="2">
@@ -20317,11 +20321,7 @@
         </is>
       </c>
       <c r="E719" s="2"/>
-      <c r="F719" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">fornecedores</t>
-        </is>
-      </c>
+      <c r="F719" s="2"/>
       <c r="G719" s="2"/>
     </row>
     <row r="720">
@@ -20332,12 +20332,12 @@
       </c>
       <c r="B720" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">telefone_suporte_fornecedor</t>
+          <t xml:space="preserve">fornecedor_id</t>
         </is>
       </c>
       <c r="C720" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D720" t="inlineStr" s="2">
@@ -20346,28 +20346,32 @@
         </is>
       </c>
       <c r="E720" s="2"/>
-      <c r="F720" s="2"/>
+      <c r="F720" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">fornecedores</t>
+        </is>
+      </c>
       <c r="G720" s="2"/>
     </row>
     <row r="721">
       <c r="A721" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">parametros_tarifarios</t>
+          <t xml:space="preserve">equipamentos</t>
         </is>
       </c>
       <c r="B721" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ano</t>
+          <t xml:space="preserve">telefone_suporte_fornecedor</t>
         </is>
       </c>
       <c r="C721" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D721" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E721" s="2"/>
@@ -20382,12 +20386,12 @@
       </c>
       <c r="B722" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">classe</t>
+          <t xml:space="preserve">ano</t>
         </is>
       </c>
       <c r="C722" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D722" t="inlineStr" s="2">
@@ -20395,11 +20399,7 @@
           <t xml:space="preserve">Sim</t>
         </is>
       </c>
-      <c r="E722" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">residencial | comercial</t>
-        </is>
-      </c>
+      <c r="E722" s="2"/>
       <c r="F722" s="2"/>
       <c r="G722" s="2"/>
     </row>
@@ -20411,20 +20411,24 @@
       </c>
       <c r="B723" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tarifa</t>
+          <t xml:space="preserve">classe</t>
         </is>
       </c>
       <c r="C723" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D723" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E723" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E723" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">residencial | comercial</t>
+        </is>
+      </c>
       <c r="F723" s="2"/>
       <c r="G723" s="2"/>
     </row>
@@ -20436,7 +20440,7 @@
       </c>
       <c r="B724" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fio_b</t>
+          <t xml:space="preserve">tarifa</t>
         </is>
       </c>
       <c r="C724" t="inlineStr" s="2">
@@ -20461,7 +20465,7 @@
       </c>
       <c r="B725" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fs</t>
+          <t xml:space="preserve">fio_b</t>
         </is>
       </c>
       <c r="C725" t="inlineStr" s="2">
@@ -20486,7 +20490,7 @@
       </c>
       <c r="B726" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gd_eco_liquida</t>
+          <t xml:space="preserve">fs</t>
         </is>
       </c>
       <c r="C726" t="inlineStr" s="2">
@@ -20511,12 +20515,12 @@
       </c>
       <c r="B727" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">gd_eco_liquida</t>
         </is>
       </c>
       <c r="C727" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D727" t="inlineStr" s="2">
@@ -20526,11 +20530,7 @@
       </c>
       <c r="E727" s="2"/>
       <c r="F727" s="2"/>
-      <c r="G727" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G727" s="2"/>
     </row>
     <row r="728">
       <c r="A728" t="inlineStr" s="2">
@@ -20540,7 +20540,7 @@
       </c>
       <c r="B728" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C728" t="inlineStr" s="2">
@@ -20557,34 +20557,38 @@
       <c r="F728" s="2"/>
       <c r="G728" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="729">
       <c r="A729" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">parametros_tarifarios</t>
         </is>
       </c>
       <c r="B729" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">nome</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C729" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D729" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E729" s="2"/>
       <c r="F729" s="2"/>
-      <c r="G729" s="2"/>
+      <c r="G729" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="730">
       <c r="A730" t="inlineStr" s="2">
@@ -20594,12 +20598,12 @@
       </c>
       <c r="B730" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gatilho</t>
+          <t xml:space="preserve">nome</t>
         </is>
       </c>
       <c r="C730" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D730" t="inlineStr" s="2">
@@ -20607,11 +20611,7 @@
           <t xml:space="preserve">Sim</t>
         </is>
       </c>
-      <c r="E730" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">status_mudou | instalacao_concluida | atividade_concluida | data_especifica | dias_apos_evento</t>
-        </is>
-      </c>
+      <c r="E730" s="2"/>
       <c r="F730" s="2"/>
       <c r="G730" s="2"/>
     </row>
@@ -20623,26 +20623,26 @@
       </c>
       <c r="B731" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">configuracao_gatilho</t>
+          <t xml:space="preserve">gatilho</t>
         </is>
       </c>
       <c r="C731" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D731" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E731" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">status_mudou | instalacao_concluida | atividade_concluida | data_especifica | dias_apos_evento</t>
+        </is>
+      </c>
       <c r="F731" s="2"/>
-      <c r="G731" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="G731" s="2"/>
     </row>
     <row r="732">
       <c r="A732" t="inlineStr" s="2">
@@ -20652,26 +20652,26 @@
       </c>
       <c r="B732" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">acao</t>
+          <t xml:space="preserve">configuracao_gatilho</t>
         </is>
       </c>
       <c r="C732" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D732" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E732" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">criar_atividade | enviar_whatsapp | enviar_email | mudar_status</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E732" s="2"/>
       <c r="F732" s="2"/>
-      <c r="G732" s="2"/>
+      <c r="G732" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Estrutura JSON livre</t>
+        </is>
+      </c>
     </row>
     <row r="733">
       <c r="A733" t="inlineStr" s="2">
@@ -20681,26 +20681,26 @@
       </c>
       <c r="B733" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">configuracao_acao</t>
+          <t xml:space="preserve">acao</t>
         </is>
       </c>
       <c r="C733" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D733" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E733" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">criar_atividade | enviar_whatsapp | enviar_email | mudar_status</t>
+        </is>
+      </c>
       <c r="F733" s="2"/>
-      <c r="G733" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="G733" s="2"/>
     </row>
     <row r="734">
       <c r="A734" t="inlineStr" s="2">
@@ -20710,26 +20710,26 @@
       </c>
       <c r="B734" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">destino</t>
+          <t xml:space="preserve">configuracao_acao</t>
         </is>
       </c>
       <c r="C734" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D734" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E734" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">cliente_evento | responsavel_empresa | cliente_especifico</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E734" s="2"/>
       <c r="F734" s="2"/>
-      <c r="G734" s="2"/>
+      <c r="G734" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Estrutura JSON livre</t>
+        </is>
+      </c>
     </row>
     <row r="735">
       <c r="A735" t="inlineStr" s="2">
@@ -20739,25 +20739,25 @@
       </c>
       <c r="B735" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_especifico_id</t>
+          <t xml:space="preserve">destino</t>
         </is>
       </c>
       <c r="C735" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D735" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E735" s="2"/>
-      <c r="F735" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E735" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">cliente_evento | responsavel_empresa | cliente_especifico</t>
+        </is>
+      </c>
+      <c r="F735" s="2"/>
       <c r="G735" s="2"/>
     </row>
     <row r="736">
@@ -20768,12 +20768,12 @@
       </c>
       <c r="B736" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ativa</t>
+          <t xml:space="preserve">cliente_especifico_id</t>
         </is>
       </c>
       <c r="C736" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D736" t="inlineStr" s="2">
@@ -20781,12 +20781,12 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E736" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
-      <c r="F736" s="2"/>
+      <c r="E736" s="2"/>
+      <c r="F736" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G736" s="2"/>
     </row>
     <row r="737">
@@ -20797,12 +20797,12 @@
       </c>
       <c r="B737" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">ativa</t>
         </is>
       </c>
       <c r="C737" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D737" t="inlineStr" s="2">
@@ -20810,13 +20810,13 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E737" s="2"/>
+      <c r="E737" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F737" s="2"/>
-      <c r="G737" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G737" s="2"/>
     </row>
     <row r="738">
       <c r="A738" t="inlineStr" s="2">
@@ -20826,7 +20826,7 @@
       </c>
       <c r="B738" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C738" t="inlineStr" s="2">
@@ -20843,38 +20843,38 @@
       <c r="F738" s="2"/>
       <c r="G738" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="739">
       <c r="A739" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes_execucoes</t>
+          <t xml:space="preserve">automacoes</t>
         </is>
       </c>
       <c r="B739" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacao</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C739" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D739" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E739" s="2"/>
-      <c r="F739" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">automacoes</t>
-        </is>
-      </c>
-      <c r="G739" s="2"/>
+      <c r="F739" s="2"/>
+      <c r="G739" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="740">
       <c r="A740" t="inlineStr" s="2">
@@ -20884,12 +20884,12 @@
       </c>
       <c r="B740" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_execucao</t>
+          <t xml:space="preserve">automacao</t>
         </is>
       </c>
       <c r="C740" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D740" t="inlineStr" s="2">
@@ -20898,7 +20898,11 @@
         </is>
       </c>
       <c r="E740" s="2"/>
-      <c r="F740" s="2"/>
+      <c r="F740" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">automacoes</t>
+        </is>
+      </c>
       <c r="G740" s="2"/>
     </row>
     <row r="741">
@@ -20909,24 +20913,20 @@
       </c>
       <c r="B741" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">sucesso</t>
+          <t xml:space="preserve">data_execucao</t>
         </is>
       </c>
       <c r="C741" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D741" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E741" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E741" s="2"/>
       <c r="F741" s="2"/>
       <c r="G741" s="2"/>
     </row>
@@ -20938,12 +20938,12 @@
       </c>
       <c r="B742" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mensagem</t>
+          <t xml:space="preserve">sucesso</t>
         </is>
       </c>
       <c r="C742" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D742" t="inlineStr" s="2">
@@ -20951,7 +20951,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E742" s="2"/>
+      <c r="E742" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F742" s="2"/>
       <c r="G742" s="2"/>
     </row>
@@ -20963,7 +20967,7 @@
       </c>
       <c r="B743" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">referencia_registro</t>
+          <t xml:space="preserve">mensagem</t>
         </is>
       </c>
       <c r="C743" t="inlineStr" s="2">
@@ -20988,12 +20992,12 @@
       </c>
       <c r="B744" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente</t>
+          <t xml:space="preserve">referencia_registro</t>
         </is>
       </c>
       <c r="C744" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D744" t="inlineStr" s="2">
@@ -21002,11 +21006,7 @@
         </is>
       </c>
       <c r="E744" s="2"/>
-      <c r="F744" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+      <c r="F744" s="2"/>
       <c r="G744" s="2"/>
     </row>
     <row r="745">
@@ -21017,12 +21017,12 @@
       </c>
       <c r="B745" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">dados_execucao</t>
+          <t xml:space="preserve">cliente</t>
         </is>
       </c>
       <c r="C745" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D745" t="inlineStr" s="2">
@@ -21031,12 +21031,12 @@
         </is>
       </c>
       <c r="E745" s="2"/>
-      <c r="F745" s="2"/>
-      <c r="G745" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="F745" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
+      <c r="G745" s="2"/>
     </row>
     <row r="746">
       <c r="A746" t="inlineStr" s="2">
@@ -21046,12 +21046,12 @@
       </c>
       <c r="B746" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">dados_execucao</t>
         </is>
       </c>
       <c r="C746" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D746" t="inlineStr" s="2">
@@ -21063,7 +21063,7 @@
       <c r="F746" s="2"/>
       <c r="G746" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
+          <t xml:space="preserve">Estrutura JSON livre</t>
         </is>
       </c>
     </row>
@@ -21075,7 +21075,7 @@
       </c>
       <c r="B747" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C747" t="inlineStr" s="2">
@@ -21092,38 +21092,38 @@
       <c r="F747" s="2"/>
       <c r="G747" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="748">
       <c r="A748" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">automacoes_execucoes</t>
         </is>
       </c>
       <c r="B748" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C748" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D748" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E748" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">atividade_atrasada | lembrete | sistema</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E748" s="2"/>
       <c r="F748" s="2"/>
-      <c r="G748" s="2"/>
+      <c r="G748" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="749">
       <c r="A749" t="inlineStr" s="2">
@@ -21133,12 +21133,12 @@
       </c>
       <c r="B749" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">tipo</t>
         </is>
       </c>
       <c r="C749" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D749" t="inlineStr" s="2">
@@ -21146,7 +21146,11 @@
           <t xml:space="preserve">Sim</t>
         </is>
       </c>
-      <c r="E749" s="2"/>
+      <c r="E749" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">atividade_atrasada | lembrete | sistema</t>
+        </is>
+      </c>
       <c r="F749" s="2"/>
       <c r="G749" s="2"/>
     </row>
@@ -21158,7 +21162,7 @@
       </c>
       <c r="B750" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mensagem</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C750" t="inlineStr" s="2">
@@ -21168,7 +21172,7 @@
       </c>
       <c r="D750" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E750" s="2"/>
@@ -21183,12 +21187,12 @@
       </c>
       <c r="B751" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">atividade_id</t>
+          <t xml:space="preserve">mensagem</t>
         </is>
       </c>
       <c r="C751" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D751" t="inlineStr" s="2">
@@ -21197,11 +21201,7 @@
         </is>
       </c>
       <c r="E751" s="2"/>
-      <c r="F751" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">atividades</t>
-        </is>
-      </c>
+      <c r="F751" s="2"/>
       <c r="G751" s="2"/>
     </row>
     <row r="752">
@@ -21212,7 +21212,7 @@
       </c>
       <c r="B752" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_id</t>
+          <t xml:space="preserve">atividade_id</t>
         </is>
       </c>
       <c r="C752" t="inlineStr" s="2">
@@ -21228,7 +21228,7 @@
       <c r="E752" s="2"/>
       <c r="F752" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">clientes</t>
+          <t xml:space="preserve">atividades</t>
         </is>
       </c>
       <c r="G752" s="2"/>
@@ -21241,12 +21241,12 @@
       </c>
       <c r="B753" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_nome</t>
+          <t xml:space="preserve">cliente_id</t>
         </is>
       </c>
       <c r="C753" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D753" t="inlineStr" s="2">
@@ -21255,7 +21255,11 @@
         </is>
       </c>
       <c r="E753" s="2"/>
-      <c r="F753" s="2"/>
+      <c r="F753" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G753" s="2"/>
     </row>
     <row r="754">
@@ -21266,12 +21270,12 @@
       </c>
       <c r="B754" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_prevista</t>
+          <t xml:space="preserve">cliente_nome</t>
         </is>
       </c>
       <c r="C754" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D754" t="inlineStr" s="2">
@@ -21291,12 +21295,12 @@
       </c>
       <c r="B755" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">dias_atraso</t>
+          <t xml:space="preserve">data_prevista</t>
         </is>
       </c>
       <c r="C755" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D755" t="inlineStr" s="2">
@@ -21316,12 +21320,12 @@
       </c>
       <c r="B756" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">lida</t>
+          <t xml:space="preserve">dias_atraso</t>
         </is>
       </c>
       <c r="C756" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D756" t="inlineStr" s="2">
@@ -21329,11 +21333,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E756" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E756" s="2"/>
       <c r="F756" s="2"/>
       <c r="G756" s="2"/>
     </row>
@@ -21345,12 +21345,12 @@
       </c>
       <c r="B757" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">lida_em</t>
+          <t xml:space="preserve">lida</t>
         </is>
       </c>
       <c r="C757" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D757" t="inlineStr" s="2">
@@ -21358,7 +21358,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E757" s="2"/>
+      <c r="E757" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F757" s="2"/>
       <c r="G757" s="2"/>
     </row>
@@ -21370,24 +21374,20 @@
       </c>
       <c r="B758" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">lida_em</t>
         </is>
       </c>
       <c r="C758" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D758" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E758" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">ativa | resolvida | arquivada</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E758" s="2"/>
       <c r="F758" s="2"/>
       <c r="G758" s="2"/>
     </row>
@@ -21399,20 +21399,24 @@
       </c>
       <c r="B759" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">resolvida_em</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="C759" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D759" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E759" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E759" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativa | resolvida | arquivada</t>
+        </is>
+      </c>
       <c r="F759" s="2"/>
       <c r="G759" s="2"/>
     </row>
@@ -21424,12 +21428,12 @@
       </c>
       <c r="B760" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">resolvida_em</t>
         </is>
       </c>
       <c r="C760" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D760" t="inlineStr" s="2">
@@ -21439,11 +21443,7 @@
       </c>
       <c r="E760" s="2"/>
       <c r="F760" s="2"/>
-      <c r="G760" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G760" s="2"/>
     </row>
     <row r="761">
       <c r="A761" t="inlineStr" s="2">
@@ -21453,7 +21453,7 @@
       </c>
       <c r="B761" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C761" t="inlineStr" s="2">
@@ -21470,38 +21470,38 @@
       <c r="F761" s="2"/>
       <c r="G761" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="762">
       <c r="A762" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">notificacoes_internas</t>
         </is>
       </c>
       <c r="B762" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_id</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C762" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D762" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E762" s="2"/>
-      <c r="F762" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
-      <c r="G762" s="2"/>
+      <c r="F762" s="2"/>
+      <c r="G762" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="763">
       <c r="A763" t="inlineStr" s="2">
@@ -21511,25 +21511,25 @@
       </c>
       <c r="B763" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_negocio</t>
+          <t xml:space="preserve">cliente_id</t>
         </is>
       </c>
       <c r="C763" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D763" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E763" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">venda usina | bateria | expansão | renovação | serviço | venda bateria</t>
-        </is>
-      </c>
-      <c r="F763" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E763" s="2"/>
+      <c r="F763" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G763" s="2"/>
     </row>
     <row r="764">
@@ -21540,12 +21540,12 @@
       </c>
       <c r="B764" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">valor_estimado</t>
+          <t xml:space="preserve">tipo_negocio</t>
         </is>
       </c>
       <c r="C764" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D764" t="inlineStr" s="2">
@@ -21553,7 +21553,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E764" s="2"/>
+      <c r="E764" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">venda usina | bateria | expansão | renovação | serviço | venda bateria</t>
+        </is>
+      </c>
       <c r="F764" s="2"/>
       <c r="G764" s="2"/>
     </row>
@@ -21565,7 +21569,7 @@
       </c>
       <c r="B765" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">valor_final</t>
+          <t xml:space="preserve">valor_estimado</t>
         </is>
       </c>
       <c r="C765" t="inlineStr" s="2">
@@ -21590,12 +21594,12 @@
       </c>
       <c r="B766" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">etapa_funil</t>
+          <t xml:space="preserve">valor_final</t>
         </is>
       </c>
       <c r="C766" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D766" t="inlineStr" s="2">
@@ -21603,11 +21607,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E766" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">novo lead | qualificado | proposta enviada | negociação | contrato assinado</t>
-        </is>
-      </c>
+      <c r="E766" s="2"/>
       <c r="F766" s="2"/>
       <c r="G766" s="2"/>
     </row>
@@ -21619,12 +21619,12 @@
       </c>
       <c r="B767" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">probabilidade</t>
+          <t xml:space="preserve">etapa_funil</t>
         </is>
       </c>
       <c r="C767" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D767" t="inlineStr" s="2">
@@ -21632,7 +21632,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E767" s="2"/>
+      <c r="E767" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">novo lead | qualificado | proposta enviada | negociação | contrato assinado</t>
+        </is>
+      </c>
       <c r="F767" s="2"/>
       <c r="G767" s="2"/>
     </row>
@@ -21644,12 +21648,12 @@
       </c>
       <c r="B768" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_previsao_fechamento</t>
+          <t xml:space="preserve">probabilidade</t>
         </is>
       </c>
       <c r="C768" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D768" t="inlineStr" s="2">
@@ -21669,7 +21673,7 @@
       </c>
       <c r="B769" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_fechamento</t>
+          <t xml:space="preserve">data_previsao_fechamento</t>
         </is>
       </c>
       <c r="C769" t="inlineStr" s="2">
@@ -21694,12 +21698,12 @@
       </c>
       <c r="B770" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">data_fechamento</t>
         </is>
       </c>
       <c r="C770" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D770" t="inlineStr" s="2">
@@ -21707,11 +21711,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E770" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">em andamento | ganho | perdido</t>
-        </is>
-      </c>
+      <c r="E770" s="2"/>
       <c r="F770" s="2"/>
       <c r="G770" s="2"/>
     </row>
@@ -21723,12 +21723,12 @@
       </c>
       <c r="B771" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">motivo_perda</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="C771" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D771" t="inlineStr" s="2">
@@ -21736,7 +21736,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E771" s="2"/>
+      <c r="E771" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">em andamento | ganho | perdido</t>
+        </is>
+      </c>
       <c r="F771" s="2"/>
       <c r="G771" s="2"/>
     </row>
@@ -21748,12 +21752,12 @@
       </c>
       <c r="B772" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">reabertura</t>
+          <t xml:space="preserve">motivo_perda</t>
         </is>
       </c>
       <c r="C772" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D772" t="inlineStr" s="2">
@@ -21761,11 +21765,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E772" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E772" s="2"/>
       <c r="F772" s="2"/>
       <c r="G772" s="2"/>
     </row>
@@ -21777,12 +21777,12 @@
       </c>
       <c r="B773" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">motivo_reabertura</t>
+          <t xml:space="preserve">reabertura</t>
         </is>
       </c>
       <c r="C773" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D773" t="inlineStr" s="2">
@@ -21790,7 +21790,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E773" s="2"/>
+      <c r="E773" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F773" s="2"/>
       <c r="G773" s="2"/>
     </row>
@@ -21802,7 +21806,7 @@
       </c>
       <c r="B774" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">condicao_pagamento</t>
+          <t xml:space="preserve">motivo_reabertura</t>
         </is>
       </c>
       <c r="C774" t="inlineStr" s="2">
@@ -21827,12 +21831,12 @@
       </c>
       <c r="B775" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">condicao_pagamento</t>
         </is>
       </c>
       <c r="C775" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D775" t="inlineStr" s="2">
@@ -21842,11 +21846,7 @@
       </c>
       <c r="E775" s="2"/>
       <c r="F775" s="2"/>
-      <c r="G775" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G775" s="2"/>
     </row>
     <row r="776">
       <c r="A776" t="inlineStr" s="2">
@@ -21856,7 +21856,7 @@
       </c>
       <c r="B776" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C776" t="inlineStr" s="2">
@@ -21873,7 +21873,7 @@
       <c r="F776" s="2"/>
       <c r="G776" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
@@ -21885,12 +21885,12 @@
       </c>
       <c r="B777" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_venda</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C777" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D777" t="inlineStr" s="2">
@@ -21898,13 +21898,13 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E777" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Energia Solar | O&amp;M (Operação e Manutenção) | Baterias | Carregadores Veículos Elétricos</t>
-        </is>
-      </c>
+      <c r="E777" s="2"/>
       <c r="F777" s="2"/>
-      <c r="G777" s="2"/>
+      <c r="G777" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="778">
       <c r="A778" t="inlineStr" s="2">
@@ -21914,12 +21914,12 @@
       </c>
       <c r="B778" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">tipo_venda</t>
         </is>
       </c>
       <c r="C778" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D778" t="inlineStr" s="2">
@@ -21927,7 +21927,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E778" s="2"/>
+      <c r="E778" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Energia Solar | O&amp;M (Operação e Manutenção) | Baterias | Carregadores Veículos Elétricos</t>
+        </is>
+      </c>
       <c r="F778" s="2"/>
       <c r="G778" s="2"/>
     </row>
@@ -21939,12 +21943,12 @@
       </c>
       <c r="B779" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">valor</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C779" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D779" t="inlineStr" s="2">
@@ -21964,12 +21968,12 @@
       </c>
       <c r="B780" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">consultor_responsavel</t>
+          <t xml:space="preserve">valor</t>
         </is>
       </c>
       <c r="C780" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D780" t="inlineStr" s="2">
@@ -21978,11 +21982,7 @@
         </is>
       </c>
       <c r="E780" s="2"/>
-      <c r="F780" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">users</t>
-        </is>
-      </c>
+      <c r="F780" s="2"/>
       <c r="G780" s="2"/>
     </row>
     <row r="781">
@@ -21993,12 +21993,12 @@
       </c>
       <c r="B781" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">recorrencia_mensal</t>
+          <t xml:space="preserve">consultor_responsavel</t>
         </is>
       </c>
       <c r="C781" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D781" t="inlineStr" s="2">
@@ -22006,36 +22006,40 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E781" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
-      <c r="F781" s="2"/>
+      <c r="E781" s="2"/>
+      <c r="F781" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">users</t>
+        </is>
+      </c>
       <c r="G781" s="2"/>
     </row>
     <row r="782">
       <c r="A782" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">analises_fatura</t>
+          <t xml:space="preserve">negocios</t>
         </is>
       </c>
       <c r="B782" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">token</t>
+          <t xml:space="preserve">recorrencia_mensal</t>
         </is>
       </c>
       <c r="C782" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D782" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E782" s="2"/>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E782" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F782" s="2"/>
       <c r="G782" s="2"/>
     </row>
@@ -22047,25 +22051,21 @@
       </c>
       <c r="B783" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_id</t>
+          <t xml:space="preserve">token</t>
         </is>
       </c>
       <c r="C783" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D783" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E783" s="2"/>
-      <c r="F783" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+      <c r="F783" s="2"/>
       <c r="G783" s="2"/>
     </row>
     <row r="784">
@@ -22076,12 +22076,12 @@
       </c>
       <c r="B784" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_nome</t>
+          <t xml:space="preserve">cliente_id</t>
         </is>
       </c>
       <c r="C784" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D784" t="inlineStr" s="2">
@@ -22090,7 +22090,11 @@
         </is>
       </c>
       <c r="E784" s="2"/>
-      <c r="F784" s="2"/>
+      <c r="F784" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G784" s="2"/>
     </row>
     <row r="785">
@@ -22101,7 +22105,7 @@
       </c>
       <c r="B785" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">uc</t>
+          <t xml:space="preserve">cliente_nome</t>
         </is>
       </c>
       <c r="C785" t="inlineStr" s="2">
@@ -22126,7 +22130,7 @@
       </c>
       <c r="B786" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">competencia</t>
+          <t xml:space="preserve">uc</t>
         </is>
       </c>
       <c r="C786" t="inlineStr" s="2">
@@ -22151,7 +22155,7 @@
       </c>
       <c r="B787" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">vencimento</t>
+          <t xml:space="preserve">competencia</t>
         </is>
       </c>
       <c r="C787" t="inlineStr" s="2">
@@ -22176,12 +22180,12 @@
       </c>
       <c r="B788" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">total_pagar</t>
+          <t xml:space="preserve">vencimento</t>
         </is>
       </c>
       <c r="C788" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D788" t="inlineStr" s="2">
@@ -22201,7 +22205,7 @@
       </c>
       <c r="B789" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">consumo_kwh</t>
+          <t xml:space="preserve">total_pagar</t>
         </is>
       </c>
       <c r="C789" t="inlineStr" s="2">
@@ -22226,7 +22230,7 @@
       </c>
       <c r="B790" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">energia_injetada_kwh</t>
+          <t xml:space="preserve">consumo_kwh</t>
         </is>
       </c>
       <c r="C790" t="inlineStr" s="2">
@@ -22251,7 +22255,7 @@
       </c>
       <c r="B791" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">creditos_compensados_kwh</t>
+          <t xml:space="preserve">energia_injetada_kwh</t>
         </is>
       </c>
       <c r="C791" t="inlineStr" s="2">
@@ -22276,7 +22280,7 @@
       </c>
       <c r="B792" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">saldo_energia_kwh</t>
+          <t xml:space="preserve">creditos_compensados_kwh</t>
         </is>
       </c>
       <c r="C792" t="inlineStr" s="2">
@@ -22301,7 +22305,7 @@
       </c>
       <c r="B793" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">saldo_expirar_kwh</t>
+          <t xml:space="preserve">saldo_energia_kwh</t>
         </is>
       </c>
       <c r="C793" t="inlineStr" s="2">
@@ -22326,7 +22330,7 @@
       </c>
       <c r="B794" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">economia_estimada_rs</t>
+          <t xml:space="preserve">saldo_expirar_kwh</t>
         </is>
       </c>
       <c r="C794" t="inlineStr" s="2">
@@ -22351,12 +22355,12 @@
       </c>
       <c r="B795" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">papel_uc</t>
+          <t xml:space="preserve">economia_estimada_rs</t>
         </is>
       </c>
       <c r="C795" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D795" t="inlineStr" s="2">
@@ -22376,12 +22380,12 @@
       </c>
       <c r="B796" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">arquivos_nomes</t>
+          <t xml:space="preserve">papel_uc</t>
         </is>
       </c>
       <c r="C796" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D796" t="inlineStr" s="2">
@@ -22391,11 +22395,7 @@
       </c>
       <c r="E796" s="2"/>
       <c r="F796" s="2"/>
-      <c r="G796" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="G796" s="2"/>
     </row>
     <row r="797">
       <c r="A797" t="inlineStr" s="2">
@@ -22405,7 +22405,7 @@
       </c>
       <c r="B797" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">dados_completos</t>
+          <t xml:space="preserve">arquivos_nomes</t>
         </is>
       </c>
       <c r="C797" t="inlineStr" s="2">
@@ -22434,12 +22434,12 @@
       </c>
       <c r="B798" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">atividade_id</t>
+          <t xml:space="preserve">dados_completos</t>
         </is>
       </c>
       <c r="C798" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D798" t="inlineStr" s="2">
@@ -22449,7 +22449,11 @@
       </c>
       <c r="E798" s="2"/>
       <c r="F798" s="2"/>
-      <c r="G798" s="2"/>
+      <c r="G798" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Estrutura JSON livre</t>
+        </is>
+      </c>
     </row>
     <row r="799">
       <c r="A799" t="inlineStr" s="2">
@@ -22459,12 +22463,12 @@
       </c>
       <c r="B799" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">whatsapp_enviado</t>
+          <t xml:space="preserve">atividade_id</t>
         </is>
       </c>
       <c r="C799" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D799" t="inlineStr" s="2">
@@ -22472,11 +22476,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E799" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E799" s="2"/>
       <c r="F799" s="2"/>
       <c r="G799" s="2"/>
     </row>
@@ -22488,12 +22488,12 @@
       </c>
       <c r="B800" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">whatsapp_enviado_em</t>
+          <t xml:space="preserve">whatsapp_enviado</t>
         </is>
       </c>
       <c r="C800" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D800" t="inlineStr" s="2">
@@ -22501,7 +22501,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E800" s="2"/>
+      <c r="E800" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F800" s="2"/>
       <c r="G800" s="2"/>
     </row>
@@ -22513,12 +22517,12 @@
       </c>
       <c r="B801" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">whatsapp_enviado_em</t>
         </is>
       </c>
       <c r="C801" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D801" t="inlineStr" s="2">
@@ -22528,11 +22532,7 @@
       </c>
       <c r="E801" s="2"/>
       <c r="F801" s="2"/>
-      <c r="G801" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G801" s="2"/>
     </row>
     <row r="802">
       <c r="A802" t="inlineStr" s="2">
@@ -22542,7 +22542,7 @@
       </c>
       <c r="B802" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C802" t="inlineStr" s="2">
@@ -22559,34 +22559,38 @@
       <c r="F802" s="2"/>
       <c r="G802" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="803">
       <c r="A803" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">knowledge_categories</t>
+          <t xml:space="preserve">analises_fatura</t>
         </is>
       </c>
       <c r="B803" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C803" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D803" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E803" s="2"/>
       <c r="F803" s="2"/>
-      <c r="G803" s="2"/>
+      <c r="G803" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="804">
       <c r="A804" t="inlineStr" s="2">
@@ -22596,7 +22600,7 @@
       </c>
       <c r="B804" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">descricao</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C804" t="inlineStr" s="2">
@@ -22606,7 +22610,7 @@
       </c>
       <c r="D804" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E804" s="2"/>
@@ -22621,7 +22625,7 @@
       </c>
       <c r="B805" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">icone</t>
+          <t xml:space="preserve">descricao</t>
         </is>
       </c>
       <c r="C805" t="inlineStr" s="2">
@@ -22646,12 +22650,12 @@
       </c>
       <c r="B806" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ordem</t>
+          <t xml:space="preserve">icone</t>
         </is>
       </c>
       <c r="C806" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D806" t="inlineStr" s="2">
@@ -22671,12 +22675,12 @@
       </c>
       <c r="B807" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">ordem</t>
         </is>
       </c>
       <c r="C807" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D807" t="inlineStr" s="2">
@@ -22686,11 +22690,7 @@
       </c>
       <c r="E807" s="2"/>
       <c r="F807" s="2"/>
-      <c r="G807" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G807" s="2"/>
     </row>
     <row r="808">
       <c r="A808" t="inlineStr" s="2">
@@ -22700,7 +22700,7 @@
       </c>
       <c r="B808" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C808" t="inlineStr" s="2">
@@ -22717,38 +22717,38 @@
       <c r="F808" s="2"/>
       <c r="G808" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="809">
       <c r="A809" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">knowledge_articles</t>
+          <t xml:space="preserve">knowledge_categories</t>
         </is>
       </c>
       <c r="B809" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">categoria_id</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C809" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D809" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E809" s="2"/>
-      <c r="F809" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">knowledge_categories</t>
-        </is>
-      </c>
-      <c r="G809" s="2"/>
+      <c r="F809" s="2"/>
+      <c r="G809" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="810">
       <c r="A810" t="inlineStr" s="2">
@@ -22758,12 +22758,12 @@
       </c>
       <c r="B810" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">categoria_id</t>
         </is>
       </c>
       <c r="C810" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D810" t="inlineStr" s="2">
@@ -22772,7 +22772,11 @@
         </is>
       </c>
       <c r="E810" s="2"/>
-      <c r="F810" s="2"/>
+      <c r="F810" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_categories</t>
+        </is>
+      </c>
       <c r="G810" s="2"/>
     </row>
     <row r="811">
@@ -22783,7 +22787,7 @@
       </c>
       <c r="B811" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">conteudo</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C811" t="inlineStr" s="2">
@@ -22808,7 +22812,7 @@
       </c>
       <c r="B812" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">texto_extraido</t>
+          <t xml:space="preserve">conteudo</t>
         </is>
       </c>
       <c r="C812" t="inlineStr" s="2">
@@ -22818,7 +22822,7 @@
       </c>
       <c r="D812" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E812" s="2"/>
@@ -22833,12 +22837,12 @@
       </c>
       <c r="B813" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">anexos</t>
+          <t xml:space="preserve">texto_extraido</t>
         </is>
       </c>
       <c r="C813" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">file</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D813" t="inlineStr" s="2">
@@ -22848,11 +22852,7 @@
       </c>
       <c r="E813" s="2"/>
       <c r="F813" s="2"/>
-      <c r="G813" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
-        </is>
-      </c>
+      <c r="G813" s="2"/>
     </row>
     <row r="814">
       <c r="A814" t="inlineStr" s="2">
@@ -22862,12 +22862,12 @@
       </c>
       <c r="B814" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">criado_por</t>
+          <t xml:space="preserve">anexos</t>
         </is>
       </c>
       <c r="C814" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="D814" t="inlineStr" s="2">
@@ -22876,12 +22876,12 @@
         </is>
       </c>
       <c r="E814" s="2"/>
-      <c r="F814" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">users</t>
-        </is>
-      </c>
-      <c r="G814" s="2"/>
+      <c r="F814" s="2"/>
+      <c r="G814" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
+        </is>
+      </c>
     </row>
     <row r="815">
       <c r="A815" t="inlineStr" s="2">
@@ -22891,12 +22891,12 @@
       </c>
       <c r="B815" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autor_nome</t>
+          <t xml:space="preserve">criado_por</t>
         </is>
       </c>
       <c r="C815" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D815" t="inlineStr" s="2">
@@ -22905,7 +22905,11 @@
         </is>
       </c>
       <c r="E815" s="2"/>
-      <c r="F815" s="2"/>
+      <c r="F815" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">users</t>
+        </is>
+      </c>
       <c r="G815" s="2"/>
     </row>
     <row r="816">
@@ -22916,7 +22920,7 @@
       </c>
       <c r="B816" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tags</t>
+          <t xml:space="preserve">autor_nome</t>
         </is>
       </c>
       <c r="C816" t="inlineStr" s="2">
@@ -22941,12 +22945,12 @@
       </c>
       <c r="B817" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">tags</t>
         </is>
       </c>
       <c r="C817" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D817" t="inlineStr" s="2">
@@ -22956,11 +22960,7 @@
       </c>
       <c r="E817" s="2"/>
       <c r="F817" s="2"/>
-      <c r="G817" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G817" s="2"/>
     </row>
     <row r="818">
       <c r="A818" t="inlineStr" s="2">
@@ -22970,7 +22970,7 @@
       </c>
       <c r="B818" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C818" t="inlineStr" s="2">
@@ -22987,38 +22987,38 @@
       <c r="F818" s="2"/>
       <c r="G818" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="819">
       <c r="A819" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contratos_usinas</t>
+          <t xml:space="preserve">knowledge_articles</t>
         </is>
       </c>
       <c r="B819" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contrato_id</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C819" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D819" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E819" s="2"/>
-      <c r="F819" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">contratos_om</t>
-        </is>
-      </c>
-      <c r="G819" s="2"/>
+      <c r="F819" s="2"/>
+      <c r="G819" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="820">
       <c r="A820" t="inlineStr" s="2">
@@ -23028,7 +23028,7 @@
       </c>
       <c r="B820" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">usina_id</t>
+          <t xml:space="preserve">contrato_id</t>
         </is>
       </c>
       <c r="C820" t="inlineStr" s="2">
@@ -23044,7 +23044,7 @@
       <c r="E820" s="2"/>
       <c r="F820" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">usinas</t>
+          <t xml:space="preserve">contratos_om</t>
         </is>
       </c>
       <c r="G820" s="2"/>
@@ -23057,25 +23057,25 @@
       </c>
       <c r="B821" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ativo</t>
+          <t xml:space="preserve">usina_id</t>
         </is>
       </c>
       <c r="C821" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D821" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E821" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
-      <c r="F821" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E821" s="2"/>
+      <c r="F821" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usinas</t>
+        </is>
+      </c>
       <c r="G821" s="2"/>
     </row>
     <row r="822">
@@ -23086,12 +23086,12 @@
       </c>
       <c r="B822" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_vinculo</t>
+          <t xml:space="preserve">ativo</t>
         </is>
       </c>
       <c r="C822" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D822" t="inlineStr" s="2">
@@ -23099,7 +23099,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E822" s="2"/>
+      <c r="E822" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F822" s="2"/>
       <c r="G822" s="2"/>
     </row>
@@ -23111,7 +23115,7 @@
       </c>
       <c r="B823" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_desvinculo</t>
+          <t xml:space="preserve">data_vinculo</t>
         </is>
       </c>
       <c r="C823" t="inlineStr" s="2">
@@ -23136,12 +23140,12 @@
       </c>
       <c r="B824" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">observacoes</t>
+          <t xml:space="preserve">data_desvinculo</t>
         </is>
       </c>
       <c r="C824" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D824" t="inlineStr" s="2">
@@ -23161,12 +23165,12 @@
       </c>
       <c r="B825" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">observacoes</t>
         </is>
       </c>
       <c r="C825" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D825" t="inlineStr" s="2">
@@ -23176,11 +23180,7 @@
       </c>
       <c r="E825" s="2"/>
       <c r="F825" s="2"/>
-      <c r="G825" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G825" s="2"/>
     </row>
     <row r="826">
       <c r="A826" t="inlineStr" s="2">
@@ -23190,7 +23190,7 @@
       </c>
       <c r="B826" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C826" t="inlineStr" s="2">
@@ -23207,24 +23207,24 @@
       <c r="F826" s="2"/>
       <c r="G826" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="827">
       <c r="A827" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ativos</t>
+          <t xml:space="preserve">contratos_usinas</t>
         </is>
       </c>
       <c r="B827" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">usina_id</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C827" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D827" t="inlineStr" s="2">
@@ -23233,12 +23233,12 @@
         </is>
       </c>
       <c r="E827" s="2"/>
-      <c r="F827" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">usinas</t>
-        </is>
-      </c>
-      <c r="G827" s="2"/>
+      <c r="F827" s="2"/>
+      <c r="G827" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="828">
       <c r="A828" t="inlineStr" s="2">
@@ -23248,25 +23248,25 @@
       </c>
       <c r="B828" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo</t>
+          <t xml:space="preserve">usina_id</t>
         </is>
       </c>
       <c r="C828" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D828" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E828" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">inversor | placa_solar | bateria | string_box | outros</t>
-        </is>
-      </c>
-      <c r="F828" s="2"/>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E828" s="2"/>
+      <c r="F828" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usinas</t>
+        </is>
+      </c>
       <c r="G828" s="2"/>
     </row>
     <row r="829">
@@ -23277,20 +23277,24 @@
       </c>
       <c r="B829" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_outro_descricao</t>
+          <t xml:space="preserve">tipo</t>
         </is>
       </c>
       <c r="C829" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D829" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E829" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E829" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">inversor | placa_solar | bateria | string_box | outros</t>
+        </is>
+      </c>
       <c r="F829" s="2"/>
       <c r="G829" s="2"/>
     </row>
@@ -23302,7 +23306,7 @@
       </c>
       <c r="B830" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fabricante</t>
+          <t xml:space="preserve">tipo_outro_descricao</t>
         </is>
       </c>
       <c r="C830" t="inlineStr" s="2">
@@ -23312,7 +23316,7 @@
       </c>
       <c r="D830" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E830" s="2"/>
@@ -23327,7 +23331,7 @@
       </c>
       <c r="B831" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">modelo</t>
+          <t xml:space="preserve">fabricante</t>
         </is>
       </c>
       <c r="C831" t="inlineStr" s="2">
@@ -23352,7 +23356,7 @@
       </c>
       <c r="B832" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">numero_serie</t>
+          <t xml:space="preserve">modelo</t>
         </is>
       </c>
       <c r="C832" t="inlineStr" s="2">
@@ -23362,7 +23366,7 @@
       </c>
       <c r="D832" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E832" s="2"/>
@@ -23377,12 +23381,12 @@
       </c>
       <c r="B833" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_instalacao</t>
+          <t xml:space="preserve">numero_serie</t>
         </is>
       </c>
       <c r="C833" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D833" t="inlineStr" s="2">
@@ -23402,7 +23406,7 @@
       </c>
       <c r="B834" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_fim_garantia</t>
+          <t xml:space="preserve">data_instalacao</t>
         </is>
       </c>
       <c r="C834" t="inlineStr" s="2">
@@ -23427,12 +23431,12 @@
       </c>
       <c r="B835" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">responsavel_id</t>
+          <t xml:space="preserve">data_fim_garantia</t>
         </is>
       </c>
       <c r="C835" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D835" t="inlineStr" s="2">
@@ -23441,11 +23445,7 @@
         </is>
       </c>
       <c r="E835" s="2"/>
-      <c r="F835" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">users</t>
-        </is>
-      </c>
+      <c r="F835" s="2"/>
       <c r="G835" s="2"/>
     </row>
     <row r="836">
@@ -23456,12 +23456,12 @@
       </c>
       <c r="B836" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">observacoes</t>
+          <t xml:space="preserve">responsavel_id</t>
         </is>
       </c>
       <c r="C836" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D836" t="inlineStr" s="2">
@@ -23470,7 +23470,11 @@
         </is>
       </c>
       <c r="E836" s="2"/>
-      <c r="F836" s="2"/>
+      <c r="F836" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">users</t>
+        </is>
+      </c>
       <c r="G836" s="2"/>
     </row>
     <row r="837">
@@ -23481,12 +23485,12 @@
       </c>
       <c r="B837" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">status_operacional</t>
+          <t xml:space="preserve">observacoes</t>
         </is>
       </c>
       <c r="C837" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D837" t="inlineStr" s="2">
@@ -23494,11 +23498,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E837" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">operacional | em_alerta | manutencao | desativado</t>
-        </is>
-      </c>
+      <c r="E837" s="2"/>
       <c r="F837" s="2"/>
       <c r="G837" s="2"/>
     </row>
@@ -23510,12 +23510,12 @@
       </c>
       <c r="B838" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">status_operacional</t>
         </is>
       </c>
       <c r="C838" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D838" t="inlineStr" s="2">
@@ -23523,13 +23523,13 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E838" s="2"/>
+      <c r="E838" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">operacional | em_alerta | manutencao | desativado</t>
+        </is>
+      </c>
       <c r="F838" s="2"/>
-      <c r="G838" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G838" s="2"/>
     </row>
     <row r="839">
       <c r="A839" t="inlineStr" s="2">
@@ -23539,7 +23539,7 @@
       </c>
       <c r="B839" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C839" t="inlineStr" s="2">
@@ -23556,7 +23556,7 @@
       <c r="F839" s="2"/>
       <c r="G839" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
@@ -23568,12 +23568,12 @@
       </c>
       <c r="B840" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">chave_importacao</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C840" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D840" t="inlineStr" s="2">
@@ -23583,7 +23583,11 @@
       </c>
       <c r="E840" s="2"/>
       <c r="F840" s="2"/>
-      <c r="G840" s="2"/>
+      <c r="G840" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="841">
       <c r="A841" t="inlineStr" s="2">
@@ -23593,7 +23597,7 @@
       </c>
       <c r="B841" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_inversor_id</t>
+          <t xml:space="preserve">chave_importacao</t>
         </is>
       </c>
       <c r="C841" t="inlineStr" s="2">
@@ -23613,12 +23617,12 @@
     <row r="842">
       <c r="A842" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contatos</t>
+          <t xml:space="preserve">ativos</t>
         </is>
       </c>
       <c r="B842" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">nome</t>
+          <t xml:space="preserve">cliente_inversor_id</t>
         </is>
       </c>
       <c r="C842" t="inlineStr" s="2">
@@ -23628,7 +23632,7 @@
       </c>
       <c r="D842" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E842" s="2"/>
@@ -23643,7 +23647,7 @@
       </c>
       <c r="B843" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">telefone</t>
+          <t xml:space="preserve">nome</t>
         </is>
       </c>
       <c r="C843" t="inlineStr" s="2">
@@ -23653,7 +23657,7 @@
       </c>
       <c r="D843" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E843" s="2"/>
@@ -23668,7 +23672,7 @@
       </c>
       <c r="B844" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">whatsapp</t>
+          <t xml:space="preserve">telefone</t>
         </is>
       </c>
       <c r="C844" t="inlineStr" s="2">
@@ -23693,12 +23697,12 @@
       </c>
       <c r="B845" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">email</t>
+          <t xml:space="preserve">whatsapp</t>
         </is>
       </c>
       <c r="C845" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">email</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D845" t="inlineStr" s="2">
@@ -23718,12 +23722,12 @@
       </c>
       <c r="B846" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">papel</t>
+          <t xml:space="preserve">email</t>
         </is>
       </c>
       <c r="C846" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">email</t>
         </is>
       </c>
       <c r="D846" t="inlineStr" s="2">
@@ -23731,11 +23735,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E846" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">cliente | lead | fornecedor | tecnico | parceiro | familiar | responsavel | financeiro | outro</t>
-        </is>
-      </c>
+      <c r="E846" s="2"/>
       <c r="F846" s="2"/>
       <c r="G846" s="2"/>
     </row>
@@ -23747,12 +23747,12 @@
       </c>
       <c r="B847" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cargo</t>
+          <t xml:space="preserve">papel</t>
         </is>
       </c>
       <c r="C847" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D847" t="inlineStr" s="2">
@@ -23760,7 +23760,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E847" s="2"/>
+      <c r="E847" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">cliente | lead | fornecedor | tecnico | parceiro | familiar | responsavel | financeiro | outro</t>
+        </is>
+      </c>
       <c r="F847" s="2"/>
       <c r="G847" s="2"/>
     </row>
@@ -23772,7 +23776,7 @@
       </c>
       <c r="B848" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">observacoes</t>
+          <t xml:space="preserve">cargo</t>
         </is>
       </c>
       <c r="C848" t="inlineStr" s="2">
@@ -23797,12 +23801,12 @@
       </c>
       <c r="B849" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">clientes_vinculados</t>
+          <t xml:space="preserve">observacoes</t>
         </is>
       </c>
       <c r="C849" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D849" t="inlineStr" s="2">
@@ -23811,11 +23815,7 @@
         </is>
       </c>
       <c r="E849" s="2"/>
-      <c r="F849" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+      <c r="F849" s="2"/>
       <c r="G849" s="2"/>
     </row>
     <row r="850">
@@ -23826,7 +23826,7 @@
       </c>
       <c r="B850" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios_vinculados</t>
+          <t xml:space="preserve">clientes_vinculados</t>
         </is>
       </c>
       <c r="C850" t="inlineStr" s="2">
@@ -23842,7 +23842,7 @@
       <c r="E850" s="2"/>
       <c r="F850" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">clientes</t>
         </is>
       </c>
       <c r="G850" s="2"/>
@@ -23855,12 +23855,12 @@
       </c>
       <c r="B851" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">conversa_id</t>
+          <t xml:space="preserve">negocios_vinculados</t>
         </is>
       </c>
       <c r="C851" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D851" t="inlineStr" s="2">
@@ -23869,7 +23869,11 @@
         </is>
       </c>
       <c r="E851" s="2"/>
-      <c r="F851" s="2"/>
+      <c r="F851" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
       <c r="G851" s="2"/>
     </row>
     <row r="852">
@@ -23880,7 +23884,7 @@
       </c>
       <c r="B852" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">origem_registro</t>
+          <t xml:space="preserve">conversa_id</t>
         </is>
       </c>
       <c r="C852" t="inlineStr" s="2">
@@ -23905,12 +23909,12 @@
       </c>
       <c r="B853" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">origem_registro</t>
         </is>
       </c>
       <c r="C853" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D853" t="inlineStr" s="2">
@@ -23920,11 +23924,7 @@
       </c>
       <c r="E853" s="2"/>
       <c r="F853" s="2"/>
-      <c r="G853" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G853" s="2"/>
     </row>
     <row r="854">
       <c r="A854" t="inlineStr" s="2">
@@ -23934,7 +23934,7 @@
       </c>
       <c r="B854" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C854" t="inlineStr" s="2">
@@ -23951,38 +23951,38 @@
       <c r="F854" s="2"/>
       <c r="G854" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="855">
       <c r="A855" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">usina_equipamentos</t>
+          <t xml:space="preserve">contatos</t>
         </is>
       </c>
       <c r="B855" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">usina_id</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C855" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D855" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E855" s="2"/>
-      <c r="F855" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">usinas</t>
-        </is>
-      </c>
-      <c r="G855" s="2"/>
+      <c r="F855" s="2"/>
+      <c r="G855" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="856">
       <c r="A856" t="inlineStr" s="2">
@@ -23992,7 +23992,7 @@
       </c>
       <c r="B856" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">equipamento_id</t>
+          <t xml:space="preserve">usina_id</t>
         </is>
       </c>
       <c r="C856" t="inlineStr" s="2">
@@ -24008,7 +24008,7 @@
       <c r="E856" s="2"/>
       <c r="F856" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">equipamentos</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="G856" s="2"/>
@@ -24021,21 +24021,25 @@
       </c>
       <c r="B857" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">quantidade</t>
+          <t xml:space="preserve">equipamento_id</t>
         </is>
       </c>
       <c r="C857" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D857" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E857" s="2"/>
-      <c r="F857" s="2"/>
+      <c r="F857" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">equipamentos</t>
+        </is>
+      </c>
       <c r="G857" s="2"/>
     </row>
     <row r="858">
@@ -24046,12 +24050,12 @@
       </c>
       <c r="B858" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">numero_serie</t>
+          <t xml:space="preserve">quantidade</t>
         </is>
       </c>
       <c r="C858" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D858" t="inlineStr" s="2">
@@ -24071,7 +24075,7 @@
       </c>
       <c r="B859" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">observacoes</t>
+          <t xml:space="preserve">numero_serie</t>
         </is>
       </c>
       <c r="C859" t="inlineStr" s="2">
@@ -24096,12 +24100,12 @@
       </c>
       <c r="B860" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">observacoes</t>
         </is>
       </c>
       <c r="C860" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D860" t="inlineStr" s="2">
@@ -24111,11 +24115,7 @@
       </c>
       <c r="E860" s="2"/>
       <c r="F860" s="2"/>
-      <c r="G860" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G860" s="2"/>
     </row>
     <row r="861">
       <c r="A861" t="inlineStr" s="2">
@@ -24125,7 +24125,7 @@
       </c>
       <c r="B861" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C861" t="inlineStr" s="2">
@@ -24141,6 +24141,35 @@
       <c r="E861" s="2"/>
       <c r="F861" s="2"/>
       <c r="G861" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usina_equipamentos</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">updated</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D862" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E862" s="2"/>
+      <c r="F862" s="2"/>
+      <c r="G862" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
         </is>

</xml_diff>

<commit_message>
feat(usinas): opcao de adicionar documento aos existentes vs sobrescrever na ficha da usina
</commit_message>
<xml_diff>
--- a/public/schema-delfos-solar.xlsx
+++ b/public/schema-delfos-solar.xlsx
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="C31" s="2">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D31" t="inlineStr" s="2">
         <is>
@@ -1421,7 +1421,7 @@
         </is>
       </c>
       <c r="C48" s="2">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="D48" s="2"/>
       <c r="E48" s="2">
@@ -19338,31 +19338,31 @@
     <row r="683">
       <c r="A683" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contatos_adicionais</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="B683" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente</t>
+          <t xml:space="preserve">documentos_usina</t>
         </is>
       </c>
       <c r="C683" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D683" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E683" s="2"/>
-      <c r="F683" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
-      <c r="G683" s="2"/>
+      <c r="F683" s="2"/>
+      <c r="G683" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Estrutura JSON livre</t>
+        </is>
+      </c>
     </row>
     <row r="684">
       <c r="A684" t="inlineStr" s="2">
@@ -19372,12 +19372,12 @@
       </c>
       <c r="B684" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">nome</t>
+          <t xml:space="preserve">cliente</t>
         </is>
       </c>
       <c r="C684" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D684" t="inlineStr" s="2">
@@ -19386,7 +19386,11 @@
         </is>
       </c>
       <c r="E684" s="2"/>
-      <c r="F684" s="2"/>
+      <c r="F684" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G684" s="2"/>
     </row>
     <row r="685">
@@ -19397,7 +19401,7 @@
       </c>
       <c r="B685" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cargo</t>
+          <t xml:space="preserve">nome</t>
         </is>
       </c>
       <c r="C685" t="inlineStr" s="2">
@@ -19407,7 +19411,7 @@
       </c>
       <c r="D685" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E685" s="2"/>
@@ -19422,7 +19426,7 @@
       </c>
       <c r="B686" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">telefone</t>
+          <t xml:space="preserve">cargo</t>
         </is>
       </c>
       <c r="C686" t="inlineStr" s="2">
@@ -19447,7 +19451,7 @@
       </c>
       <c r="B687" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">email</t>
+          <t xml:space="preserve">telefone</t>
         </is>
       </c>
       <c r="C687" t="inlineStr" s="2">
@@ -19472,12 +19476,12 @@
       </c>
       <c r="B688" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">email</t>
         </is>
       </c>
       <c r="C688" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D688" t="inlineStr" s="2">
@@ -19487,11 +19491,7 @@
       </c>
       <c r="E688" s="2"/>
       <c r="F688" s="2"/>
-      <c r="G688" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G688" s="2"/>
     </row>
     <row r="689">
       <c r="A689" t="inlineStr" s="2">
@@ -19501,7 +19501,7 @@
       </c>
       <c r="B689" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C689" t="inlineStr" s="2">
@@ -19518,7 +19518,7 @@
       <c r="F689" s="2"/>
       <c r="G689" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
@@ -19530,12 +19530,12 @@
       </c>
       <c r="B690" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">papel</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C690" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D690" t="inlineStr" s="2">
@@ -19543,13 +19543,13 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E690" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">principal | financeiro | tecnico | responsavel | outro</t>
-        </is>
-      </c>
+      <c r="E690" s="2"/>
       <c r="F690" s="2"/>
-      <c r="G690" s="2"/>
+      <c r="G690" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="691">
       <c r="A691" t="inlineStr" s="2">
@@ -19559,12 +19559,12 @@
       </c>
       <c r="B691" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">is_whatsapp</t>
+          <t xml:space="preserve">papel</t>
         </is>
       </c>
       <c r="C691" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D691" t="inlineStr" s="2">
@@ -19574,7 +19574,7 @@
       </c>
       <c r="E691" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">true / false</t>
+          <t xml:space="preserve">principal | financeiro | tecnico | responsavel | outro</t>
         </is>
       </c>
       <c r="F691" s="2"/>
@@ -19588,7 +19588,7 @@
       </c>
       <c r="B692" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">is_principal</t>
+          <t xml:space="preserve">is_whatsapp</t>
         </is>
       </c>
       <c r="C692" t="inlineStr" s="2">
@@ -19612,25 +19612,29 @@
     <row r="693">
       <c r="A693" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">instalacoes_galeria</t>
+          <t xml:space="preserve">contatos_adicionais</t>
         </is>
       </c>
       <c r="B693" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">is_principal</t>
         </is>
       </c>
       <c r="C693" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D693" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E693" s="2"/>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F693" s="2"/>
       <c r="G693" s="2"/>
     </row>
@@ -19642,7 +19646,7 @@
       </c>
       <c r="B694" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cidade</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C694" t="inlineStr" s="2">
@@ -19652,7 +19656,7 @@
       </c>
       <c r="D694" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E694" s="2"/>
@@ -19667,12 +19671,12 @@
       </c>
       <c r="B695" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">potencia_kwp</t>
+          <t xml:space="preserve">cidade</t>
         </is>
       </c>
       <c r="C695" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D695" t="inlineStr" s="2">
@@ -19692,12 +19696,12 @@
       </c>
       <c r="B696" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">foto</t>
+          <t xml:space="preserve">potencia_kwp</t>
         </is>
       </c>
       <c r="C696" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">file</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D696" t="inlineStr" s="2">
@@ -19707,11 +19711,7 @@
       </c>
       <c r="E696" s="2"/>
       <c r="F696" s="2"/>
-      <c r="G696" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
-        </is>
-      </c>
+      <c r="G696" s="2"/>
     </row>
     <row r="697">
       <c r="A697" t="inlineStr" s="2">
@@ -19721,12 +19721,12 @@
       </c>
       <c r="B697" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">foto_url</t>
+          <t xml:space="preserve">foto</t>
         </is>
       </c>
       <c r="C697" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="D697" t="inlineStr" s="2">
@@ -19736,7 +19736,11 @@
       </c>
       <c r="E697" s="2"/>
       <c r="F697" s="2"/>
-      <c r="G697" s="2"/>
+      <c r="G697" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
+        </is>
+      </c>
     </row>
     <row r="698">
       <c r="A698" t="inlineStr" s="2">
@@ -19746,12 +19750,12 @@
       </c>
       <c r="B698" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ordem</t>
+          <t xml:space="preserve">foto_url</t>
         </is>
       </c>
       <c r="C698" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D698" t="inlineStr" s="2">
@@ -19771,12 +19775,12 @@
       </c>
       <c r="B699" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">destaque</t>
+          <t xml:space="preserve">ordem</t>
         </is>
       </c>
       <c r="C699" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D699" t="inlineStr" s="2">
@@ -19784,11 +19788,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E699" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E699" s="2"/>
       <c r="F699" s="2"/>
       <c r="G699" s="2"/>
     </row>
@@ -19800,12 +19800,12 @@
       </c>
       <c r="B700" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">destaque</t>
         </is>
       </c>
       <c r="C700" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D700" t="inlineStr" s="2">
@@ -19813,13 +19813,13 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E700" s="2"/>
+      <c r="E700" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F700" s="2"/>
-      <c r="G700" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G700" s="2"/>
     </row>
     <row r="701">
       <c r="A701" t="inlineStr" s="2">
@@ -19829,7 +19829,7 @@
       </c>
       <c r="B701" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C701" t="inlineStr" s="2">
@@ -19846,34 +19846,38 @@
       <c r="F701" s="2"/>
       <c r="G701" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="702">
       <c r="A702" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">projecao_tarifaria</t>
+          <t xml:space="preserve">instalacoes_galeria</t>
         </is>
       </c>
       <c r="B702" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ano</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C702" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D702" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E702" s="2"/>
       <c r="F702" s="2"/>
-      <c r="G702" s="2"/>
+      <c r="G702" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="703">
       <c r="A703" t="inlineStr" s="2">
@@ -19883,12 +19887,12 @@
       </c>
       <c r="B703" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_cliente</t>
+          <t xml:space="preserve">ano</t>
         </is>
       </c>
       <c r="C703" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D703" t="inlineStr" s="2">
@@ -19896,11 +19900,7 @@
           <t xml:space="preserve">Sim</t>
         </is>
       </c>
-      <c r="E703" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">residencial | comercial</t>
-        </is>
-      </c>
+      <c r="E703" s="2"/>
       <c r="F703" s="2"/>
       <c r="G703" s="2"/>
     </row>
@@ -19912,20 +19912,24 @@
       </c>
       <c r="B704" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tarifa_kwh</t>
+          <t xml:space="preserve">tipo_cliente</t>
         </is>
       </c>
       <c r="C704" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D704" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E704" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">residencial | comercial</t>
+        </is>
+      </c>
       <c r="F704" s="2"/>
       <c r="G704" s="2"/>
     </row>
@@ -19937,7 +19941,7 @@
       </c>
       <c r="B705" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fio_b_kwh</t>
+          <t xml:space="preserve">tarifa_kwh</t>
         </is>
       </c>
       <c r="C705" t="inlineStr" s="2">
@@ -19962,7 +19966,7 @@
       </c>
       <c r="B706" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fs</t>
+          <t xml:space="preserve">fio_b_kwh</t>
         </is>
       </c>
       <c r="C706" t="inlineStr" s="2">
@@ -19987,7 +19991,7 @@
       </c>
       <c r="B707" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gd_eco_liquida</t>
+          <t xml:space="preserve">fs</t>
         </is>
       </c>
       <c r="C707" t="inlineStr" s="2">
@@ -20012,7 +20016,7 @@
       </c>
       <c r="B708" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">economia_acumulada</t>
+          <t xml:space="preserve">gd_eco_liquida</t>
         </is>
       </c>
       <c r="C708" t="inlineStr" s="2">
@@ -20037,7 +20041,7 @@
       </c>
       <c r="B709" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gasto_acumulado</t>
+          <t xml:space="preserve">economia_acumulada</t>
         </is>
       </c>
       <c r="C709" t="inlineStr" s="2">
@@ -20062,12 +20066,12 @@
       </c>
       <c r="B710" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">gasto_acumulado</t>
         </is>
       </c>
       <c r="C710" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D710" t="inlineStr" s="2">
@@ -20077,11 +20081,7 @@
       </c>
       <c r="E710" s="2"/>
       <c r="F710" s="2"/>
-      <c r="G710" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G710" s="2"/>
     </row>
     <row r="711">
       <c r="A711" t="inlineStr" s="2">
@@ -20091,7 +20091,7 @@
       </c>
       <c r="B711" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C711" t="inlineStr" s="2">
@@ -20108,38 +20108,38 @@
       <c r="F711" s="2"/>
       <c r="G711" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="712">
       <c r="A712" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">equipamentos</t>
+          <t xml:space="preserve">projecao_tarifaria</t>
         </is>
       </c>
       <c r="B712" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C712" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D712" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E712" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">inversor | modulo_fv | outro</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E712" s="2"/>
       <c r="F712" s="2"/>
-      <c r="G712" s="2"/>
+      <c r="G712" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="713">
       <c r="A713" t="inlineStr" s="2">
@@ -20149,12 +20149,12 @@
       </c>
       <c r="B713" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">marca</t>
+          <t xml:space="preserve">tipo</t>
         </is>
       </c>
       <c r="C713" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D713" t="inlineStr" s="2">
@@ -20162,7 +20162,11 @@
           <t xml:space="preserve">Sim</t>
         </is>
       </c>
-      <c r="E713" s="2"/>
+      <c r="E713" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">inversor | modulo_fv | outro</t>
+        </is>
+      </c>
       <c r="F713" s="2"/>
       <c r="G713" s="2"/>
     </row>
@@ -20174,7 +20178,7 @@
       </c>
       <c r="B714" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">modelo</t>
+          <t xml:space="preserve">marca</t>
         </is>
       </c>
       <c r="C714" t="inlineStr" s="2">
@@ -20199,12 +20203,12 @@
       </c>
       <c r="B715" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">potencia_w</t>
+          <t xml:space="preserve">modelo</t>
         </is>
       </c>
       <c r="C715" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D715" t="inlineStr" s="2">
@@ -20224,17 +20228,17 @@
       </c>
       <c r="B716" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">descricao_padrao</t>
+          <t xml:space="preserve">potencia_w</t>
         </is>
       </c>
       <c r="C716" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D716" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E716" s="2"/>
@@ -20249,12 +20253,12 @@
       </c>
       <c r="B717" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">garantia_anos</t>
+          <t xml:space="preserve">descricao_padrao</t>
         </is>
       </c>
       <c r="C717" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D717" t="inlineStr" s="2">
@@ -20274,12 +20278,12 @@
       </c>
       <c r="B718" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">foto</t>
+          <t xml:space="preserve">garantia_anos</t>
         </is>
       </c>
       <c r="C718" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">file</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D718" t="inlineStr" s="2">
@@ -20289,11 +20293,7 @@
       </c>
       <c r="E718" s="2"/>
       <c r="F718" s="2"/>
-      <c r="G718" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
-        </is>
-      </c>
+      <c r="G718" s="2"/>
     </row>
     <row r="719">
       <c r="A719" t="inlineStr" s="2">
@@ -20303,12 +20303,12 @@
       </c>
       <c r="B719" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">foto</t>
         </is>
       </c>
       <c r="C719" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="D719" t="inlineStr" s="2">
@@ -20320,7 +20320,7 @@
       <c r="F719" s="2"/>
       <c r="G719" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
+          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
         </is>
       </c>
     </row>
@@ -20332,7 +20332,7 @@
       </c>
       <c r="B720" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C720" t="inlineStr" s="2">
@@ -20349,7 +20349,7 @@
       <c r="F720" s="2"/>
       <c r="G720" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
@@ -20361,12 +20361,12 @@
       </c>
       <c r="B721" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">datasheet_pdf</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C721" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">file</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D721" t="inlineStr" s="2">
@@ -20378,7 +20378,7 @@
       <c r="F721" s="2"/>
       <c r="G721" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
         </is>
       </c>
     </row>
@@ -20390,12 +20390,12 @@
       </c>
       <c r="B722" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">datasheet_url</t>
+          <t xml:space="preserve">datasheet_pdf</t>
         </is>
       </c>
       <c r="C722" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">url</t>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="D722" t="inlineStr" s="2">
@@ -20405,7 +20405,11 @@
       </c>
       <c r="E722" s="2"/>
       <c r="F722" s="2"/>
-      <c r="G722" s="2"/>
+      <c r="G722" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
+        </is>
+      </c>
     </row>
     <row r="723">
       <c r="A723" t="inlineStr" s="2">
@@ -20415,7 +20419,7 @@
       </c>
       <c r="B723" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">datalogger_url</t>
+          <t xml:space="preserve">datasheet_url</t>
         </is>
       </c>
       <c r="C723" t="inlineStr" s="2">
@@ -20440,12 +20444,12 @@
       </c>
       <c r="B724" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fornecedor_id</t>
+          <t xml:space="preserve">datalogger_url</t>
         </is>
       </c>
       <c r="C724" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">url</t>
         </is>
       </c>
       <c r="D724" t="inlineStr" s="2">
@@ -20454,11 +20458,7 @@
         </is>
       </c>
       <c r="E724" s="2"/>
-      <c r="F724" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">fornecedores</t>
-        </is>
-      </c>
+      <c r="F724" s="2"/>
       <c r="G724" s="2"/>
     </row>
     <row r="725">
@@ -20469,12 +20469,12 @@
       </c>
       <c r="B725" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">telefone_suporte_fornecedor</t>
+          <t xml:space="preserve">fornecedor_id</t>
         </is>
       </c>
       <c r="C725" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D725" t="inlineStr" s="2">
@@ -20483,28 +20483,32 @@
         </is>
       </c>
       <c r="E725" s="2"/>
-      <c r="F725" s="2"/>
+      <c r="F725" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">fornecedores</t>
+        </is>
+      </c>
       <c r="G725" s="2"/>
     </row>
     <row r="726">
       <c r="A726" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">parametros_tarifarios</t>
+          <t xml:space="preserve">equipamentos</t>
         </is>
       </c>
       <c r="B726" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ano</t>
+          <t xml:space="preserve">telefone_suporte_fornecedor</t>
         </is>
       </c>
       <c r="C726" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D726" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E726" s="2"/>
@@ -20519,12 +20523,12 @@
       </c>
       <c r="B727" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">classe</t>
+          <t xml:space="preserve">ano</t>
         </is>
       </c>
       <c r="C727" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D727" t="inlineStr" s="2">
@@ -20532,11 +20536,7 @@
           <t xml:space="preserve">Sim</t>
         </is>
       </c>
-      <c r="E727" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">residencial | comercial</t>
-        </is>
-      </c>
+      <c r="E727" s="2"/>
       <c r="F727" s="2"/>
       <c r="G727" s="2"/>
     </row>
@@ -20548,20 +20548,24 @@
       </c>
       <c r="B728" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tarifa</t>
+          <t xml:space="preserve">classe</t>
         </is>
       </c>
       <c r="C728" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D728" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E728" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E728" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">residencial | comercial</t>
+        </is>
+      </c>
       <c r="F728" s="2"/>
       <c r="G728" s="2"/>
     </row>
@@ -20573,7 +20577,7 @@
       </c>
       <c r="B729" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fio_b</t>
+          <t xml:space="preserve">tarifa</t>
         </is>
       </c>
       <c r="C729" t="inlineStr" s="2">
@@ -20598,7 +20602,7 @@
       </c>
       <c r="B730" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fs</t>
+          <t xml:space="preserve">fio_b</t>
         </is>
       </c>
       <c r="C730" t="inlineStr" s="2">
@@ -20623,7 +20627,7 @@
       </c>
       <c r="B731" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gd_eco_liquida</t>
+          <t xml:space="preserve">fs</t>
         </is>
       </c>
       <c r="C731" t="inlineStr" s="2">
@@ -20648,12 +20652,12 @@
       </c>
       <c r="B732" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">gd_eco_liquida</t>
         </is>
       </c>
       <c r="C732" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D732" t="inlineStr" s="2">
@@ -20663,11 +20667,7 @@
       </c>
       <c r="E732" s="2"/>
       <c r="F732" s="2"/>
-      <c r="G732" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G732" s="2"/>
     </row>
     <row r="733">
       <c r="A733" t="inlineStr" s="2">
@@ -20677,7 +20677,7 @@
       </c>
       <c r="B733" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C733" t="inlineStr" s="2">
@@ -20694,34 +20694,38 @@
       <c r="F733" s="2"/>
       <c r="G733" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="734">
       <c r="A734" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes</t>
+          <t xml:space="preserve">parametros_tarifarios</t>
         </is>
       </c>
       <c r="B734" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">nome</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C734" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D734" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E734" s="2"/>
       <c r="F734" s="2"/>
-      <c r="G734" s="2"/>
+      <c r="G734" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="735">
       <c r="A735" t="inlineStr" s="2">
@@ -20731,12 +20735,12 @@
       </c>
       <c r="B735" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">gatilho</t>
+          <t xml:space="preserve">nome</t>
         </is>
       </c>
       <c r="C735" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D735" t="inlineStr" s="2">
@@ -20744,11 +20748,7 @@
           <t xml:space="preserve">Sim</t>
         </is>
       </c>
-      <c r="E735" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">status_mudou | instalacao_concluida | atividade_concluida | data_especifica | dias_apos_evento</t>
-        </is>
-      </c>
+      <c r="E735" s="2"/>
       <c r="F735" s="2"/>
       <c r="G735" s="2"/>
     </row>
@@ -20760,26 +20760,26 @@
       </c>
       <c r="B736" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">configuracao_gatilho</t>
+          <t xml:space="preserve">gatilho</t>
         </is>
       </c>
       <c r="C736" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D736" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E736" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E736" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">status_mudou | instalacao_concluida | atividade_concluida | data_especifica | dias_apos_evento</t>
+        </is>
+      </c>
       <c r="F736" s="2"/>
-      <c r="G736" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="G736" s="2"/>
     </row>
     <row r="737">
       <c r="A737" t="inlineStr" s="2">
@@ -20789,26 +20789,26 @@
       </c>
       <c r="B737" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">acao</t>
+          <t xml:space="preserve">configuracao_gatilho</t>
         </is>
       </c>
       <c r="C737" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D737" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E737" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">criar_atividade | enviar_whatsapp | enviar_email | mudar_status</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E737" s="2"/>
       <c r="F737" s="2"/>
-      <c r="G737" s="2"/>
+      <c r="G737" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Estrutura JSON livre</t>
+        </is>
+      </c>
     </row>
     <row r="738">
       <c r="A738" t="inlineStr" s="2">
@@ -20818,26 +20818,26 @@
       </c>
       <c r="B738" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">configuracao_acao</t>
+          <t xml:space="preserve">acao</t>
         </is>
       </c>
       <c r="C738" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D738" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E738" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E738" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">criar_atividade | enviar_whatsapp | enviar_email | mudar_status</t>
+        </is>
+      </c>
       <c r="F738" s="2"/>
-      <c r="G738" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="G738" s="2"/>
     </row>
     <row r="739">
       <c r="A739" t="inlineStr" s="2">
@@ -20847,26 +20847,26 @@
       </c>
       <c r="B739" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">destino</t>
+          <t xml:space="preserve">configuracao_acao</t>
         </is>
       </c>
       <c r="C739" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D739" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E739" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">cliente_evento | responsavel_empresa | cliente_especifico</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E739" s="2"/>
       <c r="F739" s="2"/>
-      <c r="G739" s="2"/>
+      <c r="G739" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Estrutura JSON livre</t>
+        </is>
+      </c>
     </row>
     <row r="740">
       <c r="A740" t="inlineStr" s="2">
@@ -20876,25 +20876,25 @@
       </c>
       <c r="B740" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_especifico_id</t>
+          <t xml:space="preserve">destino</t>
         </is>
       </c>
       <c r="C740" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D740" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E740" s="2"/>
-      <c r="F740" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E740" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">cliente_evento | responsavel_empresa | cliente_especifico</t>
+        </is>
+      </c>
+      <c r="F740" s="2"/>
       <c r="G740" s="2"/>
     </row>
     <row r="741">
@@ -20905,12 +20905,12 @@
       </c>
       <c r="B741" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ativa</t>
+          <t xml:space="preserve">cliente_especifico_id</t>
         </is>
       </c>
       <c r="C741" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D741" t="inlineStr" s="2">
@@ -20918,12 +20918,12 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E741" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
-      <c r="F741" s="2"/>
+      <c r="E741" s="2"/>
+      <c r="F741" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G741" s="2"/>
     </row>
     <row r="742">
@@ -20934,12 +20934,12 @@
       </c>
       <c r="B742" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">ativa</t>
         </is>
       </c>
       <c r="C742" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D742" t="inlineStr" s="2">
@@ -20947,13 +20947,13 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E742" s="2"/>
+      <c r="E742" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F742" s="2"/>
-      <c r="G742" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G742" s="2"/>
     </row>
     <row r="743">
       <c r="A743" t="inlineStr" s="2">
@@ -20963,7 +20963,7 @@
       </c>
       <c r="B743" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C743" t="inlineStr" s="2">
@@ -20980,38 +20980,38 @@
       <c r="F743" s="2"/>
       <c r="G743" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="744">
       <c r="A744" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacoes_execucoes</t>
+          <t xml:space="preserve">automacoes</t>
         </is>
       </c>
       <c r="B744" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">automacao</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C744" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D744" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E744" s="2"/>
-      <c r="F744" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">automacoes</t>
-        </is>
-      </c>
-      <c r="G744" s="2"/>
+      <c r="F744" s="2"/>
+      <c r="G744" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="745">
       <c r="A745" t="inlineStr" s="2">
@@ -21021,12 +21021,12 @@
       </c>
       <c r="B745" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_execucao</t>
+          <t xml:space="preserve">automacao</t>
         </is>
       </c>
       <c r="C745" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D745" t="inlineStr" s="2">
@@ -21035,7 +21035,11 @@
         </is>
       </c>
       <c r="E745" s="2"/>
-      <c r="F745" s="2"/>
+      <c r="F745" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">automacoes</t>
+        </is>
+      </c>
       <c r="G745" s="2"/>
     </row>
     <row r="746">
@@ -21046,24 +21050,20 @@
       </c>
       <c r="B746" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">sucesso</t>
+          <t xml:space="preserve">data_execucao</t>
         </is>
       </c>
       <c r="C746" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D746" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E746" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E746" s="2"/>
       <c r="F746" s="2"/>
       <c r="G746" s="2"/>
     </row>
@@ -21075,12 +21075,12 @@
       </c>
       <c r="B747" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mensagem</t>
+          <t xml:space="preserve">sucesso</t>
         </is>
       </c>
       <c r="C747" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D747" t="inlineStr" s="2">
@@ -21088,7 +21088,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E747" s="2"/>
+      <c r="E747" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F747" s="2"/>
       <c r="G747" s="2"/>
     </row>
@@ -21100,7 +21104,7 @@
       </c>
       <c r="B748" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">referencia_registro</t>
+          <t xml:space="preserve">mensagem</t>
         </is>
       </c>
       <c r="C748" t="inlineStr" s="2">
@@ -21125,12 +21129,12 @@
       </c>
       <c r="B749" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente</t>
+          <t xml:space="preserve">referencia_registro</t>
         </is>
       </c>
       <c r="C749" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D749" t="inlineStr" s="2">
@@ -21139,11 +21143,7 @@
         </is>
       </c>
       <c r="E749" s="2"/>
-      <c r="F749" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+      <c r="F749" s="2"/>
       <c r="G749" s="2"/>
     </row>
     <row r="750">
@@ -21154,12 +21154,12 @@
       </c>
       <c r="B750" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">dados_execucao</t>
+          <t xml:space="preserve">cliente</t>
         </is>
       </c>
       <c r="C750" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D750" t="inlineStr" s="2">
@@ -21168,12 +21168,12 @@
         </is>
       </c>
       <c r="E750" s="2"/>
-      <c r="F750" s="2"/>
-      <c r="G750" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="F750" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
+      <c r="G750" s="2"/>
     </row>
     <row r="751">
       <c r="A751" t="inlineStr" s="2">
@@ -21183,12 +21183,12 @@
       </c>
       <c r="B751" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">dados_execucao</t>
         </is>
       </c>
       <c r="C751" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D751" t="inlineStr" s="2">
@@ -21200,7 +21200,7 @@
       <c r="F751" s="2"/>
       <c r="G751" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
+          <t xml:space="preserve">Estrutura JSON livre</t>
         </is>
       </c>
     </row>
@@ -21212,7 +21212,7 @@
       </c>
       <c r="B752" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C752" t="inlineStr" s="2">
@@ -21229,38 +21229,38 @@
       <c r="F752" s="2"/>
       <c r="G752" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="753">
       <c r="A753" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">notificacoes_internas</t>
+          <t xml:space="preserve">automacoes_execucoes</t>
         </is>
       </c>
       <c r="B753" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C753" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D753" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E753" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">atividade_atrasada | lembrete | sistema</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E753" s="2"/>
       <c r="F753" s="2"/>
-      <c r="G753" s="2"/>
+      <c r="G753" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="754">
       <c r="A754" t="inlineStr" s="2">
@@ -21270,12 +21270,12 @@
       </c>
       <c r="B754" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">tipo</t>
         </is>
       </c>
       <c r="C754" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D754" t="inlineStr" s="2">
@@ -21283,7 +21283,11 @@
           <t xml:space="preserve">Sim</t>
         </is>
       </c>
-      <c r="E754" s="2"/>
+      <c r="E754" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">atividade_atrasada | lembrete | sistema</t>
+        </is>
+      </c>
       <c r="F754" s="2"/>
       <c r="G754" s="2"/>
     </row>
@@ -21295,7 +21299,7 @@
       </c>
       <c r="B755" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mensagem</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C755" t="inlineStr" s="2">
@@ -21305,7 +21309,7 @@
       </c>
       <c r="D755" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E755" s="2"/>
@@ -21320,12 +21324,12 @@
       </c>
       <c r="B756" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">atividade_id</t>
+          <t xml:space="preserve">mensagem</t>
         </is>
       </c>
       <c r="C756" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D756" t="inlineStr" s="2">
@@ -21334,11 +21338,7 @@
         </is>
       </c>
       <c r="E756" s="2"/>
-      <c r="F756" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">atividades</t>
-        </is>
-      </c>
+      <c r="F756" s="2"/>
       <c r="G756" s="2"/>
     </row>
     <row r="757">
@@ -21349,7 +21349,7 @@
       </c>
       <c r="B757" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_id</t>
+          <t xml:space="preserve">atividade_id</t>
         </is>
       </c>
       <c r="C757" t="inlineStr" s="2">
@@ -21365,7 +21365,7 @@
       <c r="E757" s="2"/>
       <c r="F757" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">clientes</t>
+          <t xml:space="preserve">atividades</t>
         </is>
       </c>
       <c r="G757" s="2"/>
@@ -21378,12 +21378,12 @@
       </c>
       <c r="B758" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_nome</t>
+          <t xml:space="preserve">cliente_id</t>
         </is>
       </c>
       <c r="C758" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D758" t="inlineStr" s="2">
@@ -21392,7 +21392,11 @@
         </is>
       </c>
       <c r="E758" s="2"/>
-      <c r="F758" s="2"/>
+      <c r="F758" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G758" s="2"/>
     </row>
     <row r="759">
@@ -21403,12 +21407,12 @@
       </c>
       <c r="B759" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_prevista</t>
+          <t xml:space="preserve">cliente_nome</t>
         </is>
       </c>
       <c r="C759" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D759" t="inlineStr" s="2">
@@ -21428,12 +21432,12 @@
       </c>
       <c r="B760" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">dias_atraso</t>
+          <t xml:space="preserve">data_prevista</t>
         </is>
       </c>
       <c r="C760" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D760" t="inlineStr" s="2">
@@ -21453,12 +21457,12 @@
       </c>
       <c r="B761" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">lida</t>
+          <t xml:space="preserve">dias_atraso</t>
         </is>
       </c>
       <c r="C761" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D761" t="inlineStr" s="2">
@@ -21466,11 +21470,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E761" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E761" s="2"/>
       <c r="F761" s="2"/>
       <c r="G761" s="2"/>
     </row>
@@ -21482,12 +21482,12 @@
       </c>
       <c r="B762" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">lida_em</t>
+          <t xml:space="preserve">lida</t>
         </is>
       </c>
       <c r="C762" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D762" t="inlineStr" s="2">
@@ -21495,7 +21495,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E762" s="2"/>
+      <c r="E762" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F762" s="2"/>
       <c r="G762" s="2"/>
     </row>
@@ -21507,24 +21511,20 @@
       </c>
       <c r="B763" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">lida_em</t>
         </is>
       </c>
       <c r="C763" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D763" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E763" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">ativa | resolvida | arquivada</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E763" s="2"/>
       <c r="F763" s="2"/>
       <c r="G763" s="2"/>
     </row>
@@ -21536,20 +21536,24 @@
       </c>
       <c r="B764" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">resolvida_em</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="C764" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D764" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E764" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E764" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ativa | resolvida | arquivada</t>
+        </is>
+      </c>
       <c r="F764" s="2"/>
       <c r="G764" s="2"/>
     </row>
@@ -21561,12 +21565,12 @@
       </c>
       <c r="B765" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">resolvida_em</t>
         </is>
       </c>
       <c r="C765" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D765" t="inlineStr" s="2">
@@ -21576,11 +21580,7 @@
       </c>
       <c r="E765" s="2"/>
       <c r="F765" s="2"/>
-      <c r="G765" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G765" s="2"/>
     </row>
     <row r="766">
       <c r="A766" t="inlineStr" s="2">
@@ -21590,7 +21590,7 @@
       </c>
       <c r="B766" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C766" t="inlineStr" s="2">
@@ -21607,38 +21607,38 @@
       <c r="F766" s="2"/>
       <c r="G766" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="767">
       <c r="A767" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">notificacoes_internas</t>
         </is>
       </c>
       <c r="B767" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_id</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C767" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D767" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E767" s="2"/>
-      <c r="F767" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
-      <c r="G767" s="2"/>
+      <c r="F767" s="2"/>
+      <c r="G767" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="768">
       <c r="A768" t="inlineStr" s="2">
@@ -21648,25 +21648,25 @@
       </c>
       <c r="B768" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_negocio</t>
+          <t xml:space="preserve">cliente_id</t>
         </is>
       </c>
       <c r="C768" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D768" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E768" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">venda usina | bateria | expansão | renovação | serviço | venda bateria</t>
-        </is>
-      </c>
-      <c r="F768" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E768" s="2"/>
+      <c r="F768" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G768" s="2"/>
     </row>
     <row r="769">
@@ -21677,12 +21677,12 @@
       </c>
       <c r="B769" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">valor_estimado</t>
+          <t xml:space="preserve">tipo_negocio</t>
         </is>
       </c>
       <c r="C769" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D769" t="inlineStr" s="2">
@@ -21690,7 +21690,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E769" s="2"/>
+      <c r="E769" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">venda usina | bateria | expansão | renovação | serviço | venda bateria</t>
+        </is>
+      </c>
       <c r="F769" s="2"/>
       <c r="G769" s="2"/>
     </row>
@@ -21702,7 +21706,7 @@
       </c>
       <c r="B770" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">valor_final</t>
+          <t xml:space="preserve">valor_estimado</t>
         </is>
       </c>
       <c r="C770" t="inlineStr" s="2">
@@ -21727,12 +21731,12 @@
       </c>
       <c r="B771" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">etapa_funil</t>
+          <t xml:space="preserve">valor_final</t>
         </is>
       </c>
       <c r="C771" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D771" t="inlineStr" s="2">
@@ -21740,11 +21744,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E771" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">novo lead | qualificado | proposta enviada | negociação | contrato assinado</t>
-        </is>
-      </c>
+      <c r="E771" s="2"/>
       <c r="F771" s="2"/>
       <c r="G771" s="2"/>
     </row>
@@ -21756,12 +21756,12 @@
       </c>
       <c r="B772" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">probabilidade</t>
+          <t xml:space="preserve">etapa_funil</t>
         </is>
       </c>
       <c r="C772" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D772" t="inlineStr" s="2">
@@ -21769,7 +21769,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E772" s="2"/>
+      <c r="E772" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">novo lead | qualificado | proposta enviada | negociação | contrato assinado</t>
+        </is>
+      </c>
       <c r="F772" s="2"/>
       <c r="G772" s="2"/>
     </row>
@@ -21781,12 +21785,12 @@
       </c>
       <c r="B773" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_previsao_fechamento</t>
+          <t xml:space="preserve">probabilidade</t>
         </is>
       </c>
       <c r="C773" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D773" t="inlineStr" s="2">
@@ -21806,7 +21810,7 @@
       </c>
       <c r="B774" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_fechamento</t>
+          <t xml:space="preserve">data_previsao_fechamento</t>
         </is>
       </c>
       <c r="C774" t="inlineStr" s="2">
@@ -21831,12 +21835,12 @@
       </c>
       <c r="B775" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">data_fechamento</t>
         </is>
       </c>
       <c r="C775" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D775" t="inlineStr" s="2">
@@ -21844,11 +21848,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E775" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">em andamento | ganho | perdido</t>
-        </is>
-      </c>
+      <c r="E775" s="2"/>
       <c r="F775" s="2"/>
       <c r="G775" s="2"/>
     </row>
@@ -21860,12 +21860,12 @@
       </c>
       <c r="B776" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">motivo_perda</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="C776" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D776" t="inlineStr" s="2">
@@ -21873,7 +21873,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E776" s="2"/>
+      <c r="E776" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">em andamento | ganho | perdido</t>
+        </is>
+      </c>
       <c r="F776" s="2"/>
       <c r="G776" s="2"/>
     </row>
@@ -21885,12 +21889,12 @@
       </c>
       <c r="B777" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">reabertura</t>
+          <t xml:space="preserve">motivo_perda</t>
         </is>
       </c>
       <c r="C777" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D777" t="inlineStr" s="2">
@@ -21898,11 +21902,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E777" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E777" s="2"/>
       <c r="F777" s="2"/>
       <c r="G777" s="2"/>
     </row>
@@ -21914,12 +21914,12 @@
       </c>
       <c r="B778" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">motivo_reabertura</t>
+          <t xml:space="preserve">reabertura</t>
         </is>
       </c>
       <c r="C778" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D778" t="inlineStr" s="2">
@@ -21927,7 +21927,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E778" s="2"/>
+      <c r="E778" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F778" s="2"/>
       <c r="G778" s="2"/>
     </row>
@@ -21939,7 +21943,7 @@
       </c>
       <c r="B779" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">condicao_pagamento</t>
+          <t xml:space="preserve">motivo_reabertura</t>
         </is>
       </c>
       <c r="C779" t="inlineStr" s="2">
@@ -21964,12 +21968,12 @@
       </c>
       <c r="B780" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">condicao_pagamento</t>
         </is>
       </c>
       <c r="C780" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D780" t="inlineStr" s="2">
@@ -21979,11 +21983,7 @@
       </c>
       <c r="E780" s="2"/>
       <c r="F780" s="2"/>
-      <c r="G780" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G780" s="2"/>
     </row>
     <row r="781">
       <c r="A781" t="inlineStr" s="2">
@@ -21993,7 +21993,7 @@
       </c>
       <c r="B781" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C781" t="inlineStr" s="2">
@@ -22010,7 +22010,7 @@
       <c r="F781" s="2"/>
       <c r="G781" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
@@ -22022,12 +22022,12 @@
       </c>
       <c r="B782" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_venda</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C782" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D782" t="inlineStr" s="2">
@@ -22035,13 +22035,13 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E782" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Energia Solar | O&amp;M (Operação e Manutenção) | Baterias | Carregadores Veículos Elétricos</t>
-        </is>
-      </c>
+      <c r="E782" s="2"/>
       <c r="F782" s="2"/>
-      <c r="G782" s="2"/>
+      <c r="G782" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="783">
       <c r="A783" t="inlineStr" s="2">
@@ -22051,12 +22051,12 @@
       </c>
       <c r="B783" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">tipo_venda</t>
         </is>
       </c>
       <c r="C783" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D783" t="inlineStr" s="2">
@@ -22064,7 +22064,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E783" s="2"/>
+      <c r="E783" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Energia Solar | O&amp;M (Operação e Manutenção) | Baterias | Carregadores Veículos Elétricos</t>
+        </is>
+      </c>
       <c r="F783" s="2"/>
       <c r="G783" s="2"/>
     </row>
@@ -22076,12 +22080,12 @@
       </c>
       <c r="B784" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">valor</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C784" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D784" t="inlineStr" s="2">
@@ -22101,12 +22105,12 @@
       </c>
       <c r="B785" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">consultor_responsavel</t>
+          <t xml:space="preserve">valor</t>
         </is>
       </c>
       <c r="C785" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D785" t="inlineStr" s="2">
@@ -22115,11 +22119,7 @@
         </is>
       </c>
       <c r="E785" s="2"/>
-      <c r="F785" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">users</t>
-        </is>
-      </c>
+      <c r="F785" s="2"/>
       <c r="G785" s="2"/>
     </row>
     <row r="786">
@@ -22130,12 +22130,12 @@
       </c>
       <c r="B786" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">recorrencia_mensal</t>
+          <t xml:space="preserve">consultor_responsavel</t>
         </is>
       </c>
       <c r="C786" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D786" t="inlineStr" s="2">
@@ -22143,36 +22143,40 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E786" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
-      <c r="F786" s="2"/>
+      <c r="E786" s="2"/>
+      <c r="F786" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">users</t>
+        </is>
+      </c>
       <c r="G786" s="2"/>
     </row>
     <row r="787">
       <c r="A787" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">analises_fatura</t>
+          <t xml:space="preserve">negocios</t>
         </is>
       </c>
       <c r="B787" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">token</t>
+          <t xml:space="preserve">recorrencia_mensal</t>
         </is>
       </c>
       <c r="C787" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D787" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E787" s="2"/>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E787" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F787" s="2"/>
       <c r="G787" s="2"/>
     </row>
@@ -22184,25 +22188,21 @@
       </c>
       <c r="B788" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_id</t>
+          <t xml:space="preserve">token</t>
         </is>
       </c>
       <c r="C788" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D788" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E788" s="2"/>
-      <c r="F788" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+      <c r="F788" s="2"/>
       <c r="G788" s="2"/>
     </row>
     <row r="789">
@@ -22213,12 +22213,12 @@
       </c>
       <c r="B789" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_nome</t>
+          <t xml:space="preserve">cliente_id</t>
         </is>
       </c>
       <c r="C789" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D789" t="inlineStr" s="2">
@@ -22227,7 +22227,11 @@
         </is>
       </c>
       <c r="E789" s="2"/>
-      <c r="F789" s="2"/>
+      <c r="F789" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">clientes</t>
+        </is>
+      </c>
       <c r="G789" s="2"/>
     </row>
     <row r="790">
@@ -22238,7 +22242,7 @@
       </c>
       <c r="B790" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">uc</t>
+          <t xml:space="preserve">cliente_nome</t>
         </is>
       </c>
       <c r="C790" t="inlineStr" s="2">
@@ -22263,7 +22267,7 @@
       </c>
       <c r="B791" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">competencia</t>
+          <t xml:space="preserve">uc</t>
         </is>
       </c>
       <c r="C791" t="inlineStr" s="2">
@@ -22288,7 +22292,7 @@
       </c>
       <c r="B792" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">vencimento</t>
+          <t xml:space="preserve">competencia</t>
         </is>
       </c>
       <c r="C792" t="inlineStr" s="2">
@@ -22313,12 +22317,12 @@
       </c>
       <c r="B793" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">total_pagar</t>
+          <t xml:space="preserve">vencimento</t>
         </is>
       </c>
       <c r="C793" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D793" t="inlineStr" s="2">
@@ -22338,7 +22342,7 @@
       </c>
       <c r="B794" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">consumo_kwh</t>
+          <t xml:space="preserve">total_pagar</t>
         </is>
       </c>
       <c r="C794" t="inlineStr" s="2">
@@ -22363,7 +22367,7 @@
       </c>
       <c r="B795" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">energia_injetada_kwh</t>
+          <t xml:space="preserve">consumo_kwh</t>
         </is>
       </c>
       <c r="C795" t="inlineStr" s="2">
@@ -22388,7 +22392,7 @@
       </c>
       <c r="B796" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">creditos_compensados_kwh</t>
+          <t xml:space="preserve">energia_injetada_kwh</t>
         </is>
       </c>
       <c r="C796" t="inlineStr" s="2">
@@ -22413,7 +22417,7 @@
       </c>
       <c r="B797" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">saldo_energia_kwh</t>
+          <t xml:space="preserve">creditos_compensados_kwh</t>
         </is>
       </c>
       <c r="C797" t="inlineStr" s="2">
@@ -22438,7 +22442,7 @@
       </c>
       <c r="B798" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">saldo_expirar_kwh</t>
+          <t xml:space="preserve">saldo_energia_kwh</t>
         </is>
       </c>
       <c r="C798" t="inlineStr" s="2">
@@ -22463,7 +22467,7 @@
       </c>
       <c r="B799" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">economia_estimada_rs</t>
+          <t xml:space="preserve">saldo_expirar_kwh</t>
         </is>
       </c>
       <c r="C799" t="inlineStr" s="2">
@@ -22488,12 +22492,12 @@
       </c>
       <c r="B800" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">papel_uc</t>
+          <t xml:space="preserve">economia_estimada_rs</t>
         </is>
       </c>
       <c r="C800" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D800" t="inlineStr" s="2">
@@ -22513,12 +22517,12 @@
       </c>
       <c r="B801" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">arquivos_nomes</t>
+          <t xml:space="preserve">papel_uc</t>
         </is>
       </c>
       <c r="C801" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">json</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D801" t="inlineStr" s="2">
@@ -22528,11 +22532,7 @@
       </c>
       <c r="E801" s="2"/>
       <c r="F801" s="2"/>
-      <c r="G801" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Estrutura JSON livre</t>
-        </is>
-      </c>
+      <c r="G801" s="2"/>
     </row>
     <row r="802">
       <c r="A802" t="inlineStr" s="2">
@@ -22542,7 +22542,7 @@
       </c>
       <c r="B802" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">dados_completos</t>
+          <t xml:space="preserve">arquivos_nomes</t>
         </is>
       </c>
       <c r="C802" t="inlineStr" s="2">
@@ -22571,12 +22571,12 @@
       </c>
       <c r="B803" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">atividade_id</t>
+          <t xml:space="preserve">dados_completos</t>
         </is>
       </c>
       <c r="C803" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">json</t>
         </is>
       </c>
       <c r="D803" t="inlineStr" s="2">
@@ -22586,7 +22586,11 @@
       </c>
       <c r="E803" s="2"/>
       <c r="F803" s="2"/>
-      <c r="G803" s="2"/>
+      <c r="G803" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Estrutura JSON livre</t>
+        </is>
+      </c>
     </row>
     <row r="804">
       <c r="A804" t="inlineStr" s="2">
@@ -22596,12 +22600,12 @@
       </c>
       <c r="B804" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">whatsapp_enviado</t>
+          <t xml:space="preserve">atividade_id</t>
         </is>
       </c>
       <c r="C804" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D804" t="inlineStr" s="2">
@@ -22609,11 +22613,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E804" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
+      <c r="E804" s="2"/>
       <c r="F804" s="2"/>
       <c r="G804" s="2"/>
     </row>
@@ -22625,12 +22625,12 @@
       </c>
       <c r="B805" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">whatsapp_enviado_em</t>
+          <t xml:space="preserve">whatsapp_enviado</t>
         </is>
       </c>
       <c r="C805" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D805" t="inlineStr" s="2">
@@ -22638,7 +22638,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E805" s="2"/>
+      <c r="E805" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F805" s="2"/>
       <c r="G805" s="2"/>
     </row>
@@ -22650,12 +22654,12 @@
       </c>
       <c r="B806" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">whatsapp_enviado_em</t>
         </is>
       </c>
       <c r="C806" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D806" t="inlineStr" s="2">
@@ -22665,11 +22669,7 @@
       </c>
       <c r="E806" s="2"/>
       <c r="F806" s="2"/>
-      <c r="G806" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G806" s="2"/>
     </row>
     <row r="807">
       <c r="A807" t="inlineStr" s="2">
@@ -22679,7 +22679,7 @@
       </c>
       <c r="B807" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C807" t="inlineStr" s="2">
@@ -22696,34 +22696,38 @@
       <c r="F807" s="2"/>
       <c r="G807" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="808">
       <c r="A808" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">knowledge_categories</t>
+          <t xml:space="preserve">analises_fatura</t>
         </is>
       </c>
       <c r="B808" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C808" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D808" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E808" s="2"/>
       <c r="F808" s="2"/>
-      <c r="G808" s="2"/>
+      <c r="G808" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="809">
       <c r="A809" t="inlineStr" s="2">
@@ -22733,7 +22737,7 @@
       </c>
       <c r="B809" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">descricao</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C809" t="inlineStr" s="2">
@@ -22743,7 +22747,7 @@
       </c>
       <c r="D809" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E809" s="2"/>
@@ -22758,7 +22762,7 @@
       </c>
       <c r="B810" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">icone</t>
+          <t xml:space="preserve">descricao</t>
         </is>
       </c>
       <c r="C810" t="inlineStr" s="2">
@@ -22783,12 +22787,12 @@
       </c>
       <c r="B811" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ordem</t>
+          <t xml:space="preserve">icone</t>
         </is>
       </c>
       <c r="C811" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D811" t="inlineStr" s="2">
@@ -22808,12 +22812,12 @@
       </c>
       <c r="B812" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">ordem</t>
         </is>
       </c>
       <c r="C812" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D812" t="inlineStr" s="2">
@@ -22823,11 +22827,7 @@
       </c>
       <c r="E812" s="2"/>
       <c r="F812" s="2"/>
-      <c r="G812" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G812" s="2"/>
     </row>
     <row r="813">
       <c r="A813" t="inlineStr" s="2">
@@ -22837,7 +22837,7 @@
       </c>
       <c r="B813" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C813" t="inlineStr" s="2">
@@ -22854,38 +22854,38 @@
       <c r="F813" s="2"/>
       <c r="G813" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="814">
       <c r="A814" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">knowledge_articles</t>
+          <t xml:space="preserve">knowledge_categories</t>
         </is>
       </c>
       <c r="B814" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">categoria_id</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C814" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D814" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E814" s="2"/>
-      <c r="F814" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">knowledge_categories</t>
-        </is>
-      </c>
-      <c r="G814" s="2"/>
+      <c r="F814" s="2"/>
+      <c r="G814" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="815">
       <c r="A815" t="inlineStr" s="2">
@@ -22895,12 +22895,12 @@
       </c>
       <c r="B815" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">titulo</t>
+          <t xml:space="preserve">categoria_id</t>
         </is>
       </c>
       <c r="C815" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D815" t="inlineStr" s="2">
@@ -22909,7 +22909,11 @@
         </is>
       </c>
       <c r="E815" s="2"/>
-      <c r="F815" s="2"/>
+      <c r="F815" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">knowledge_categories</t>
+        </is>
+      </c>
       <c r="G815" s="2"/>
     </row>
     <row r="816">
@@ -22920,7 +22924,7 @@
       </c>
       <c r="B816" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">conteudo</t>
+          <t xml:space="preserve">titulo</t>
         </is>
       </c>
       <c r="C816" t="inlineStr" s="2">
@@ -22945,7 +22949,7 @@
       </c>
       <c r="B817" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">texto_extraido</t>
+          <t xml:space="preserve">conteudo</t>
         </is>
       </c>
       <c r="C817" t="inlineStr" s="2">
@@ -22955,7 +22959,7 @@
       </c>
       <c r="D817" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E817" s="2"/>
@@ -22970,12 +22974,12 @@
       </c>
       <c r="B818" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">anexos</t>
+          <t xml:space="preserve">texto_extraido</t>
         </is>
       </c>
       <c r="C818" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">file</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D818" t="inlineStr" s="2">
@@ -22985,11 +22989,7 @@
       </c>
       <c r="E818" s="2"/>
       <c r="F818" s="2"/>
-      <c r="G818" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
-        </is>
-      </c>
+      <c r="G818" s="2"/>
     </row>
     <row r="819">
       <c r="A819" t="inlineStr" s="2">
@@ -22999,12 +22999,12 @@
       </c>
       <c r="B819" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">criado_por</t>
+          <t xml:space="preserve">anexos</t>
         </is>
       </c>
       <c r="C819" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="D819" t="inlineStr" s="2">
@@ -23013,12 +23013,12 @@
         </is>
       </c>
       <c r="E819" s="2"/>
-      <c r="F819" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">users</t>
-        </is>
-      </c>
-      <c r="G819" s="2"/>
+      <c r="F819" s="2"/>
+      <c r="G819" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Armazenamento de arquivo / mídia anexada</t>
+        </is>
+      </c>
     </row>
     <row r="820">
       <c r="A820" t="inlineStr" s="2">
@@ -23028,12 +23028,12 @@
       </c>
       <c r="B820" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autor_nome</t>
+          <t xml:space="preserve">criado_por</t>
         </is>
       </c>
       <c r="C820" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D820" t="inlineStr" s="2">
@@ -23042,7 +23042,11 @@
         </is>
       </c>
       <c r="E820" s="2"/>
-      <c r="F820" s="2"/>
+      <c r="F820" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">users</t>
+        </is>
+      </c>
       <c r="G820" s="2"/>
     </row>
     <row r="821">
@@ -23053,7 +23057,7 @@
       </c>
       <c r="B821" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tags</t>
+          <t xml:space="preserve">autor_nome</t>
         </is>
       </c>
       <c r="C821" t="inlineStr" s="2">
@@ -23078,12 +23082,12 @@
       </c>
       <c r="B822" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">tags</t>
         </is>
       </c>
       <c r="C822" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D822" t="inlineStr" s="2">
@@ -23093,11 +23097,7 @@
       </c>
       <c r="E822" s="2"/>
       <c r="F822" s="2"/>
-      <c r="G822" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G822" s="2"/>
     </row>
     <row r="823">
       <c r="A823" t="inlineStr" s="2">
@@ -23107,7 +23107,7 @@
       </c>
       <c r="B823" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C823" t="inlineStr" s="2">
@@ -23124,38 +23124,38 @@
       <c r="F823" s="2"/>
       <c r="G823" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="824">
       <c r="A824" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contratos_usinas</t>
+          <t xml:space="preserve">knowledge_articles</t>
         </is>
       </c>
       <c r="B824" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contrato_id</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C824" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D824" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E824" s="2"/>
-      <c r="F824" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">contratos_om</t>
-        </is>
-      </c>
-      <c r="G824" s="2"/>
+      <c r="F824" s="2"/>
+      <c r="G824" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="825">
       <c r="A825" t="inlineStr" s="2">
@@ -23165,7 +23165,7 @@
       </c>
       <c r="B825" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">usina_id</t>
+          <t xml:space="preserve">contrato_id</t>
         </is>
       </c>
       <c r="C825" t="inlineStr" s="2">
@@ -23181,7 +23181,7 @@
       <c r="E825" s="2"/>
       <c r="F825" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">usinas</t>
+          <t xml:space="preserve">contratos_om</t>
         </is>
       </c>
       <c r="G825" s="2"/>
@@ -23194,25 +23194,25 @@
       </c>
       <c r="B826" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ativo</t>
+          <t xml:space="preserve">usina_id</t>
         </is>
       </c>
       <c r="C826" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bool</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D826" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E826" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">true / false</t>
-        </is>
-      </c>
-      <c r="F826" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E826" s="2"/>
+      <c r="F826" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usinas</t>
+        </is>
+      </c>
       <c r="G826" s="2"/>
     </row>
     <row r="827">
@@ -23223,12 +23223,12 @@
       </c>
       <c r="B827" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_vinculo</t>
+          <t xml:space="preserve">ativo</t>
         </is>
       </c>
       <c r="C827" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="D827" t="inlineStr" s="2">
@@ -23236,7 +23236,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E827" s="2"/>
+      <c r="E827" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">true / false</t>
+        </is>
+      </c>
       <c r="F827" s="2"/>
       <c r="G827" s="2"/>
     </row>
@@ -23248,7 +23252,7 @@
       </c>
       <c r="B828" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_desvinculo</t>
+          <t xml:space="preserve">data_vinculo</t>
         </is>
       </c>
       <c r="C828" t="inlineStr" s="2">
@@ -23273,12 +23277,12 @@
       </c>
       <c r="B829" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">observacoes</t>
+          <t xml:space="preserve">data_desvinculo</t>
         </is>
       </c>
       <c r="C829" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D829" t="inlineStr" s="2">
@@ -23298,12 +23302,12 @@
       </c>
       <c r="B830" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">observacoes</t>
         </is>
       </c>
       <c r="C830" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D830" t="inlineStr" s="2">
@@ -23313,11 +23317,7 @@
       </c>
       <c r="E830" s="2"/>
       <c r="F830" s="2"/>
-      <c r="G830" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G830" s="2"/>
     </row>
     <row r="831">
       <c r="A831" t="inlineStr" s="2">
@@ -23327,7 +23327,7 @@
       </c>
       <c r="B831" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C831" t="inlineStr" s="2">
@@ -23344,24 +23344,24 @@
       <c r="F831" s="2"/>
       <c r="G831" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="832">
       <c r="A832" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ativos</t>
+          <t xml:space="preserve">contratos_usinas</t>
         </is>
       </c>
       <c r="B832" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">usina_id</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C832" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D832" t="inlineStr" s="2">
@@ -23370,12 +23370,12 @@
         </is>
       </c>
       <c r="E832" s="2"/>
-      <c r="F832" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">usinas</t>
-        </is>
-      </c>
-      <c r="G832" s="2"/>
+      <c r="F832" s="2"/>
+      <c r="G832" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="833">
       <c r="A833" t="inlineStr" s="2">
@@ -23385,25 +23385,25 @@
       </c>
       <c r="B833" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo</t>
+          <t xml:space="preserve">usina_id</t>
         </is>
       </c>
       <c r="C833" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D833" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
-        </is>
-      </c>
-      <c r="E833" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">inversor | placa_solar | bateria | string_box | outros</t>
-        </is>
-      </c>
-      <c r="F833" s="2"/>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E833" s="2"/>
+      <c r="F833" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usinas</t>
+        </is>
+      </c>
       <c r="G833" s="2"/>
     </row>
     <row r="834">
@@ -23414,20 +23414,24 @@
       </c>
       <c r="B834" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">tipo_outro_descricao</t>
+          <t xml:space="preserve">tipo</t>
         </is>
       </c>
       <c r="C834" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D834" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
-        </is>
-      </c>
-      <c r="E834" s="2"/>
+          <t xml:space="preserve">Sim</t>
+        </is>
+      </c>
+      <c r="E834" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">inversor | placa_solar | bateria | string_box | outros</t>
+        </is>
+      </c>
       <c r="F834" s="2"/>
       <c r="G834" s="2"/>
     </row>
@@ -23439,7 +23443,7 @@
       </c>
       <c r="B835" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fabricante</t>
+          <t xml:space="preserve">tipo_outro_descricao</t>
         </is>
       </c>
       <c r="C835" t="inlineStr" s="2">
@@ -23449,7 +23453,7 @@
       </c>
       <c r="D835" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E835" s="2"/>
@@ -23464,7 +23468,7 @@
       </c>
       <c r="B836" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">modelo</t>
+          <t xml:space="preserve">fabricante</t>
         </is>
       </c>
       <c r="C836" t="inlineStr" s="2">
@@ -23489,7 +23493,7 @@
       </c>
       <c r="B837" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">numero_serie</t>
+          <t xml:space="preserve">modelo</t>
         </is>
       </c>
       <c r="C837" t="inlineStr" s="2">
@@ -23499,7 +23503,7 @@
       </c>
       <c r="D837" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E837" s="2"/>
@@ -23514,12 +23518,12 @@
       </c>
       <c r="B838" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_instalacao</t>
+          <t xml:space="preserve">numero_serie</t>
         </is>
       </c>
       <c r="C838" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D838" t="inlineStr" s="2">
@@ -23539,7 +23543,7 @@
       </c>
       <c r="B839" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">data_fim_garantia</t>
+          <t xml:space="preserve">data_instalacao</t>
         </is>
       </c>
       <c r="C839" t="inlineStr" s="2">
@@ -23564,12 +23568,12 @@
       </c>
       <c r="B840" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">responsavel_id</t>
+          <t xml:space="preserve">data_fim_garantia</t>
         </is>
       </c>
       <c r="C840" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">date</t>
         </is>
       </c>
       <c r="D840" t="inlineStr" s="2">
@@ -23578,11 +23582,7 @@
         </is>
       </c>
       <c r="E840" s="2"/>
-      <c r="F840" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">users</t>
-        </is>
-      </c>
+      <c r="F840" s="2"/>
       <c r="G840" s="2"/>
     </row>
     <row r="841">
@@ -23593,12 +23593,12 @@
       </c>
       <c r="B841" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">observacoes</t>
+          <t xml:space="preserve">responsavel_id</t>
         </is>
       </c>
       <c r="C841" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D841" t="inlineStr" s="2">
@@ -23607,7 +23607,11 @@
         </is>
       </c>
       <c r="E841" s="2"/>
-      <c r="F841" s="2"/>
+      <c r="F841" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">users</t>
+        </is>
+      </c>
       <c r="G841" s="2"/>
     </row>
     <row r="842">
@@ -23618,12 +23622,12 @@
       </c>
       <c r="B842" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">status_operacional</t>
+          <t xml:space="preserve">observacoes</t>
         </is>
       </c>
       <c r="C842" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D842" t="inlineStr" s="2">
@@ -23631,11 +23635,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E842" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">operacional | em_alerta | manutencao | desativado</t>
-        </is>
-      </c>
+      <c r="E842" s="2"/>
       <c r="F842" s="2"/>
       <c r="G842" s="2"/>
     </row>
@@ -23647,12 +23647,12 @@
       </c>
       <c r="B843" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">status_operacional</t>
         </is>
       </c>
       <c r="C843" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D843" t="inlineStr" s="2">
@@ -23660,13 +23660,13 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E843" s="2"/>
+      <c r="E843" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">operacional | em_alerta | manutencao | desativado</t>
+        </is>
+      </c>
       <c r="F843" s="2"/>
-      <c r="G843" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G843" s="2"/>
     </row>
     <row r="844">
       <c r="A844" t="inlineStr" s="2">
@@ -23676,7 +23676,7 @@
       </c>
       <c r="B844" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C844" t="inlineStr" s="2">
@@ -23693,7 +23693,7 @@
       <c r="F844" s="2"/>
       <c r="G844" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
@@ -23705,12 +23705,12 @@
       </c>
       <c r="B845" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">chave_importacao</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C845" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D845" t="inlineStr" s="2">
@@ -23720,7 +23720,11 @@
       </c>
       <c r="E845" s="2"/>
       <c r="F845" s="2"/>
-      <c r="G845" s="2"/>
+      <c r="G845" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="846">
       <c r="A846" t="inlineStr" s="2">
@@ -23730,7 +23734,7 @@
       </c>
       <c r="B846" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cliente_inversor_id</t>
+          <t xml:space="preserve">chave_importacao</t>
         </is>
       </c>
       <c r="C846" t="inlineStr" s="2">
@@ -23750,12 +23754,12 @@
     <row r="847">
       <c r="A847" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">contatos</t>
+          <t xml:space="preserve">ativos</t>
         </is>
       </c>
       <c r="B847" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">nome</t>
+          <t xml:space="preserve">cliente_inversor_id</t>
         </is>
       </c>
       <c r="C847" t="inlineStr" s="2">
@@ -23765,7 +23769,7 @@
       </c>
       <c r="D847" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E847" s="2"/>
@@ -23780,7 +23784,7 @@
       </c>
       <c r="B848" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">telefone</t>
+          <t xml:space="preserve">nome</t>
         </is>
       </c>
       <c r="C848" t="inlineStr" s="2">
@@ -23790,7 +23794,7 @@
       </c>
       <c r="D848" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E848" s="2"/>
@@ -23805,7 +23809,7 @@
       </c>
       <c r="B849" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">whatsapp</t>
+          <t xml:space="preserve">telefone</t>
         </is>
       </c>
       <c r="C849" t="inlineStr" s="2">
@@ -23830,12 +23834,12 @@
       </c>
       <c r="B850" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">email</t>
+          <t xml:space="preserve">whatsapp</t>
         </is>
       </c>
       <c r="C850" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">email</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D850" t="inlineStr" s="2">
@@ -23855,12 +23859,12 @@
       </c>
       <c r="B851" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">papel</t>
+          <t xml:space="preserve">email</t>
         </is>
       </c>
       <c r="C851" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">select</t>
+          <t xml:space="preserve">email</t>
         </is>
       </c>
       <c r="D851" t="inlineStr" s="2">
@@ -23868,11 +23872,7 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E851" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">cliente | lead | fornecedor | tecnico | parceiro | familiar | responsavel | financeiro | outro</t>
-        </is>
-      </c>
+      <c r="E851" s="2"/>
       <c r="F851" s="2"/>
       <c r="G851" s="2"/>
     </row>
@@ -23884,12 +23884,12 @@
       </c>
       <c r="B852" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cargo</t>
+          <t xml:space="preserve">papel</t>
         </is>
       </c>
       <c r="C852" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">select</t>
         </is>
       </c>
       <c r="D852" t="inlineStr" s="2">
@@ -23897,7 +23897,11 @@
           <t xml:space="preserve">Não</t>
         </is>
       </c>
-      <c r="E852" s="2"/>
+      <c r="E852" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">cliente | lead | fornecedor | tecnico | parceiro | familiar | responsavel | financeiro | outro</t>
+        </is>
+      </c>
       <c r="F852" s="2"/>
       <c r="G852" s="2"/>
     </row>
@@ -23909,7 +23913,7 @@
       </c>
       <c r="B853" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">observacoes</t>
+          <t xml:space="preserve">cargo</t>
         </is>
       </c>
       <c r="C853" t="inlineStr" s="2">
@@ -23934,12 +23938,12 @@
       </c>
       <c r="B854" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">clientes_vinculados</t>
+          <t xml:space="preserve">observacoes</t>
         </is>
       </c>
       <c r="C854" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D854" t="inlineStr" s="2">
@@ -23948,11 +23952,7 @@
         </is>
       </c>
       <c r="E854" s="2"/>
-      <c r="F854" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">clientes</t>
-        </is>
-      </c>
+      <c r="F854" s="2"/>
       <c r="G854" s="2"/>
     </row>
     <row r="855">
@@ -23963,7 +23963,7 @@
       </c>
       <c r="B855" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios_vinculados</t>
+          <t xml:space="preserve">clientes_vinculados</t>
         </is>
       </c>
       <c r="C855" t="inlineStr" s="2">
@@ -23979,7 +23979,7 @@
       <c r="E855" s="2"/>
       <c r="F855" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">negocios</t>
+          <t xml:space="preserve">clientes</t>
         </is>
       </c>
       <c r="G855" s="2"/>
@@ -23992,12 +23992,12 @@
       </c>
       <c r="B856" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">conversa_id</t>
+          <t xml:space="preserve">negocios_vinculados</t>
         </is>
       </c>
       <c r="C856" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D856" t="inlineStr" s="2">
@@ -24006,7 +24006,11 @@
         </is>
       </c>
       <c r="E856" s="2"/>
-      <c r="F856" s="2"/>
+      <c r="F856" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">negocios</t>
+        </is>
+      </c>
       <c r="G856" s="2"/>
     </row>
     <row r="857">
@@ -24017,7 +24021,7 @@
       </c>
       <c r="B857" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">origem_registro</t>
+          <t xml:space="preserve">conversa_id</t>
         </is>
       </c>
       <c r="C857" t="inlineStr" s="2">
@@ -24042,12 +24046,12 @@
       </c>
       <c r="B858" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">origem_registro</t>
         </is>
       </c>
       <c r="C858" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D858" t="inlineStr" s="2">
@@ -24057,11 +24061,7 @@
       </c>
       <c r="E858" s="2"/>
       <c r="F858" s="2"/>
-      <c r="G858" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G858" s="2"/>
     </row>
     <row r="859">
       <c r="A859" t="inlineStr" s="2">
@@ -24071,7 +24071,7 @@
       </c>
       <c r="B859" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C859" t="inlineStr" s="2">
@@ -24088,38 +24088,38 @@
       <c r="F859" s="2"/>
       <c r="G859" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+          <t xml:space="preserve">Autodate: onCreate</t>
         </is>
       </c>
     </row>
     <row r="860">
       <c r="A860" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">usina_equipamentos</t>
+          <t xml:space="preserve">contatos</t>
         </is>
       </c>
       <c r="B860" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">usina_id</t>
+          <t xml:space="preserve">updated</t>
         </is>
       </c>
       <c r="C860" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">autodate</t>
         </is>
       </c>
       <c r="D860" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sim</t>
+          <t xml:space="preserve">Não</t>
         </is>
       </c>
       <c r="E860" s="2"/>
-      <c r="F860" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">usinas</t>
-        </is>
-      </c>
-      <c r="G860" s="2"/>
+      <c r="F860" s="2"/>
+      <c r="G860" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
+        </is>
+      </c>
     </row>
     <row r="861">
       <c r="A861" t="inlineStr" s="2">
@@ -24129,7 +24129,7 @@
       </c>
       <c r="B861" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">equipamento_id</t>
+          <t xml:space="preserve">usina_id</t>
         </is>
       </c>
       <c r="C861" t="inlineStr" s="2">
@@ -24145,7 +24145,7 @@
       <c r="E861" s="2"/>
       <c r="F861" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">equipamentos</t>
+          <t xml:space="preserve">usinas</t>
         </is>
       </c>
       <c r="G861" s="2"/>
@@ -24158,21 +24158,25 @@
       </c>
       <c r="B862" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">quantidade</t>
+          <t xml:space="preserve">equipamento_id</t>
         </is>
       </c>
       <c r="C862" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D862" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Não</t>
+          <t xml:space="preserve">Sim</t>
         </is>
       </c>
       <c r="E862" s="2"/>
-      <c r="F862" s="2"/>
+      <c r="F862" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">equipamentos</t>
+        </is>
+      </c>
       <c r="G862" s="2"/>
     </row>
     <row r="863">
@@ -24183,12 +24187,12 @@
       </c>
       <c r="B863" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">numero_serie</t>
+          <t xml:space="preserve">quantidade</t>
         </is>
       </c>
       <c r="C863" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D863" t="inlineStr" s="2">
@@ -24208,7 +24212,7 @@
       </c>
       <c r="B864" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">observacoes</t>
+          <t xml:space="preserve">numero_serie</t>
         </is>
       </c>
       <c r="C864" t="inlineStr" s="2">
@@ -24233,12 +24237,12 @@
       </c>
       <c r="B865" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">created</t>
+          <t xml:space="preserve">observacoes</t>
         </is>
       </c>
       <c r="C865" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">autodate</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="D865" t="inlineStr" s="2">
@@ -24248,11 +24252,7 @@
       </c>
       <c r="E865" s="2"/>
       <c r="F865" s="2"/>
-      <c r="G865" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Autodate: onCreate</t>
-        </is>
-      </c>
+      <c r="G865" s="2"/>
     </row>
     <row r="866">
       <c r="A866" t="inlineStr" s="2">
@@ -24262,7 +24262,7 @@
       </c>
       <c r="B866" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updated</t>
+          <t xml:space="preserve">created</t>
         </is>
       </c>
       <c r="C866" t="inlineStr" s="2">
@@ -24278,6 +24278,35 @@
       <c r="E866" s="2"/>
       <c r="F866" s="2"/>
       <c r="G866" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Autodate: onCreate</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">usina_equipamentos</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">updated</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">autodate</t>
+        </is>
+      </c>
+      <c r="D867" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="E867" s="2"/>
+      <c r="F867" s="2"/>
+      <c r="G867" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Autodate: onCreate, onUpdate</t>
         </is>

</xml_diff>